<commit_message>
feat(engineering): preset 2.5m east-strip tree trench template
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Elements_hybrides" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Noeuds_stockage" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Resume_checks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Template_est_2p5m" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -94,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -108,6 +109,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -577,6 +579,20 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mise a jour: bande est 2.5 m avec arbres modelisee en mode tranchee drainante + underdrain (E01/E02).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Le gabarit de section est dans Template_est_2p5m; micro-noue de surface + underdrain en emprise contrainte.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -591,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1050,6 +1066,206 @@
       <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Volume tampon noeud = Qin*temps</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>East_strip_total_width_m</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Largeur bande verte est disponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>East_surface_depression_width_m</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Largeur depression superficielle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>East_surface_depression_depth_m</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Profondeur depression de surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>East_tree_soil_zone_width_m</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Zone sol vegetal / arbres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>East_underdrain_trench_width_m</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Largeur tranchee drainante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>East_underdrain_trench_depth_m</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Profondeur tranchee drainante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>East_underdrain_pipe_diameter_mm</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Diametre perforé recommandé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>East_root_barrier_offset_m</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Distance cible entre conduite et tronc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>East_cleanout_spacing_m</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Espacement regards/cleanouts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>East_underdrain_slope_m_per_m</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Pente longitudinale de l underdrain.</t>
         </is>
       </c>
     </row>
@@ -5989,7 +6205,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>TRENCH</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -6010,26 +6226,33 @@
       <c r="F4" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G4" s="7" t="n">
-        <v>0.01</v>
+      <c r="G4" s="7">
+        <f>Inputs!$B$33</f>
+        <v/>
       </c>
       <c r="H4" s="7" t="inlineStr"/>
       <c r="I4" s="8">
         <f>IF(A4="","",IF(H4&lt;&gt;"",H4,IF(UPPER(TRIM(B4))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B4))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J4" s="7" t="inlineStr"/>
-      <c r="K4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="7" t="n">
-        <v>0.3</v>
+      <c r="J4" s="7">
+        <f>Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="K4" s="7">
+        <f>Inputs!$B$28</f>
+        <v/>
+      </c>
+      <c r="L4" s="7">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="M4" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" s="7" t="n">
         <v>0</v>
+      </c>
+      <c r="N4" s="7">
+        <f>Inputs!$B$22</f>
+        <v/>
       </c>
       <c r="O4" s="8">
         <f>IF(A4="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A4))</f>
@@ -6085,7 +6308,7 @@
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>Noue est amont (zone arbres)</t>
+          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6320,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>TRENCH</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -6118,26 +6341,33 @@
       <c r="F5" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="G5" s="7" t="n">
-        <v>0.01</v>
+      <c r="G5" s="7">
+        <f>Inputs!$B$33</f>
+        <v/>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
       <c r="I5" s="8">
         <f>IF(A5="","",IF(H5&lt;&gt;"",H5,IF(UPPER(TRIM(B5))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B5))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>0.3</v>
+      <c r="J5" s="7">
+        <f>Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="K5" s="7">
+        <f>Inputs!$B$28</f>
+        <v/>
+      </c>
+      <c r="L5" s="7">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="M5" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" s="7" t="n">
         <v>0</v>
+      </c>
+      <c r="N5" s="7">
+        <f>Inputs!$B$22</f>
+        <v/>
       </c>
       <c r="O5" s="8">
         <f>IF(A5="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A5))</f>
@@ -6193,7 +6423,7 @@
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>Noue est aval</t>
+          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.</t>
         </is>
       </c>
     </row>
@@ -6339,14 +6569,17 @@
         <v/>
       </c>
       <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="L7" s="7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M7" s="7" t="n">
-        <v>3</v>
+      <c r="K7" s="7">
+        <f>Inputs!$B$25</f>
+        <v/>
+      </c>
+      <c r="L7" s="7">
+        <f>Inputs!$B$26</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>Inputs!$B$20</f>
+        <v/>
       </c>
       <c r="N7" s="7" t="n">
         <v>0</v>
@@ -6405,7 +6638,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Noue sud recevant toiture</t>
+          <t>Noue sud peu profonde (collecte toiture/tresfond sud).</t>
         </is>
       </c>
     </row>
@@ -27472,4 +27705,321 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GABARIT BANDE EST 2.5 m (ARBRES) - SOLUTION HYBRIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Composante</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Largeur m</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Profondeur m</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Unite</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Volume utile m3/m</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Depression de surface (micro-noue)</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>Inputs!$B$25</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>Inputs!$B$26</f>
+        <v/>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Storage_surface_m3_per_m</t>
+        </is>
+      </c>
+      <c r="E4" s="5">
+        <f>B4*C4</f>
+        <v/>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>m3/m</t>
+        </is>
+      </c>
+      <c r="G4" s="9">
+        <f>B4*C4</f>
+        <v/>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Captation initiale / pretaitement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tranchee drainante (sous-sol)</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>Inputs!$B$28</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>Inputs!$B$29</f>
+        <v/>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Porosite</t>
+        </is>
+      </c>
+      <c r="E5" s="5">
+        <f>Inputs!$B$22</f>
+        <v/>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="9">
+        <f>B5*C5*E5</f>
+        <v/>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Conveyance + stockage utile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Sous-total stockage</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Storage_total_m3_per_m</t>
+        </is>
+      </c>
+      <c r="E6" s="5">
+        <f>G4+G5</f>
+        <v/>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>m3/m</t>
+        </is>
+      </c>
+      <c r="G6" s="9">
+        <f>G4+G5</f>
+        <v/>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Base dimensionnement lineaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Underdrain perforé</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Diametre_pipe_mm</t>
+        </is>
+      </c>
+      <c r="E7" s="5">
+        <f>Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>PVC/PEHD perforé, pente Inputs!B33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Espacement cleanout</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Spacing_m</t>
+        </is>
+      </c>
+      <c r="E8" s="5">
+        <f>Inputs!$B$32</f>
+        <v/>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Aux changements de direction et max 25-30 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Offset barriere racinaire</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Offset_m</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>Inputs!$B$31</f>
+        <v/>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Eloigner la conduite de la zone tronc/racines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Controle rapide capacite lineaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Longueur active bande est (m)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>(input)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Stockage lineaire m3/m</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="C13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Stockage total disponible m3</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>B12*B13</f>
+        <v/>
+      </c>
+      <c r="C14" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(engineering): relabel hybrid model nodes to project naming
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Noeuds_stockage" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Resume_checks" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Template_est_2p5m" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Convention_labels" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -590,6 +591,13 @@
       <c r="A18" t="inlineStr">
         <is>
           <t>Le gabarit de section est dans Template_est_2p5m; micro-noue de surface + underdrain en emprise contrainte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Labels harmonises: placeholders remplaces par P-01/P-02/P-03 et jonctions explicites (voir Convention_labels).</t>
         </is>
       </c>
     </row>
@@ -1303,6 +1311,13 @@
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ZONES TRIBUTAIRES - TOIT / TRESFOND / VERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Routing des zones se fait via Element_ID (colonne J), independamment du renommage des noeuds.</t>
         </is>
       </c>
     </row>
@@ -6210,12 +6225,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P-01</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P-02</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -6308,7 +6323,7 @@
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.</t>
+          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6325,12 +6340,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P-02</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -6423,7 +6438,7 @@
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.</t>
+          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6440,12 +6455,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>BASIN_IN</t>
+          <t>J-BASSIN-IN</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -6527,7 +6542,7 @@
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>Collecteur vers bassin</t>
+          <t>Collecteur vers bassin; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6544,12 +6559,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>S_EAST</t>
+          <t>J-SUD-EST</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>S_MID</t>
+          <t>J-SUD-OUEST</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -6638,7 +6653,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Noue sud peu profonde (collecte toiture/tresfond sud).</t>
+          <t>Noue sud peu profonde (collecte toiture/tresfond sud).; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6655,12 +6670,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>W_UP</t>
+          <t>J-OUEST-AMONT</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>W_LOW</t>
+          <t>J-OUEST-AVAL</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -6746,7 +6761,7 @@
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>Tranchee drainante ouest</t>
+          <t>Tranchee drainante ouest; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6763,12 +6778,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>W_LOW</t>
+          <t>J-OUEST-AVAL</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>BASIN_IN</t>
+          <t>J-BASSIN-IN</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -6850,7 +6865,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Branche ouest vers bassin</t>
+          <t>Branche ouest vers bassin; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -6867,12 +6882,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>BASIN_IN</t>
+          <t>J-BASSIN-IN</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>BASIN_RET</t>
+          <t>BASSIN-RET</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
@@ -6950,7 +6965,7 @@
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>Troncon final au bassin</t>
+          <t>Troncon final au bassin; Labels projet harmonises (2026-07-02).</t>
         </is>
       </c>
     </row>
@@ -21419,7 +21434,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P-01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -21466,7 +21481,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P-02</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -21513,7 +21528,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -21560,7 +21575,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>S_EAST</t>
+          <t>J-SUD-EST</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -21609,7 +21624,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>S_MID</t>
+          <t>J-SUD-OUEST</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -21658,7 +21673,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>W_UP</t>
+          <t>J-OUEST-AMONT</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -21705,7 +21720,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>W_LOW</t>
+          <t>J-OUEST-AVAL</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -21752,7 +21767,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>BASIN_IN</t>
+          <t>J-BASSIN-IN</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -21799,7 +21814,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>BASIN_RET</t>
+          <t>BASSIN-RET</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -28022,4 +28037,305 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONVENTION DE NOMMAGE - MODELE HYBRIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Label projet</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Role hydraulique</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Noeud amont est</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Puisard/CB existant amont</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Noeud intermediaire est</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Puisard/CB milieu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Noeud aval est</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Puisard/CB aval</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>S_EAST</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>J-SUD-EST</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>SWALE_NODE</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Jonction sud est</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Point de collecte sud est</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>S_MID</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>J-SUD-OUEST</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>SWALE_NODE</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Jonction sud ouest</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Point de rassemblement sud</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>W_UP</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>J-OUEST-AMONT</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Noeud ouest amont</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Collecte bande ouest</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>W_LOW</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>J-OUEST-AVAL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Noeud ouest aval</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Transition vers pipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>BASIN_IN</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>J-BASSIN-IN</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Regard amont bassin</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Noeud avant bassin</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>BASIN_RET</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>RETENTION</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Bassin de retention</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Exutoire final</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(engineering): align hybrid model with site constraints and area labels
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Resume_checks" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Template_est_2p5m" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Convention_labels" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Contraintes_ouest_utilites" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dimensionnement_est" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -42,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -111,6 +118,8 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -601,9 +610,342 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Implantation mise a jour: bassin lineaire dans bande sud 2m + guidance conflits utilites ouest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Voir Dimensionnement_est et Contraintes_ouest_utilites pour dimensionnement et implantation recommandee.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DIMENSIONNEMENT BANDE EST (2.5m) - ESTIMATION A PARTIR DES AIRES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Formule/Source</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Unite</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Critere</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Q_design est aval (E02)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Elements_hybrides Q(E02)</t>
+        </is>
+      </c>
+      <c r="C4" s="8">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH("E02",Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Capacite pipe 200mm (s=Inputs!B33)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Manning plein</t>
+        </is>
+      </c>
+      <c r="C5" s="8">
+        <f>(1/Inputs!$B$9)*(PI()*(Inputs!$B$30/1000)^2/4)*(((Inputs!$B$30/1000)/4)^(2/3))*SQRT(Inputs!$B$33)</f>
+        <v/>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Capacite pipe 250mm</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Manning plein</t>
+        </is>
+      </c>
+      <c r="C6" s="8">
+        <f>(1/Inputs!$B$9)*(PI()*(0.25)^2/4)*((0.25/4)^(2/3))*SQRT(Inputs!$B$33)</f>
+        <v/>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Capacite pipe 300mm</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Manning plein</t>
+        </is>
+      </c>
+      <c r="C7" s="8">
+        <f>(1/Inputs!$B$9)*(PI()*(0.30)^2/4)*((0.30/4)^(2/3))*SQRT(Inputs!$B$33)</f>
+        <v/>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Diametre recommande est</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Q_design / fill_limit</t>
+        </is>
+      </c>
+      <c r="C8" s="11">
+        <f>IF(C4="","",IF(C4/Inputs!$B$19&lt;=C5,200,IF(C4/Inputs!$B$19&lt;=C6,250,IF(C4/Inputs!$B$19&lt;=C7,300,375))))</f>
+        <v/>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Stockage lineaire surface+tranchee (m3/m)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Template_est_2p5m</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <f>IFERROR(Template_est_2p5m!$G$6,"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>m3/m</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Longueur active bande est</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>E01+E02</t>
+        </is>
+      </c>
+      <c r="C11" s="8">
+        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E01",Elements_hybrides!$A$4:$A$204,0)),0)+IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E02",Elements_hybrides!$A$4:$A$204,0)),0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Stockage dispo bande est</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>C10*C11</t>
+        </is>
+      </c>
+      <c r="C12" s="8">
+        <f>IF(OR(C10="",C11=""),"",C10*C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Volume tampon requis est</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Q_design*buffer</t>
+        </is>
+      </c>
+      <c r="C13" s="8">
+        <f>IF(C4="","",C4*Inputs!$B$23*60)</f>
+        <v/>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Check stockage est</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>C12 vs C13</t>
+        </is>
+      </c>
+      <c r="C14" s="11">
+        <f>IF(OR(C12="",C13=""),"",IF(C12&gt;=C13,"OK","AUGMENTER VOLUME"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -615,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1274,6 +1616,127 @@
       <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Pente longitudinale de l underdrain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Basin_corridor_width_m</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Largeur disponible entre batiment et cheminement pieton sud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Basin_corridor_length_m</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Longueur exploitable du bassin lineaire sud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Basin_target_depth_m</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Profondeur cible bassin de retention lineaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Basin_ret_top_level_m</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Niveau de reference du bassin (a ajuster avec topographie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Basin_ret_invert_m</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>B37-B36</f>
+        <v/>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Radier bassin lineaire (derive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Max_cover_near_utilities_m</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Profondeur max recommandee dans zone lateraux ouest (approche conservatrice).</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1849,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Toiture principale</t>
+          <t>Toiture principale (bloc jaune)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1420,7 +1883,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Toiture vers noue sud</t>
+          <t>Toiture vers collecte sud</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1895,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Tresfond est</t>
+          <t>Tresfond est (gris)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1466,7 +1929,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Pente vers noue est</t>
+          <t>Pente vers bande est</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1975,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Noue est peu profonde</t>
+          <t>Vers underdrain est</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1987,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Bande verte ouest haute</t>
+          <t>Ouest vert 1</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1533,7 +1996,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>51.3</v>
+        <v>12.5</v>
       </c>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="8">
@@ -1558,7 +2021,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Vers tranchee ouest</t>
+          <t>Vers collecte ouest</t>
         </is>
       </c>
     </row>
@@ -1570,7 +2033,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Bande verte ouest milieu</t>
+          <t>Ouest vert 2</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1579,7 +2042,7 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>27.2</v>
+        <v>6.7</v>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
       <c r="F8" s="8">
@@ -1604,7 +2067,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Vers tranchee ouest</t>
+          <t>Vers collecte ouest</t>
         </is>
       </c>
     </row>
@@ -1616,7 +2079,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Bande verte sud gauche</t>
+          <t>Ouest vert 3</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1625,7 +2088,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>21.9</v>
+        <v>27.2</v>
       </c>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="8">
@@ -1650,7 +2113,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Vers collecteur ouest</t>
+          <t>Vers collecte ouest</t>
         </is>
       </c>
     </row>
@@ -1662,16 +2125,16 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Bande verte sud droite</t>
+          <t>Ouest pave-uni</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>GRASS</t>
+          <t>TRESFOND</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>20.5</v>
+        <v>37.5</v>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
       <c r="F10" s="8">
@@ -1679,7 +2142,7 @@
         <v/>
       </c>
       <c r="G10" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H10" s="8">
         <f>IF(A10="","",Inputs!$B$3/((IF(G10="",Inputs!$B$14,G10)+Inputs!$B$4)^Inputs!$B$5))</f>
@@ -1691,12 +2154,12 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Vers noue sud</t>
+          <t>Surface mineralisee ouest</t>
         </is>
       </c>
     </row>
@@ -1708,16 +2171,16 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Surface mineralisee sud</t>
+          <t>Ouest vert 4</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>GRASS</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>44.3</v>
+        <v>21.9</v>
       </c>
       <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="8">
@@ -1725,7 +2188,7 @@
         <v/>
       </c>
       <c r="G11" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H11" s="8">
         <f>IF(A11="","",Inputs!$B$3/((IF(G11="",Inputs!$B$14,G11)+Inputs!$B$4)^Inputs!$B$5))</f>
@@ -1737,12 +2200,12 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Vers noue sud</t>
+          <t>Vers collecte ouest</t>
         </is>
       </c>
     </row>
@@ -1754,16 +2217,16 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Petite surface minerale</t>
+          <t>Bande sud verte centrale</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>GRASS</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>5.8</v>
+        <v>109.7</v>
       </c>
       <c r="E12" s="7" t="inlineStr"/>
       <c r="F12" s="8">
@@ -1771,7 +2234,7 @@
         <v/>
       </c>
       <c r="G12" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H12" s="8">
         <f>IF(A12="","",Inputs!$B$3/((IF(G12="",Inputs!$B$14,G12)+Inputs!$B$4)^Inputs!$B$5))</f>
@@ -1793,16 +2256,32 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Z10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Sud gris local</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>TRESFOND</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="8">
         <f>IF(E13&lt;&gt;"",E13,IF(UPPER(TRIM(C13))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C13))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C13))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
         <v/>
       </c>
-      <c r="G13" s="7" t="n"/>
+      <c r="G13" s="7" t="n">
+        <v>8</v>
+      </c>
       <c r="H13" s="8">
         <f>IF(A13="","",Inputs!$B$3/((IF(G13="",Inputs!$B$14,G13)+Inputs!$B$4)^Inputs!$B$5))</f>
         <v/>
@@ -1811,20 +2290,44 @@
         <f>IF(A13="","",2.78E-7*F13*D13*H13)</f>
         <v/>
       </c>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Vers noue sud</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Z11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Sud est vert</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>GRASS</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
       <c r="F14" s="8">
         <f>IF(E14&lt;&gt;"",E14,IF(UPPER(TRIM(C14))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C14))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C14))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
         <v/>
       </c>
-      <c r="G14" s="7" t="n"/>
+      <c r="G14" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H14" s="8">
         <f>IF(A14="","",Inputs!$B$3/((IF(G14="",Inputs!$B$14,G14)+Inputs!$B$4)^Inputs!$B$5))</f>
         <v/>
@@ -1833,20 +2336,44 @@
         <f>IF(A14="","",2.78E-7*F14*D14*H14)</f>
         <v/>
       </c>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Vers noue sud</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Z12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Sud est gris petit</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>TRESFOND</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="8">
         <f>IF(E15&lt;&gt;"",E15,IF(UPPER(TRIM(C15))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C15))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C15))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
         <v/>
       </c>
-      <c r="G15" s="7" t="n"/>
+      <c r="G15" s="7" t="n">
+        <v>8</v>
+      </c>
       <c r="H15" s="8">
         <f>IF(A15="","",Inputs!$B$3/((IF(G15="",Inputs!$B$14,G15)+Inputs!$B$4)^Inputs!$B$5))</f>
         <v/>
@@ -1855,8 +2382,16 @@
         <f>IF(A15="","",2.78E-7*F15*D15*H15)</f>
         <v/>
       </c>
-      <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Vers noue sud</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -6239,7 +6774,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>12</v>
+        <v>21.6</v>
       </c>
       <c r="G4" s="7">
         <f>Inputs!$B$33</f>
@@ -6323,7 +6858,7 @@
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.; Labels projet harmonises (2026-07-02).</t>
+          <t>Bande est amont: tranchee drainante sous arbres (segment 1).</t>
         </is>
       </c>
     </row>
@@ -6354,7 +6889,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>14</v>
+        <v>21.6</v>
       </c>
       <c r="G5" s="7">
         <f>Inputs!$B$33</f>
@@ -6438,7 +6973,7 @@
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>Bande est 2.5m: tranchee drainante + underdrain; micro-noue de surface 0.6x0.10 m en complement.; Labels projet harmonises (2026-07-02).</t>
+          <t>Bande est aval: tranchee drainante sous arbres (segment 2).</t>
         </is>
       </c>
     </row>
@@ -6469,7 +7004,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>0.006</v>
@@ -6542,7 +7077,7 @@
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>Collecteur vers bassin; Labels projet harmonises (2026-07-02).</t>
+          <t>Collecteur est vers J-BASSIN-IN (hors zone racinaire dense).</t>
         </is>
       </c>
     </row>
@@ -6572,8 +7107,9 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>29.4</v>
+      <c r="F7" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.008</v>
@@ -6653,7 +7189,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Noue sud peu profonde (collecte toiture/tresfond sud).; Labels projet harmonises (2026-07-02).</t>
+          <t>Noue/tranchee sud dans bande 2.0m vers bassin lineaire.</t>
         </is>
       </c>
     </row>
@@ -6665,7 +7201,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>TRENCH</t>
+          <t>SWALE</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -6684,7 +7220,7 @@
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>0.008</v>
@@ -6694,18 +7230,18 @@
         <f>IF(A8="","",IF(H8&lt;&gt;"",H8,IF(UPPER(TRIM(B8))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B8))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>3</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="O8" s="8">
         <f>IF(A8="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A8))</f>
@@ -6761,7 +7297,7 @@
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>Tranchee drainante ouest; Labels projet harmonises (2026-07-02).</t>
+          <t>Collecte ouest avec conduite peu profonde/element lineaire compatible utilites.</t>
         </is>
       </c>
     </row>
@@ -6792,7 +7328,7 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.008</v>
@@ -6865,7 +7401,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Branche ouest vers bassin; Labels projet harmonises (2026-07-02).</t>
+          <t>Branche ouest vers J-BASSIN-IN (traverse utilites avec precautions).</t>
         </is>
       </c>
     </row>
@@ -6892,7 +7428,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>0.006</v>
@@ -6965,7 +7501,7 @@
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>Troncon final au bassin; Labels projet harmonises (2026-07-02).</t>
+          <t>Injection finale vers BASSIN-RET lineaire sud.</t>
         </is>
       </c>
     </row>
@@ -21787,7 +22323,7 @@
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
       <c r="I11" s="8">
@@ -21822,8 +22358,14 @@
           <t>RETENTION</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr"/>
-      <c r="D12" s="7" t="inlineStr"/>
+      <c r="C12" s="7">
+        <f>Inputs!$B$37</f>
+        <v/>
+      </c>
+      <c r="D12" s="7">
+        <f>Inputs!$B$38</f>
+        <v/>
+      </c>
       <c r="E12" s="8">
         <f>IF(OR(C12="",D12=""),"",MAX(0,C12-D12))</f>
         <v/>
@@ -21833,19 +22375,20 @@
           <t>RECT</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>15</v>
+      <c r="G12" s="7">
+        <f>Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="H12" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
       </c>
       <c r="I12" s="8">
         <f>IF(A12="","",IF(UPPER(TRIM(F12))="CIRC",PI()*(G12/2)^2*E12,IF(UPPER(TRIM(F12))="RECT",G12*H12*E12,"")))</f>
         <v/>
       </c>
-      <c r="J12" s="7">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J12" s="7" t="n">
+        <v>30</v>
       </c>
       <c r="K12" s="8">
         <f>IF(A12="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A12))</f>
@@ -28338,4 +28881,204 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>IMPLANTATION OUEST - CONFLITS UTILITES (AEP / PLUVIAL / SANITAIRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Contrainte</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Strategie recommandee</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Element modele</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Parametre cible</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Ouest haut</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Lateraux multiples</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Privilegier ecoulement de surface (noue peu profonde)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>E05 (SWALE)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>profondeur ~0.20 m</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Limiter fouille profonde dans emprise chargee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Traverse vers bassin</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Croisement inevitable</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Croiser perpendiculaire + gaine + pente mini</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>E06 (PIPE)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>slope 0.8%</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Verifier degagement vertical avec as-built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Bande sud 2m</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Emprise contrainte</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Bassin lineaire + noue/tranchee compacte</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>E04 + BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>width 2.0 m</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Stockage distribue + transfert au bassin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Bande est arbres</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Zone racinaire</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Tranchee drainante + underdrain + barriere racinaire</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>E01/E02 (TRENCH)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>offset &gt;=1.0 m</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Eviter conduite profonde continue en pied d arbres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Note: Les degagements finaux avec lateraux existants doivent etre confirmes par releves terrain/TQC avant IFC.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A9:F9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(engineering): add decision summary and element type color coding
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Convention_labels" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Contraintes_ouest_utilites" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Dimensionnement_est" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Decision_Summary" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -103,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -120,10 +121,46 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -485,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -621,6 +658,13 @@
       <c r="A21" t="inlineStr">
         <is>
           <t>Voir Dimensionnement_est et Contraintes_ouest_utilites pour dimensionnement et implantation recommandee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Presentation pass added: row color coding in Elements_hybrides and one-page Decision_Summary tab.</t>
         </is>
       </c>
     </row>
@@ -947,6 +991,478 @@
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DECISION SUMMARY - DRAINAGE HYBRIDE TRESFOND (PRET POUR PARTAGE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Project strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1) Bande est (arbres): tranchee drainante + underdrain (E01/E02) au lieu d une noue profonde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2) Bande sud (2.0 m): noue lineaire + volume de retention dans le corridor contraint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3) Ouest (utilities): collecte de surface peu profonde priorisee, traverses ponctuelles controlees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4) Exutoire final au bassin de retention via J-BASSIN-IN -&gt; BASSIN-RET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Key dimensions and constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Qdesign (m3/s)</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>East strip total width (m)</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>Inputs!B24</f>
+        <v/>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>&lt;= site 2.5 m</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="F11" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E11,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E11,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E11,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Underdrain trench width x depth (m)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>Inputs!B28&amp;" x "&amp;Inputs!B29</f>
+        <v/>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Tree-compatible trench</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="F12" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E12,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E12,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E12,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Underdrain diameter (mm)</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>Inputs!B30</f>
+        <v/>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Initial recommendation</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="F13" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E13,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E13,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E13,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>South basin corridor width x length (m)</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>Inputs!B34&amp;" x "&amp;Inputs!B35</f>
+        <v/>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Between building and pedestrian road</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="F14" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E14,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E14,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E14,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Basin target depth (m)</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>Inputs!B36</f>
+        <v/>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Adjust with topo survey</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="F15" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Max cover near west utilities (m)</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>Inputs!B39</f>
+        <v/>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Conservative limit</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="F16" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E16,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E16,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E16,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="F17" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E17,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E17,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E17,Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>KPI checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Elements CHECK count</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>Resume_checks!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Nodes CHECK count</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>Resume_checks!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Global status</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>Resume_checks!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Total peak runoff (m3/s)</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>Resume_checks!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Total element storage (m3)</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>Resume_checks!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Retention storage node (m3)</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <f>Resume_checks!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Actions before IFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>- Confirmer positions/degagements exacts des lateraux ouest (AEP/pluvial/sanitaire) avec releves TQC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>- Valider niveau radier/top bassin avec topographie terrain et profil final du cheminement pieton.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- Ajuster diametre underdrain est (Inputs!B30) selon Qdesign final de E02 et critere de remplissage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>- Verifier protection racinaire et details constructifs (barriere racinaire + cleanouts + acces entretien).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A6:H6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H11:H17">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>=$H11="CHECK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21:B26">
+    <cfRule type="expression" priority="2" dxfId="3">
+      <formula>=OR(AND($A21="Elements CHECK count",$B21&gt;0),AND($A22="Nodes CHECK count",$B22&gt;0),AND($A23="Global status",$B23="CHECK"))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6605,6 +7121,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Legend: PIPE=blue, SWALE=green, TRENCH=orange, CHECK=red.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -21862,9 +22385,31 @@
       <c r="AB204" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A2:AB2"/>
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A4:AB204">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>=$B4="PIPE"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>=$B4="SWALE"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>=$B4="TRENCH"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA4:AA204">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>=$AA4="CHECK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U4:U204">
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>=$U4&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refine west branch lengths using plan dimension chain inputs
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -129,6 +129,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -528,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -685,6 +686,20 @@
       <c r="A24" t="inlineStr">
         <is>
           <t>Connexion entre types d elements implementee via AC:AH (controle continuité d invert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Geometrie J-OUEST pilotee par cotes plan dans Inputs!B40:B50 (23.58 m total; 11.1 m amont; 2.3 m pave1; 5.1 m pave2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E05A/E05C sont repartis proportionnellement aux aires (12.5 vs 27.2 m2); E05E est le solde vers le coin sud-ouest (21.9 m2).</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2273,6 +2288,230 @@
       <c r="D39" s="4" t="inlineStr">
         <is>
           <t>Profondeur max recommandee dans zone lateraux ouest (approche conservatrice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>West_chain_total_m</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Somme E05A..E05E (chaine J-OUEST).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>West_amont_to_PU2_chain_m</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Cote plan visible (J-OUEST-AMONT jusqu'a fin zone amont avant troncon pave inferieur).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>West_pave1_short_span_m</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Traverse pave-uni courte (amont).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>West_pave2_span_m</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Traverse pave-uni inferieure (cote plan visible).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>West_grass1_area_m2</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Aire zone gazon 1 (image).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>West_grass2_area_m2</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Aire zone gazon 2 (image).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>West_grass3_area_m2</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Aire zone gazon 3 (image).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>West_grass12_total_m</t>
+        </is>
+      </c>
+      <c r="B47" s="9">
+        <f>B41-B42</f>
+        <v/>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Longueur gazon amont+milieu (derivee).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>West_grass1_len_m</t>
+        </is>
+      </c>
+      <c r="B48" s="9">
+        <f>IFERROR(B47*B44/(B44+B45),"")</f>
+        <v/>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Longueur E05A (repartition proportionnelle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>West_grass2_len_m</t>
+        </is>
+      </c>
+      <c r="B49" s="9">
+        <f>IFERROR(B47*B45/(B44+B45),"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Longueur E05C (repartition proportionnelle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>West_grass3_len_m</t>
+        </is>
+      </c>
+      <c r="B50" s="9">
+        <f>B40-B41-B43</f>
+        <v/>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Longueur E05E (solde vers coin sud-ouest).</t>
         </is>
       </c>
     </row>
@@ -7881,8 +8120,9 @@
           <t>E05B</t>
         </is>
       </c>
-      <c r="F8" s="7" t="n">
-        <v>4</v>
+      <c r="F8" s="15">
+        <f>Inputs!$B$48</f>
+        <v/>
       </c>
       <c r="G8" s="7" t="n">
         <v>0.01</v>
@@ -7959,7 +8199,7 @@
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>Ouest grass 12.5 m2 (surface).</t>
+          <t>Ouest gazon amont - longueur issue cotes plan (chaine 11.1 m repartie par aires).</t>
         </is>
       </c>
       <c r="AC8" s="7" t="n"/>
@@ -8010,8 +8250,9 @@
           <t>E05C</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n">
-        <v>2</v>
+      <c r="F9" s="15">
+        <f>Inputs!$B$42</f>
+        <v/>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.01</v>
@@ -8084,7 +8325,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni 6.7 m2 (caniveau/pipe).</t>
+          <t>Ouest pave-uni court - longueur cotee 2.3 m.</t>
         </is>
       </c>
       <c r="AC9" s="7" t="n"/>
@@ -8135,8 +8376,9 @@
           <t>E05D</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n">
-        <v>8.5</v>
+      <c r="F10" s="15">
+        <f>Inputs!$B$49</f>
+        <v/>
       </c>
       <c r="G10" s="7" t="n">
         <v>0.008999999999999999</v>
@@ -8213,7 +8455,7 @@
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>Ouest grass 27.2 m2 (surface).</t>
+          <t>Ouest gazon milieu - longueur issue cotes plan (chaine 11.1 m repartie par aires).</t>
         </is>
       </c>
       <c r="AC10" s="7" t="n"/>
@@ -8264,8 +8506,9 @@
           <t>E05E</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>5.5</v>
+      <c r="F11" s="15">
+        <f>Inputs!$B$43</f>
+        <v/>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.008999999999999999</v>
@@ -8338,7 +8581,7 @@
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni 37.5 m2 (caniveau/pipe).</t>
+          <t>Ouest pave-uni inferieur - longueur cotee 5.1 m.</t>
         </is>
       </c>
       <c r="AC11" s="7" t="n"/>
@@ -8389,8 +8632,9 @@
           <t>E06</t>
         </is>
       </c>
-      <c r="F12" s="7" t="n">
-        <v>3.6</v>
+      <c r="F12" s="15">
+        <f>Inputs!$B$50</f>
+        <v/>
       </c>
       <c r="G12" s="7" t="n">
         <v>0.008</v>
@@ -8467,7 +8711,7 @@
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
-          <t>Ouest grass 21.9 m2 (surface vers aval).</t>
+          <t>Ouest gazon aval - longueur solde sur chaine totale 23.58 m.</t>
         </is>
       </c>
       <c r="AC12" s="7" t="n"/>

</xml_diff>

<commit_message>
Clarify west zone labels and add top-central tresfond tributary
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -700,6 +700,20 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>E05A/E05C sont repartis proportionnellement aux aires (12.5 vs 27.2 m2); E05E est le solde vers le coin sud-ouest (21.9 m2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Clarification labels image: Z08 = pave-uni principal 37.5 m2 (entre Z05 et Z06).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Zone ajoutee: Z13 = tresfond haut central (aire via Inputs!B51, route E01).</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2512,6 +2526,26 @@
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Longueur E05E (solde vers coin sud-ouest).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Top_central_tresfond_area_m2</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>A renseigner depuis plan releve. Zone tresfond bande haute centrale.</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2796,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ouest vert 1</t>
+          <t>Ouest gazon amont (12.5 m2)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2796,24 +2830,24 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Vers collecte ouest</t>
+          <t>Image: zone verte amont gauche.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Z05</t>
+          <t>Z07</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Ouest vert 2</t>
+          <t>Ouest pave-uni court (6.7 m2)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>GRASS</t>
+          <t>TRESFOND</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -2842,19 +2876,19 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Vers collecte ouest</t>
+          <t>Image: petit troncon pave entre zones gazon.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Z06</t>
+          <t>Z05</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Ouest vert 3</t>
+          <t>Ouest gazon milieu (27.2 m2)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2888,19 +2922,19 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Vers collecte ouest</t>
+          <t>Image: bande verte milieu ouest.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Z07</t>
+          <t>Z08</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Ouest pave-uni</t>
+          <t>Ouest pave-uni principal (37.5 m2)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -2934,19 +2968,19 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Surface mineralisee ouest</t>
+          <t>LOCALISATION: zone pavee entre Z05 et Z06 (pas l'entree pavee externe).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Z08</t>
+          <t>Z06</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ouest vert 4</t>
+          <t>Ouest gazon aval coin sud-ouest (21.9 m2)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2980,7 +3014,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Vers collecte ouest</t>
+          <t>Image: zone verte pres J-OUEST-AVAL.</t>
         </is>
       </c>
     </row>
@@ -3169,16 +3203,33 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Z13</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Tresfond haut central (bande nord centrale)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>TRESFOND</t>
+        </is>
+      </c>
+      <c r="D16" s="7">
+        <f>Inputs!$B$51</f>
+        <v/>
+      </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="8">
         <f>IF(E16&lt;&gt;"",E16,IF(UPPER(TRIM(C16))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C16))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C16))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
         <v/>
       </c>
-      <c r="G16" s="7" t="n"/>
+      <c r="G16" s="7" t="n">
+        <v>8</v>
+      </c>
       <c r="H16" s="8">
         <f>IF(A16="","",Inputs!$B$3/((IF(G16="",Inputs!$B$14,G16)+Inputs!$B$4)^Inputs!$B$5))</f>
         <v/>
@@ -3187,8 +3238,16 @@
         <f>IF(A16="","",2.78E-7*F16*D16*H16)</f>
         <v/>
       </c>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Ajoute pour inclure le tresfond central haut; saisir aire exacte Inputs!B51.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>

</xml_diff>

<commit_message>
Fix E03/E04 overlap and model basin footprint as non-contributing
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -714,6 +714,34 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>Zone ajoutee: Z13 = tresfond haut central (aire via Inputs!B51, route E01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Correction topologie: E03 (P-03-&gt;J-BASSIN-IN) = 16.1 m; E04 = 20 m (J-OUEST-AVAL-&gt;J-BASSIN-IN).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E04 ne superpose plus E03; E06 desactive pour eviter double chemin parallelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Z09 est defini BASIN (empreinte bassin), non contributif par defaut (Inputs!B52=NO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Bassin retention longueur mise a 20 m (Inputs!B35) selon releve plan.</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2211,7 +2239,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>29.4</v>
+        <v>20</v>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
@@ -2220,7 +2248,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Longueur exploitable du bassin lineaire sud.</t>
+          <t>Longueur bassin retention (plan utilisateur) - remplace valeur preliminaire 29.4 m.</t>
         </is>
       </c>
     </row>
@@ -2546,6 +2574,28 @@
       <c r="D51" s="4" t="inlineStr">
         <is>
           <t>A renseigner depuis plan releve. Zone tresfond bande haute centrale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Include_basin_footprint_runoff (YES/NO)</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>NO recommande: empreinte bassin n'est pas contributive au bassin lui-meme.</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2721,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr"/>
       <c r="F4" s="8">
-        <f>IF(E4&lt;&gt;"",E4,IF(UPPER(TRIM(C4))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C4))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C4))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E4&lt;&gt;"",E4,IF(UPPER(TRIM(C4))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C4))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C4))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C4))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G4" s="7" t="n">
@@ -2717,7 +2767,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="8">
-        <f>IF(E5&lt;&gt;"",E5,IF(UPPER(TRIM(C5))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C5))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C5))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E5&lt;&gt;"",E5,IF(UPPER(TRIM(C5))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C5))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C5))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C5))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G5" s="7" t="n">
@@ -2733,7 +2783,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -2763,7 +2813,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr"/>
       <c r="F6" s="8">
-        <f>IF(E6&lt;&gt;"",E6,IF(UPPER(TRIM(C6))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C6))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C6))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E6&lt;&gt;"",E6,IF(UPPER(TRIM(C6))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C6))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C6))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C6))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G6" s="7" t="n">
@@ -2809,7 +2859,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="8">
-        <f>IF(E7&lt;&gt;"",E7,IF(UPPER(TRIM(C7))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C7))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C7))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E7&lt;&gt;"",E7,IF(UPPER(TRIM(C7))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C7))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C7))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C7))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G7" s="7" t="n">
@@ -2855,7 +2905,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr"/>
       <c r="F8" s="8">
-        <f>IF(E8&lt;&gt;"",E8,IF(UPPER(TRIM(C8))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C8))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C8))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E8&lt;&gt;"",E8,IF(UPPER(TRIM(C8))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C8))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C8))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C8))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G8" s="7" t="n">
@@ -2901,7 +2951,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="8">
-        <f>IF(E9&lt;&gt;"",E9,IF(UPPER(TRIM(C9))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C9))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C9))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E9&lt;&gt;"",E9,IF(UPPER(TRIM(C9))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C9))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C9))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C9))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G9" s="7" t="n">
@@ -2947,7 +2997,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr"/>
       <c r="F10" s="8">
-        <f>IF(E10&lt;&gt;"",E10,IF(UPPER(TRIM(C10))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C10))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C10))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E10&lt;&gt;"",E10,IF(UPPER(TRIM(C10))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C10))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C10))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C10))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G10" s="7" t="n">
@@ -2993,7 +3043,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="8">
-        <f>IF(E11&lt;&gt;"",E11,IF(UPPER(TRIM(C11))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C11))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C11))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E11&lt;&gt;"",E11,IF(UPPER(TRIM(C11))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C11))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C11))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C11))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G11" s="7" t="n">
@@ -3026,12 +3076,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Bande sud verte centrale</t>
+          <t>Empreinte bassin retention (zone de stockage)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>GRASS</t>
+          <t>BASIN</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
@@ -3039,7 +3089,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr"/>
       <c r="F12" s="8">
-        <f>IF(E12&lt;&gt;"",E12,IF(UPPER(TRIM(C12))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C12))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C12))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E12&lt;&gt;"",E12,IF(UPPER(TRIM(C12))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C12))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C12))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C12))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G12" s="7" t="n">
@@ -3053,14 +3103,10 @@
         <f>IF(A12="","",2.78E-7*F12*D12*H12)</f>
         <v/>
       </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>E04</t>
-        </is>
-      </c>
+      <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Vers noue sud</t>
+          <t>Non contributive par defaut (Inputs!B52=NO). Mettre YES pour sensibilité si requis.</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3131,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="8">
-        <f>IF(E13&lt;&gt;"",E13,IF(UPPER(TRIM(C13))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C13))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C13))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E13&lt;&gt;"",E13,IF(UPPER(TRIM(C13))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C13))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C13))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C13))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G13" s="7" t="n">
@@ -3131,7 +3177,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr"/>
       <c r="F14" s="8">
-        <f>IF(E14&lt;&gt;"",E14,IF(UPPER(TRIM(C14))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C14))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C14))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E14&lt;&gt;"",E14,IF(UPPER(TRIM(C14))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C14))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C14))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C14))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G14" s="7" t="n">
@@ -3147,7 +3193,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -3177,7 +3223,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="8">
-        <f>IF(E15&lt;&gt;"",E15,IF(UPPER(TRIM(C15))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C15))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C15))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E15&lt;&gt;"",E15,IF(UPPER(TRIM(C15))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C15))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C15))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C15))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G15" s="7" t="n">
@@ -3193,7 +3239,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -3224,7 +3270,7 @@
       </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="8">
-        <f>IF(E16&lt;&gt;"",E16,IF(UPPER(TRIM(C16))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C16))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C16))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E16&lt;&gt;"",E16,IF(UPPER(TRIM(C16))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C16))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C16))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C16))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G16" s="7" t="n">
@@ -3240,7 +3286,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -3256,7 +3302,7 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="8">
-        <f>IF(E17&lt;&gt;"",E17,IF(UPPER(TRIM(C17))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C17))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C17))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E17&lt;&gt;"",E17,IF(UPPER(TRIM(C17))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C17))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C17))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C17))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G17" s="7" t="n"/>
@@ -3278,7 +3324,7 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="8">
-        <f>IF(E18&lt;&gt;"",E18,IF(UPPER(TRIM(C18))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C18))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C18))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E18&lt;&gt;"",E18,IF(UPPER(TRIM(C18))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C18))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C18))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C18))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G18" s="7" t="n"/>
@@ -3300,7 +3346,7 @@
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="8">
-        <f>IF(E19&lt;&gt;"",E19,IF(UPPER(TRIM(C19))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C19))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C19))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E19&lt;&gt;"",E19,IF(UPPER(TRIM(C19))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C19))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C19))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C19))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G19" s="7" t="n"/>
@@ -3322,7 +3368,7 @@
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="8">
-        <f>IF(E20&lt;&gt;"",E20,IF(UPPER(TRIM(C20))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C20))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C20))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E20&lt;&gt;"",E20,IF(UPPER(TRIM(C20))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C20))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C20))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C20))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G20" s="7" t="n"/>
@@ -3344,7 +3390,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="8">
-        <f>IF(E21&lt;&gt;"",E21,IF(UPPER(TRIM(C21))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C21))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C21))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E21&lt;&gt;"",E21,IF(UPPER(TRIM(C21))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C21))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C21))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C21))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G21" s="7" t="n"/>
@@ -3366,7 +3412,7 @@
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="8">
-        <f>IF(E22&lt;&gt;"",E22,IF(UPPER(TRIM(C22))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C22))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C22))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E22&lt;&gt;"",E22,IF(UPPER(TRIM(C22))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C22))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C22))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C22))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G22" s="7" t="n"/>
@@ -3388,7 +3434,7 @@
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="8">
-        <f>IF(E23&lt;&gt;"",E23,IF(UPPER(TRIM(C23))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C23))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C23))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E23&lt;&gt;"",E23,IF(UPPER(TRIM(C23))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C23))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C23))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C23))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G23" s="7" t="n"/>
@@ -3410,7 +3456,7 @@
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="8">
-        <f>IF(E24&lt;&gt;"",E24,IF(UPPER(TRIM(C24))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C24))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C24))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E24&lt;&gt;"",E24,IF(UPPER(TRIM(C24))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C24))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C24))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C24))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G24" s="7" t="n"/>
@@ -3432,7 +3478,7 @@
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="8">
-        <f>IF(E25&lt;&gt;"",E25,IF(UPPER(TRIM(C25))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C25))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C25))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E25&lt;&gt;"",E25,IF(UPPER(TRIM(C25))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C25))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C25))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C25))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G25" s="7" t="n"/>
@@ -3454,7 +3500,7 @@
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="8">
-        <f>IF(E26&lt;&gt;"",E26,IF(UPPER(TRIM(C26))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C26))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C26))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E26&lt;&gt;"",E26,IF(UPPER(TRIM(C26))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C26))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C26))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C26))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G26" s="7" t="n"/>
@@ -3476,7 +3522,7 @@
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="8">
-        <f>IF(E27&lt;&gt;"",E27,IF(UPPER(TRIM(C27))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C27))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C27))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E27&lt;&gt;"",E27,IF(UPPER(TRIM(C27))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C27))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C27))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C27))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G27" s="7" t="n"/>
@@ -3498,7 +3544,7 @@
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="8">
-        <f>IF(E28&lt;&gt;"",E28,IF(UPPER(TRIM(C28))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C28))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C28))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E28&lt;&gt;"",E28,IF(UPPER(TRIM(C28))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C28))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C28))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C28))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G28" s="7" t="n"/>
@@ -3520,7 +3566,7 @@
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="8">
-        <f>IF(E29&lt;&gt;"",E29,IF(UPPER(TRIM(C29))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C29))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C29))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E29&lt;&gt;"",E29,IF(UPPER(TRIM(C29))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C29))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C29))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C29))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G29" s="7" t="n"/>
@@ -3542,7 +3588,7 @@
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="8">
-        <f>IF(E30&lt;&gt;"",E30,IF(UPPER(TRIM(C30))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C30))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C30))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E30&lt;&gt;"",E30,IF(UPPER(TRIM(C30))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C30))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C30))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C30))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G30" s="7" t="n"/>
@@ -3564,7 +3610,7 @@
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="8">
-        <f>IF(E31&lt;&gt;"",E31,IF(UPPER(TRIM(C31))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C31))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C31))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E31&lt;&gt;"",E31,IF(UPPER(TRIM(C31))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C31))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C31))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C31))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G31" s="7" t="n"/>
@@ -3586,7 +3632,7 @@
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="8">
-        <f>IF(E32&lt;&gt;"",E32,IF(UPPER(TRIM(C32))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C32))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C32))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E32&lt;&gt;"",E32,IF(UPPER(TRIM(C32))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C32))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C32))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C32))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G32" s="7" t="n"/>
@@ -3608,7 +3654,7 @@
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="8">
-        <f>IF(E33&lt;&gt;"",E33,IF(UPPER(TRIM(C33))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C33))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C33))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E33&lt;&gt;"",E33,IF(UPPER(TRIM(C33))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C33))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C33))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C33))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G33" s="7" t="n"/>
@@ -3630,7 +3676,7 @@
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="8">
-        <f>IF(E34&lt;&gt;"",E34,IF(UPPER(TRIM(C34))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C34))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C34))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E34&lt;&gt;"",E34,IF(UPPER(TRIM(C34))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C34))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C34))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C34))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G34" s="7" t="n"/>
@@ -3652,7 +3698,7 @@
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="8">
-        <f>IF(E35&lt;&gt;"",E35,IF(UPPER(TRIM(C35))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C35))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C35))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E35&lt;&gt;"",E35,IF(UPPER(TRIM(C35))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C35))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C35))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C35))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G35" s="7" t="n"/>
@@ -3674,7 +3720,7 @@
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="8">
-        <f>IF(E36&lt;&gt;"",E36,IF(UPPER(TRIM(C36))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C36))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C36))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E36&lt;&gt;"",E36,IF(UPPER(TRIM(C36))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C36))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C36))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C36))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G36" s="7" t="n"/>
@@ -3696,7 +3742,7 @@
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="8">
-        <f>IF(E37&lt;&gt;"",E37,IF(UPPER(TRIM(C37))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C37))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C37))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E37&lt;&gt;"",E37,IF(UPPER(TRIM(C37))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C37))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C37))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C37))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G37" s="7" t="n"/>
@@ -3718,7 +3764,7 @@
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="8">
-        <f>IF(E38&lt;&gt;"",E38,IF(UPPER(TRIM(C38))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C38))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C38))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E38&lt;&gt;"",E38,IF(UPPER(TRIM(C38))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C38))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C38))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C38))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G38" s="7" t="n"/>
@@ -3740,7 +3786,7 @@
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="8">
-        <f>IF(E39&lt;&gt;"",E39,IF(UPPER(TRIM(C39))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C39))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C39))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E39&lt;&gt;"",E39,IF(UPPER(TRIM(C39))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C39))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C39))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C39))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G39" s="7" t="n"/>
@@ -3762,7 +3808,7 @@
       <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="8">
-        <f>IF(E40&lt;&gt;"",E40,IF(UPPER(TRIM(C40))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C40))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C40))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E40&lt;&gt;"",E40,IF(UPPER(TRIM(C40))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C40))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C40))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C40))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G40" s="7" t="n"/>
@@ -3784,7 +3830,7 @@
       <c r="D41" s="7" t="n"/>
       <c r="E41" s="7" t="n"/>
       <c r="F41" s="8">
-        <f>IF(E41&lt;&gt;"",E41,IF(UPPER(TRIM(C41))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C41))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C41))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E41&lt;&gt;"",E41,IF(UPPER(TRIM(C41))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C41))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C41))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C41))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G41" s="7" t="n"/>
@@ -3806,7 +3852,7 @@
       <c r="D42" s="7" t="n"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="8">
-        <f>IF(E42&lt;&gt;"",E42,IF(UPPER(TRIM(C42))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C42))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C42))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E42&lt;&gt;"",E42,IF(UPPER(TRIM(C42))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C42))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C42))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C42))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G42" s="7" t="n"/>
@@ -3828,7 +3874,7 @@
       <c r="D43" s="7" t="n"/>
       <c r="E43" s="7" t="n"/>
       <c r="F43" s="8">
-        <f>IF(E43&lt;&gt;"",E43,IF(UPPER(TRIM(C43))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C43))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C43))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E43&lt;&gt;"",E43,IF(UPPER(TRIM(C43))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C43))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C43))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C43))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G43" s="7" t="n"/>
@@ -3850,7 +3896,7 @@
       <c r="D44" s="7" t="n"/>
       <c r="E44" s="7" t="n"/>
       <c r="F44" s="8">
-        <f>IF(E44&lt;&gt;"",E44,IF(UPPER(TRIM(C44))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C44))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C44))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E44&lt;&gt;"",E44,IF(UPPER(TRIM(C44))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C44))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C44))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C44))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G44" s="7" t="n"/>
@@ -3872,7 +3918,7 @@
       <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="8">
-        <f>IF(E45&lt;&gt;"",E45,IF(UPPER(TRIM(C45))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C45))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C45))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E45&lt;&gt;"",E45,IF(UPPER(TRIM(C45))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C45))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C45))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C45))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G45" s="7" t="n"/>
@@ -3894,7 +3940,7 @@
       <c r="D46" s="7" t="n"/>
       <c r="E46" s="7" t="n"/>
       <c r="F46" s="8">
-        <f>IF(E46&lt;&gt;"",E46,IF(UPPER(TRIM(C46))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C46))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C46))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E46&lt;&gt;"",E46,IF(UPPER(TRIM(C46))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C46))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C46))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C46))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G46" s="7" t="n"/>
@@ -3916,7 +3962,7 @@
       <c r="D47" s="7" t="n"/>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="8">
-        <f>IF(E47&lt;&gt;"",E47,IF(UPPER(TRIM(C47))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C47))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C47))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E47&lt;&gt;"",E47,IF(UPPER(TRIM(C47))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C47))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C47))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C47))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G47" s="7" t="n"/>
@@ -3938,7 +3984,7 @@
       <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="8">
-        <f>IF(E48&lt;&gt;"",E48,IF(UPPER(TRIM(C48))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C48))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C48))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E48&lt;&gt;"",E48,IF(UPPER(TRIM(C48))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C48))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C48))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C48))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G48" s="7" t="n"/>
@@ -3960,7 +4006,7 @@
       <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="8">
-        <f>IF(E49&lt;&gt;"",E49,IF(UPPER(TRIM(C49))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C49))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C49))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E49&lt;&gt;"",E49,IF(UPPER(TRIM(C49))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C49))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C49))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C49))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G49" s="7" t="n"/>
@@ -3982,7 +4028,7 @@
       <c r="D50" s="7" t="n"/>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="8">
-        <f>IF(E50&lt;&gt;"",E50,IF(UPPER(TRIM(C50))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C50))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C50))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E50&lt;&gt;"",E50,IF(UPPER(TRIM(C50))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C50))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C50))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C50))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G50" s="7" t="n"/>
@@ -4004,7 +4050,7 @@
       <c r="D51" s="7" t="n"/>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="8">
-        <f>IF(E51&lt;&gt;"",E51,IF(UPPER(TRIM(C51))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C51))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C51))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E51&lt;&gt;"",E51,IF(UPPER(TRIM(C51))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C51))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C51))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C51))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G51" s="7" t="n"/>
@@ -4026,7 +4072,7 @@
       <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="8">
-        <f>IF(E52&lt;&gt;"",E52,IF(UPPER(TRIM(C52))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C52))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C52))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E52&lt;&gt;"",E52,IF(UPPER(TRIM(C52))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C52))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C52))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C52))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G52" s="7" t="n"/>
@@ -4048,7 +4094,7 @@
       <c r="D53" s="7" t="n"/>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="8">
-        <f>IF(E53&lt;&gt;"",E53,IF(UPPER(TRIM(C53))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C53))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C53))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E53&lt;&gt;"",E53,IF(UPPER(TRIM(C53))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C53))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C53))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C53))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G53" s="7" t="n"/>
@@ -4070,7 +4116,7 @@
       <c r="D54" s="7" t="n"/>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="8">
-        <f>IF(E54&lt;&gt;"",E54,IF(UPPER(TRIM(C54))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C54))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C54))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E54&lt;&gt;"",E54,IF(UPPER(TRIM(C54))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C54))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C54))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C54))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G54" s="7" t="n"/>
@@ -4092,7 +4138,7 @@
       <c r="D55" s="7" t="n"/>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="8">
-        <f>IF(E55&lt;&gt;"",E55,IF(UPPER(TRIM(C55))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C55))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C55))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E55&lt;&gt;"",E55,IF(UPPER(TRIM(C55))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C55))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C55))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C55))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G55" s="7" t="n"/>
@@ -4114,7 +4160,7 @@
       <c r="D56" s="7" t="n"/>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="8">
-        <f>IF(E56&lt;&gt;"",E56,IF(UPPER(TRIM(C56))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C56))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C56))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E56&lt;&gt;"",E56,IF(UPPER(TRIM(C56))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C56))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C56))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C56))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G56" s="7" t="n"/>
@@ -4136,7 +4182,7 @@
       <c r="D57" s="7" t="n"/>
       <c r="E57" s="7" t="n"/>
       <c r="F57" s="8">
-        <f>IF(E57&lt;&gt;"",E57,IF(UPPER(TRIM(C57))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C57))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C57))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E57&lt;&gt;"",E57,IF(UPPER(TRIM(C57))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C57))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C57))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C57))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G57" s="7" t="n"/>
@@ -4158,7 +4204,7 @@
       <c r="D58" s="7" t="n"/>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="8">
-        <f>IF(E58&lt;&gt;"",E58,IF(UPPER(TRIM(C58))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C58))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C58))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E58&lt;&gt;"",E58,IF(UPPER(TRIM(C58))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C58))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C58))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C58))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G58" s="7" t="n"/>
@@ -4180,7 +4226,7 @@
       <c r="D59" s="7" t="n"/>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="8">
-        <f>IF(E59&lt;&gt;"",E59,IF(UPPER(TRIM(C59))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C59))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C59))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E59&lt;&gt;"",E59,IF(UPPER(TRIM(C59))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C59))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C59))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C59))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G59" s="7" t="n"/>
@@ -4202,7 +4248,7 @@
       <c r="D60" s="7" t="n"/>
       <c r="E60" s="7" t="n"/>
       <c r="F60" s="8">
-        <f>IF(E60&lt;&gt;"",E60,IF(UPPER(TRIM(C60))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C60))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C60))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E60&lt;&gt;"",E60,IF(UPPER(TRIM(C60))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C60))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C60))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C60))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G60" s="7" t="n"/>
@@ -4224,7 +4270,7 @@
       <c r="D61" s="7" t="n"/>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="8">
-        <f>IF(E61&lt;&gt;"",E61,IF(UPPER(TRIM(C61))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C61))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C61))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E61&lt;&gt;"",E61,IF(UPPER(TRIM(C61))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C61))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C61))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C61))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G61" s="7" t="n"/>
@@ -4246,7 +4292,7 @@
       <c r="D62" s="7" t="n"/>
       <c r="E62" s="7" t="n"/>
       <c r="F62" s="8">
-        <f>IF(E62&lt;&gt;"",E62,IF(UPPER(TRIM(C62))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C62))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C62))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E62&lt;&gt;"",E62,IF(UPPER(TRIM(C62))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C62))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C62))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C62))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G62" s="7" t="n"/>
@@ -4268,7 +4314,7 @@
       <c r="D63" s="7" t="n"/>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="8">
-        <f>IF(E63&lt;&gt;"",E63,IF(UPPER(TRIM(C63))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C63))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C63))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E63&lt;&gt;"",E63,IF(UPPER(TRIM(C63))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C63))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C63))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C63))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G63" s="7" t="n"/>
@@ -4290,7 +4336,7 @@
       <c r="D64" s="7" t="n"/>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="8">
-        <f>IF(E64&lt;&gt;"",E64,IF(UPPER(TRIM(C64))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C64))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C64))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E64&lt;&gt;"",E64,IF(UPPER(TRIM(C64))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C64))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C64))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C64))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G64" s="7" t="n"/>
@@ -4312,7 +4358,7 @@
       <c r="D65" s="7" t="n"/>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="8">
-        <f>IF(E65&lt;&gt;"",E65,IF(UPPER(TRIM(C65))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C65))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C65))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E65&lt;&gt;"",E65,IF(UPPER(TRIM(C65))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C65))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C65))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C65))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G65" s="7" t="n"/>
@@ -4334,7 +4380,7 @@
       <c r="D66" s="7" t="n"/>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="8">
-        <f>IF(E66&lt;&gt;"",E66,IF(UPPER(TRIM(C66))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C66))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C66))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E66&lt;&gt;"",E66,IF(UPPER(TRIM(C66))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C66))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C66))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C66))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G66" s="7" t="n"/>
@@ -4356,7 +4402,7 @@
       <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="8">
-        <f>IF(E67&lt;&gt;"",E67,IF(UPPER(TRIM(C67))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C67))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C67))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E67&lt;&gt;"",E67,IF(UPPER(TRIM(C67))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C67))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C67))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C67))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G67" s="7" t="n"/>
@@ -4378,7 +4424,7 @@
       <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="8">
-        <f>IF(E68&lt;&gt;"",E68,IF(UPPER(TRIM(C68))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C68))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C68))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E68&lt;&gt;"",E68,IF(UPPER(TRIM(C68))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C68))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C68))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C68))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G68" s="7" t="n"/>
@@ -4400,7 +4446,7 @@
       <c r="D69" s="7" t="n"/>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="8">
-        <f>IF(E69&lt;&gt;"",E69,IF(UPPER(TRIM(C69))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C69))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C69))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E69&lt;&gt;"",E69,IF(UPPER(TRIM(C69))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C69))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C69))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C69))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G69" s="7" t="n"/>
@@ -4422,7 +4468,7 @@
       <c r="D70" s="7" t="n"/>
       <c r="E70" s="7" t="n"/>
       <c r="F70" s="8">
-        <f>IF(E70&lt;&gt;"",E70,IF(UPPER(TRIM(C70))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C70))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C70))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E70&lt;&gt;"",E70,IF(UPPER(TRIM(C70))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C70))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C70))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C70))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G70" s="7" t="n"/>
@@ -4444,7 +4490,7 @@
       <c r="D71" s="7" t="n"/>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="8">
-        <f>IF(E71&lt;&gt;"",E71,IF(UPPER(TRIM(C71))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C71))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C71))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E71&lt;&gt;"",E71,IF(UPPER(TRIM(C71))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C71))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C71))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C71))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G71" s="7" t="n"/>
@@ -4466,7 +4512,7 @@
       <c r="D72" s="7" t="n"/>
       <c r="E72" s="7" t="n"/>
       <c r="F72" s="8">
-        <f>IF(E72&lt;&gt;"",E72,IF(UPPER(TRIM(C72))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C72))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C72))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E72&lt;&gt;"",E72,IF(UPPER(TRIM(C72))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C72))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C72))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C72))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G72" s="7" t="n"/>
@@ -4488,7 +4534,7 @@
       <c r="D73" s="7" t="n"/>
       <c r="E73" s="7" t="n"/>
       <c r="F73" s="8">
-        <f>IF(E73&lt;&gt;"",E73,IF(UPPER(TRIM(C73))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C73))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C73))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E73&lt;&gt;"",E73,IF(UPPER(TRIM(C73))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C73))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C73))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C73))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G73" s="7" t="n"/>
@@ -4510,7 +4556,7 @@
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="8">
-        <f>IF(E74&lt;&gt;"",E74,IF(UPPER(TRIM(C74))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C74))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C74))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E74&lt;&gt;"",E74,IF(UPPER(TRIM(C74))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C74))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C74))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C74))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G74" s="7" t="n"/>
@@ -4532,7 +4578,7 @@
       <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="8">
-        <f>IF(E75&lt;&gt;"",E75,IF(UPPER(TRIM(C75))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C75))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C75))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E75&lt;&gt;"",E75,IF(UPPER(TRIM(C75))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C75))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C75))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C75))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G75" s="7" t="n"/>
@@ -4554,7 +4600,7 @@
       <c r="D76" s="7" t="n"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="8">
-        <f>IF(E76&lt;&gt;"",E76,IF(UPPER(TRIM(C76))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C76))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C76))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E76&lt;&gt;"",E76,IF(UPPER(TRIM(C76))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C76))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C76))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C76))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G76" s="7" t="n"/>
@@ -4576,7 +4622,7 @@
       <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="8">
-        <f>IF(E77&lt;&gt;"",E77,IF(UPPER(TRIM(C77))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C77))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C77))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E77&lt;&gt;"",E77,IF(UPPER(TRIM(C77))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C77))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C77))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C77))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G77" s="7" t="n"/>
@@ -4598,7 +4644,7 @@
       <c r="D78" s="7" t="n"/>
       <c r="E78" s="7" t="n"/>
       <c r="F78" s="8">
-        <f>IF(E78&lt;&gt;"",E78,IF(UPPER(TRIM(C78))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C78))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C78))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E78&lt;&gt;"",E78,IF(UPPER(TRIM(C78))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C78))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C78))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C78))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G78" s="7" t="n"/>
@@ -4620,7 +4666,7 @@
       <c r="D79" s="7" t="n"/>
       <c r="E79" s="7" t="n"/>
       <c r="F79" s="8">
-        <f>IF(E79&lt;&gt;"",E79,IF(UPPER(TRIM(C79))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C79))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C79))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E79&lt;&gt;"",E79,IF(UPPER(TRIM(C79))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C79))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C79))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C79))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G79" s="7" t="n"/>
@@ -4642,7 +4688,7 @@
       <c r="D80" s="7" t="n"/>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="8">
-        <f>IF(E80&lt;&gt;"",E80,IF(UPPER(TRIM(C80))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C80))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C80))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E80&lt;&gt;"",E80,IF(UPPER(TRIM(C80))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C80))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C80))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C80))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G80" s="7" t="n"/>
@@ -4664,7 +4710,7 @@
       <c r="D81" s="7" t="n"/>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="8">
-        <f>IF(E81&lt;&gt;"",E81,IF(UPPER(TRIM(C81))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C81))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C81))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E81&lt;&gt;"",E81,IF(UPPER(TRIM(C81))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C81))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C81))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C81))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G81" s="7" t="n"/>
@@ -4686,7 +4732,7 @@
       <c r="D82" s="7" t="n"/>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="8">
-        <f>IF(E82&lt;&gt;"",E82,IF(UPPER(TRIM(C82))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C82))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C82))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E82&lt;&gt;"",E82,IF(UPPER(TRIM(C82))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C82))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C82))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C82))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G82" s="7" t="n"/>
@@ -4708,7 +4754,7 @@
       <c r="D83" s="7" t="n"/>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="8">
-        <f>IF(E83&lt;&gt;"",E83,IF(UPPER(TRIM(C83))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C83))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C83))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E83&lt;&gt;"",E83,IF(UPPER(TRIM(C83))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C83))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C83))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C83))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G83" s="7" t="n"/>
@@ -4730,7 +4776,7 @@
       <c r="D84" s="7" t="n"/>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="8">
-        <f>IF(E84&lt;&gt;"",E84,IF(UPPER(TRIM(C84))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C84))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C84))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E84&lt;&gt;"",E84,IF(UPPER(TRIM(C84))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C84))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C84))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C84))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G84" s="7" t="n"/>
@@ -4752,7 +4798,7 @@
       <c r="D85" s="7" t="n"/>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="8">
-        <f>IF(E85&lt;&gt;"",E85,IF(UPPER(TRIM(C85))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C85))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C85))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E85&lt;&gt;"",E85,IF(UPPER(TRIM(C85))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C85))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C85))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C85))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G85" s="7" t="n"/>
@@ -4774,7 +4820,7 @@
       <c r="D86" s="7" t="n"/>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="8">
-        <f>IF(E86&lt;&gt;"",E86,IF(UPPER(TRIM(C86))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C86))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C86))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E86&lt;&gt;"",E86,IF(UPPER(TRIM(C86))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C86))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C86))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C86))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G86" s="7" t="n"/>
@@ -4796,7 +4842,7 @@
       <c r="D87" s="7" t="n"/>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="8">
-        <f>IF(E87&lt;&gt;"",E87,IF(UPPER(TRIM(C87))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C87))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C87))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E87&lt;&gt;"",E87,IF(UPPER(TRIM(C87))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C87))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C87))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C87))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G87" s="7" t="n"/>
@@ -4818,7 +4864,7 @@
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="8">
-        <f>IF(E88&lt;&gt;"",E88,IF(UPPER(TRIM(C88))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C88))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C88))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E88&lt;&gt;"",E88,IF(UPPER(TRIM(C88))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C88))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C88))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C88))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G88" s="7" t="n"/>
@@ -4840,7 +4886,7 @@
       <c r="D89" s="7" t="n"/>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="8">
-        <f>IF(E89&lt;&gt;"",E89,IF(UPPER(TRIM(C89))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C89))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C89))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E89&lt;&gt;"",E89,IF(UPPER(TRIM(C89))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C89))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C89))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C89))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G89" s="7" t="n"/>
@@ -4862,7 +4908,7 @@
       <c r="D90" s="7" t="n"/>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="8">
-        <f>IF(E90&lt;&gt;"",E90,IF(UPPER(TRIM(C90))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C90))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C90))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E90&lt;&gt;"",E90,IF(UPPER(TRIM(C90))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C90))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C90))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C90))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G90" s="7" t="n"/>
@@ -4884,7 +4930,7 @@
       <c r="D91" s="7" t="n"/>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="8">
-        <f>IF(E91&lt;&gt;"",E91,IF(UPPER(TRIM(C91))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C91))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C91))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E91&lt;&gt;"",E91,IF(UPPER(TRIM(C91))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C91))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C91))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C91))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G91" s="7" t="n"/>
@@ -4906,7 +4952,7 @@
       <c r="D92" s="7" t="n"/>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="8">
-        <f>IF(E92&lt;&gt;"",E92,IF(UPPER(TRIM(C92))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C92))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C92))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E92&lt;&gt;"",E92,IF(UPPER(TRIM(C92))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C92))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C92))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C92))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G92" s="7" t="n"/>
@@ -4928,7 +4974,7 @@
       <c r="D93" s="7" t="n"/>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="8">
-        <f>IF(E93&lt;&gt;"",E93,IF(UPPER(TRIM(C93))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C93))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C93))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E93&lt;&gt;"",E93,IF(UPPER(TRIM(C93))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C93))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C93))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C93))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G93" s="7" t="n"/>
@@ -4950,7 +4996,7 @@
       <c r="D94" s="7" t="n"/>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="8">
-        <f>IF(E94&lt;&gt;"",E94,IF(UPPER(TRIM(C94))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C94))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C94))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E94&lt;&gt;"",E94,IF(UPPER(TRIM(C94))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C94))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C94))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C94))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G94" s="7" t="n"/>
@@ -4972,7 +5018,7 @@
       <c r="D95" s="7" t="n"/>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="8">
-        <f>IF(E95&lt;&gt;"",E95,IF(UPPER(TRIM(C95))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C95))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C95))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E95&lt;&gt;"",E95,IF(UPPER(TRIM(C95))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C95))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C95))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C95))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G95" s="7" t="n"/>
@@ -4994,7 +5040,7 @@
       <c r="D96" s="7" t="n"/>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="8">
-        <f>IF(E96&lt;&gt;"",E96,IF(UPPER(TRIM(C96))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C96))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C96))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E96&lt;&gt;"",E96,IF(UPPER(TRIM(C96))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C96))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C96))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C96))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G96" s="7" t="n"/>
@@ -5016,7 +5062,7 @@
       <c r="D97" s="7" t="n"/>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="8">
-        <f>IF(E97&lt;&gt;"",E97,IF(UPPER(TRIM(C97))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C97))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C97))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E97&lt;&gt;"",E97,IF(UPPER(TRIM(C97))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C97))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C97))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C97))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G97" s="7" t="n"/>
@@ -5038,7 +5084,7 @@
       <c r="D98" s="7" t="n"/>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="8">
-        <f>IF(E98&lt;&gt;"",E98,IF(UPPER(TRIM(C98))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C98))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C98))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E98&lt;&gt;"",E98,IF(UPPER(TRIM(C98))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C98))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C98))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C98))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G98" s="7" t="n"/>
@@ -5060,7 +5106,7 @@
       <c r="D99" s="7" t="n"/>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="8">
-        <f>IF(E99&lt;&gt;"",E99,IF(UPPER(TRIM(C99))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C99))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C99))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E99&lt;&gt;"",E99,IF(UPPER(TRIM(C99))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C99))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C99))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C99))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G99" s="7" t="n"/>
@@ -5082,7 +5128,7 @@
       <c r="D100" s="7" t="n"/>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="8">
-        <f>IF(E100&lt;&gt;"",E100,IF(UPPER(TRIM(C100))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C100))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C100))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E100&lt;&gt;"",E100,IF(UPPER(TRIM(C100))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C100))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C100))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C100))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G100" s="7" t="n"/>
@@ -5104,7 +5150,7 @@
       <c r="D101" s="7" t="n"/>
       <c r="E101" s="7" t="n"/>
       <c r="F101" s="8">
-        <f>IF(E101&lt;&gt;"",E101,IF(UPPER(TRIM(C101))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C101))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C101))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E101&lt;&gt;"",E101,IF(UPPER(TRIM(C101))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C101))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C101))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C101))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G101" s="7" t="n"/>
@@ -5126,7 +5172,7 @@
       <c r="D102" s="7" t="n"/>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="8">
-        <f>IF(E102&lt;&gt;"",E102,IF(UPPER(TRIM(C102))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C102))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C102))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E102&lt;&gt;"",E102,IF(UPPER(TRIM(C102))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C102))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C102))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C102))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G102" s="7" t="n"/>
@@ -5148,7 +5194,7 @@
       <c r="D103" s="7" t="n"/>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="8">
-        <f>IF(E103&lt;&gt;"",E103,IF(UPPER(TRIM(C103))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C103))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C103))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E103&lt;&gt;"",E103,IF(UPPER(TRIM(C103))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C103))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C103))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C103))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G103" s="7" t="n"/>
@@ -5170,7 +5216,7 @@
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="8">
-        <f>IF(E104&lt;&gt;"",E104,IF(UPPER(TRIM(C104))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C104))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C104))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E104&lt;&gt;"",E104,IF(UPPER(TRIM(C104))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C104))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C104))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C104))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G104" s="7" t="n"/>
@@ -5192,7 +5238,7 @@
       <c r="D105" s="7" t="n"/>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="8">
-        <f>IF(E105&lt;&gt;"",E105,IF(UPPER(TRIM(C105))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C105))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C105))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E105&lt;&gt;"",E105,IF(UPPER(TRIM(C105))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C105))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C105))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C105))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G105" s="7" t="n"/>
@@ -5214,7 +5260,7 @@
       <c r="D106" s="7" t="n"/>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="8">
-        <f>IF(E106&lt;&gt;"",E106,IF(UPPER(TRIM(C106))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C106))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C106))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E106&lt;&gt;"",E106,IF(UPPER(TRIM(C106))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C106))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C106))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C106))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G106" s="7" t="n"/>
@@ -5236,7 +5282,7 @@
       <c r="D107" s="7" t="n"/>
       <c r="E107" s="7" t="n"/>
       <c r="F107" s="8">
-        <f>IF(E107&lt;&gt;"",E107,IF(UPPER(TRIM(C107))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C107))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C107))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E107&lt;&gt;"",E107,IF(UPPER(TRIM(C107))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C107))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C107))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C107))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G107" s="7" t="n"/>
@@ -5258,7 +5304,7 @@
       <c r="D108" s="7" t="n"/>
       <c r="E108" s="7" t="n"/>
       <c r="F108" s="8">
-        <f>IF(E108&lt;&gt;"",E108,IF(UPPER(TRIM(C108))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C108))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C108))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E108&lt;&gt;"",E108,IF(UPPER(TRIM(C108))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C108))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C108))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C108))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G108" s="7" t="n"/>
@@ -5280,7 +5326,7 @@
       <c r="D109" s="7" t="n"/>
       <c r="E109" s="7" t="n"/>
       <c r="F109" s="8">
-        <f>IF(E109&lt;&gt;"",E109,IF(UPPER(TRIM(C109))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C109))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C109))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E109&lt;&gt;"",E109,IF(UPPER(TRIM(C109))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C109))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C109))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C109))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G109" s="7" t="n"/>
@@ -5302,7 +5348,7 @@
       <c r="D110" s="7" t="n"/>
       <c r="E110" s="7" t="n"/>
       <c r="F110" s="8">
-        <f>IF(E110&lt;&gt;"",E110,IF(UPPER(TRIM(C110))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C110))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C110))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E110&lt;&gt;"",E110,IF(UPPER(TRIM(C110))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C110))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C110))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C110))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G110" s="7" t="n"/>
@@ -5324,7 +5370,7 @@
       <c r="D111" s="7" t="n"/>
       <c r="E111" s="7" t="n"/>
       <c r="F111" s="8">
-        <f>IF(E111&lt;&gt;"",E111,IF(UPPER(TRIM(C111))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C111))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C111))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E111&lt;&gt;"",E111,IF(UPPER(TRIM(C111))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C111))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C111))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C111))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G111" s="7" t="n"/>
@@ -5346,7 +5392,7 @@
       <c r="D112" s="7" t="n"/>
       <c r="E112" s="7" t="n"/>
       <c r="F112" s="8">
-        <f>IF(E112&lt;&gt;"",E112,IF(UPPER(TRIM(C112))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C112))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C112))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E112&lt;&gt;"",E112,IF(UPPER(TRIM(C112))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C112))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C112))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C112))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G112" s="7" t="n"/>
@@ -5368,7 +5414,7 @@
       <c r="D113" s="7" t="n"/>
       <c r="E113" s="7" t="n"/>
       <c r="F113" s="8">
-        <f>IF(E113&lt;&gt;"",E113,IF(UPPER(TRIM(C113))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C113))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C113))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E113&lt;&gt;"",E113,IF(UPPER(TRIM(C113))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C113))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C113))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C113))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G113" s="7" t="n"/>
@@ -5390,7 +5436,7 @@
       <c r="D114" s="7" t="n"/>
       <c r="E114" s="7" t="n"/>
       <c r="F114" s="8">
-        <f>IF(E114&lt;&gt;"",E114,IF(UPPER(TRIM(C114))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C114))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C114))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E114&lt;&gt;"",E114,IF(UPPER(TRIM(C114))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C114))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C114))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C114))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G114" s="7" t="n"/>
@@ -5412,7 +5458,7 @@
       <c r="D115" s="7" t="n"/>
       <c r="E115" s="7" t="n"/>
       <c r="F115" s="8">
-        <f>IF(E115&lt;&gt;"",E115,IF(UPPER(TRIM(C115))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C115))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C115))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E115&lt;&gt;"",E115,IF(UPPER(TRIM(C115))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C115))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C115))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C115))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G115" s="7" t="n"/>
@@ -5434,7 +5480,7 @@
       <c r="D116" s="7" t="n"/>
       <c r="E116" s="7" t="n"/>
       <c r="F116" s="8">
-        <f>IF(E116&lt;&gt;"",E116,IF(UPPER(TRIM(C116))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C116))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C116))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E116&lt;&gt;"",E116,IF(UPPER(TRIM(C116))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C116))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C116))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C116))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G116" s="7" t="n"/>
@@ -5456,7 +5502,7 @@
       <c r="D117" s="7" t="n"/>
       <c r="E117" s="7" t="n"/>
       <c r="F117" s="8">
-        <f>IF(E117&lt;&gt;"",E117,IF(UPPER(TRIM(C117))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C117))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C117))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E117&lt;&gt;"",E117,IF(UPPER(TRIM(C117))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C117))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C117))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C117))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G117" s="7" t="n"/>
@@ -5478,7 +5524,7 @@
       <c r="D118" s="7" t="n"/>
       <c r="E118" s="7" t="n"/>
       <c r="F118" s="8">
-        <f>IF(E118&lt;&gt;"",E118,IF(UPPER(TRIM(C118))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C118))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C118))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E118&lt;&gt;"",E118,IF(UPPER(TRIM(C118))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C118))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C118))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C118))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G118" s="7" t="n"/>
@@ -5500,7 +5546,7 @@
       <c r="D119" s="7" t="n"/>
       <c r="E119" s="7" t="n"/>
       <c r="F119" s="8">
-        <f>IF(E119&lt;&gt;"",E119,IF(UPPER(TRIM(C119))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C119))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C119))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E119&lt;&gt;"",E119,IF(UPPER(TRIM(C119))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C119))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C119))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C119))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G119" s="7" t="n"/>
@@ -5522,7 +5568,7 @@
       <c r="D120" s="7" t="n"/>
       <c r="E120" s="7" t="n"/>
       <c r="F120" s="8">
-        <f>IF(E120&lt;&gt;"",E120,IF(UPPER(TRIM(C120))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C120))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C120))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E120&lt;&gt;"",E120,IF(UPPER(TRIM(C120))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C120))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C120))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C120))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G120" s="7" t="n"/>
@@ -5544,7 +5590,7 @@
       <c r="D121" s="7" t="n"/>
       <c r="E121" s="7" t="n"/>
       <c r="F121" s="8">
-        <f>IF(E121&lt;&gt;"",E121,IF(UPPER(TRIM(C121))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C121))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C121))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E121&lt;&gt;"",E121,IF(UPPER(TRIM(C121))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C121))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C121))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C121))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G121" s="7" t="n"/>
@@ -5566,7 +5612,7 @@
       <c r="D122" s="7" t="n"/>
       <c r="E122" s="7" t="n"/>
       <c r="F122" s="8">
-        <f>IF(E122&lt;&gt;"",E122,IF(UPPER(TRIM(C122))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C122))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C122))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E122&lt;&gt;"",E122,IF(UPPER(TRIM(C122))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C122))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C122))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C122))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G122" s="7" t="n"/>
@@ -5588,7 +5634,7 @@
       <c r="D123" s="7" t="n"/>
       <c r="E123" s="7" t="n"/>
       <c r="F123" s="8">
-        <f>IF(E123&lt;&gt;"",E123,IF(UPPER(TRIM(C123))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C123))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C123))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E123&lt;&gt;"",E123,IF(UPPER(TRIM(C123))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C123))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C123))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C123))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G123" s="7" t="n"/>
@@ -5610,7 +5656,7 @@
       <c r="D124" s="7" t="n"/>
       <c r="E124" s="7" t="n"/>
       <c r="F124" s="8">
-        <f>IF(E124&lt;&gt;"",E124,IF(UPPER(TRIM(C124))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C124))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C124))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E124&lt;&gt;"",E124,IF(UPPER(TRIM(C124))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C124))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C124))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C124))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G124" s="7" t="n"/>
@@ -5632,7 +5678,7 @@
       <c r="D125" s="7" t="n"/>
       <c r="E125" s="7" t="n"/>
       <c r="F125" s="8">
-        <f>IF(E125&lt;&gt;"",E125,IF(UPPER(TRIM(C125))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C125))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C125))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E125&lt;&gt;"",E125,IF(UPPER(TRIM(C125))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C125))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C125))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C125))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G125" s="7" t="n"/>
@@ -5654,7 +5700,7 @@
       <c r="D126" s="7" t="n"/>
       <c r="E126" s="7" t="n"/>
       <c r="F126" s="8">
-        <f>IF(E126&lt;&gt;"",E126,IF(UPPER(TRIM(C126))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C126))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C126))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E126&lt;&gt;"",E126,IF(UPPER(TRIM(C126))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C126))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C126))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C126))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G126" s="7" t="n"/>
@@ -5676,7 +5722,7 @@
       <c r="D127" s="7" t="n"/>
       <c r="E127" s="7" t="n"/>
       <c r="F127" s="8">
-        <f>IF(E127&lt;&gt;"",E127,IF(UPPER(TRIM(C127))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C127))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C127))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E127&lt;&gt;"",E127,IF(UPPER(TRIM(C127))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C127))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C127))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C127))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G127" s="7" t="n"/>
@@ -5698,7 +5744,7 @@
       <c r="D128" s="7" t="n"/>
       <c r="E128" s="7" t="n"/>
       <c r="F128" s="8">
-        <f>IF(E128&lt;&gt;"",E128,IF(UPPER(TRIM(C128))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C128))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C128))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E128&lt;&gt;"",E128,IF(UPPER(TRIM(C128))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C128))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C128))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C128))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G128" s="7" t="n"/>
@@ -5720,7 +5766,7 @@
       <c r="D129" s="7" t="n"/>
       <c r="E129" s="7" t="n"/>
       <c r="F129" s="8">
-        <f>IF(E129&lt;&gt;"",E129,IF(UPPER(TRIM(C129))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C129))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C129))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E129&lt;&gt;"",E129,IF(UPPER(TRIM(C129))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C129))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C129))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C129))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G129" s="7" t="n"/>
@@ -5742,7 +5788,7 @@
       <c r="D130" s="7" t="n"/>
       <c r="E130" s="7" t="n"/>
       <c r="F130" s="8">
-        <f>IF(E130&lt;&gt;"",E130,IF(UPPER(TRIM(C130))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C130))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C130))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E130&lt;&gt;"",E130,IF(UPPER(TRIM(C130))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C130))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C130))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C130))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G130" s="7" t="n"/>
@@ -5764,7 +5810,7 @@
       <c r="D131" s="7" t="n"/>
       <c r="E131" s="7" t="n"/>
       <c r="F131" s="8">
-        <f>IF(E131&lt;&gt;"",E131,IF(UPPER(TRIM(C131))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C131))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C131))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E131&lt;&gt;"",E131,IF(UPPER(TRIM(C131))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C131))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C131))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C131))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G131" s="7" t="n"/>
@@ -5786,7 +5832,7 @@
       <c r="D132" s="7" t="n"/>
       <c r="E132" s="7" t="n"/>
       <c r="F132" s="8">
-        <f>IF(E132&lt;&gt;"",E132,IF(UPPER(TRIM(C132))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C132))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C132))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E132&lt;&gt;"",E132,IF(UPPER(TRIM(C132))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C132))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C132))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C132))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G132" s="7" t="n"/>
@@ -5808,7 +5854,7 @@
       <c r="D133" s="7" t="n"/>
       <c r="E133" s="7" t="n"/>
       <c r="F133" s="8">
-        <f>IF(E133&lt;&gt;"",E133,IF(UPPER(TRIM(C133))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C133))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C133))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E133&lt;&gt;"",E133,IF(UPPER(TRIM(C133))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C133))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C133))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C133))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G133" s="7" t="n"/>
@@ -5830,7 +5876,7 @@
       <c r="D134" s="7" t="n"/>
       <c r="E134" s="7" t="n"/>
       <c r="F134" s="8">
-        <f>IF(E134&lt;&gt;"",E134,IF(UPPER(TRIM(C134))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C134))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C134))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E134&lt;&gt;"",E134,IF(UPPER(TRIM(C134))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C134))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C134))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C134))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G134" s="7" t="n"/>
@@ -5852,7 +5898,7 @@
       <c r="D135" s="7" t="n"/>
       <c r="E135" s="7" t="n"/>
       <c r="F135" s="8">
-        <f>IF(E135&lt;&gt;"",E135,IF(UPPER(TRIM(C135))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C135))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C135))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E135&lt;&gt;"",E135,IF(UPPER(TRIM(C135))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C135))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C135))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C135))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G135" s="7" t="n"/>
@@ -5874,7 +5920,7 @@
       <c r="D136" s="7" t="n"/>
       <c r="E136" s="7" t="n"/>
       <c r="F136" s="8">
-        <f>IF(E136&lt;&gt;"",E136,IF(UPPER(TRIM(C136))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C136))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C136))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E136&lt;&gt;"",E136,IF(UPPER(TRIM(C136))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C136))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C136))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C136))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G136" s="7" t="n"/>
@@ -5896,7 +5942,7 @@
       <c r="D137" s="7" t="n"/>
       <c r="E137" s="7" t="n"/>
       <c r="F137" s="8">
-        <f>IF(E137&lt;&gt;"",E137,IF(UPPER(TRIM(C137))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C137))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C137))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E137&lt;&gt;"",E137,IF(UPPER(TRIM(C137))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C137))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C137))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C137))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G137" s="7" t="n"/>
@@ -5918,7 +5964,7 @@
       <c r="D138" s="7" t="n"/>
       <c r="E138" s="7" t="n"/>
       <c r="F138" s="8">
-        <f>IF(E138&lt;&gt;"",E138,IF(UPPER(TRIM(C138))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C138))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C138))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E138&lt;&gt;"",E138,IF(UPPER(TRIM(C138))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C138))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C138))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C138))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G138" s="7" t="n"/>
@@ -5940,7 +5986,7 @@
       <c r="D139" s="7" t="n"/>
       <c r="E139" s="7" t="n"/>
       <c r="F139" s="8">
-        <f>IF(E139&lt;&gt;"",E139,IF(UPPER(TRIM(C139))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C139))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C139))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E139&lt;&gt;"",E139,IF(UPPER(TRIM(C139))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C139))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C139))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C139))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G139" s="7" t="n"/>
@@ -5962,7 +6008,7 @@
       <c r="D140" s="7" t="n"/>
       <c r="E140" s="7" t="n"/>
       <c r="F140" s="8">
-        <f>IF(E140&lt;&gt;"",E140,IF(UPPER(TRIM(C140))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C140))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C140))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E140&lt;&gt;"",E140,IF(UPPER(TRIM(C140))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C140))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C140))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C140))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G140" s="7" t="n"/>
@@ -5984,7 +6030,7 @@
       <c r="D141" s="7" t="n"/>
       <c r="E141" s="7" t="n"/>
       <c r="F141" s="8">
-        <f>IF(E141&lt;&gt;"",E141,IF(UPPER(TRIM(C141))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C141))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C141))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E141&lt;&gt;"",E141,IF(UPPER(TRIM(C141))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C141))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C141))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C141))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G141" s="7" t="n"/>
@@ -6006,7 +6052,7 @@
       <c r="D142" s="7" t="n"/>
       <c r="E142" s="7" t="n"/>
       <c r="F142" s="8">
-        <f>IF(E142&lt;&gt;"",E142,IF(UPPER(TRIM(C142))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C142))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C142))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E142&lt;&gt;"",E142,IF(UPPER(TRIM(C142))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C142))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C142))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C142))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G142" s="7" t="n"/>
@@ -6028,7 +6074,7 @@
       <c r="D143" s="7" t="n"/>
       <c r="E143" s="7" t="n"/>
       <c r="F143" s="8">
-        <f>IF(E143&lt;&gt;"",E143,IF(UPPER(TRIM(C143))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C143))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C143))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E143&lt;&gt;"",E143,IF(UPPER(TRIM(C143))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C143))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C143))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C143))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G143" s="7" t="n"/>
@@ -6050,7 +6096,7 @@
       <c r="D144" s="7" t="n"/>
       <c r="E144" s="7" t="n"/>
       <c r="F144" s="8">
-        <f>IF(E144&lt;&gt;"",E144,IF(UPPER(TRIM(C144))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C144))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C144))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E144&lt;&gt;"",E144,IF(UPPER(TRIM(C144))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C144))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C144))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C144))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G144" s="7" t="n"/>
@@ -6072,7 +6118,7 @@
       <c r="D145" s="7" t="n"/>
       <c r="E145" s="7" t="n"/>
       <c r="F145" s="8">
-        <f>IF(E145&lt;&gt;"",E145,IF(UPPER(TRIM(C145))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C145))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C145))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E145&lt;&gt;"",E145,IF(UPPER(TRIM(C145))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C145))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C145))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C145))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G145" s="7" t="n"/>
@@ -6094,7 +6140,7 @@
       <c r="D146" s="7" t="n"/>
       <c r="E146" s="7" t="n"/>
       <c r="F146" s="8">
-        <f>IF(E146&lt;&gt;"",E146,IF(UPPER(TRIM(C146))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C146))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C146))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E146&lt;&gt;"",E146,IF(UPPER(TRIM(C146))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C146))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C146))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C146))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G146" s="7" t="n"/>
@@ -6116,7 +6162,7 @@
       <c r="D147" s="7" t="n"/>
       <c r="E147" s="7" t="n"/>
       <c r="F147" s="8">
-        <f>IF(E147&lt;&gt;"",E147,IF(UPPER(TRIM(C147))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C147))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C147))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E147&lt;&gt;"",E147,IF(UPPER(TRIM(C147))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C147))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C147))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C147))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G147" s="7" t="n"/>
@@ -6138,7 +6184,7 @@
       <c r="D148" s="7" t="n"/>
       <c r="E148" s="7" t="n"/>
       <c r="F148" s="8">
-        <f>IF(E148&lt;&gt;"",E148,IF(UPPER(TRIM(C148))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C148))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C148))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E148&lt;&gt;"",E148,IF(UPPER(TRIM(C148))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C148))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C148))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C148))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G148" s="7" t="n"/>
@@ -6160,7 +6206,7 @@
       <c r="D149" s="7" t="n"/>
       <c r="E149" s="7" t="n"/>
       <c r="F149" s="8">
-        <f>IF(E149&lt;&gt;"",E149,IF(UPPER(TRIM(C149))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C149))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C149))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E149&lt;&gt;"",E149,IF(UPPER(TRIM(C149))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C149))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C149))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C149))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G149" s="7" t="n"/>
@@ -6182,7 +6228,7 @@
       <c r="D150" s="7" t="n"/>
       <c r="E150" s="7" t="n"/>
       <c r="F150" s="8">
-        <f>IF(E150&lt;&gt;"",E150,IF(UPPER(TRIM(C150))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C150))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C150))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E150&lt;&gt;"",E150,IF(UPPER(TRIM(C150))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C150))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C150))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C150))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G150" s="7" t="n"/>
@@ -6204,7 +6250,7 @@
       <c r="D151" s="7" t="n"/>
       <c r="E151" s="7" t="n"/>
       <c r="F151" s="8">
-        <f>IF(E151&lt;&gt;"",E151,IF(UPPER(TRIM(C151))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C151))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C151))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E151&lt;&gt;"",E151,IF(UPPER(TRIM(C151))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C151))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C151))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C151))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G151" s="7" t="n"/>
@@ -6226,7 +6272,7 @@
       <c r="D152" s="7" t="n"/>
       <c r="E152" s="7" t="n"/>
       <c r="F152" s="8">
-        <f>IF(E152&lt;&gt;"",E152,IF(UPPER(TRIM(C152))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C152))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C152))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E152&lt;&gt;"",E152,IF(UPPER(TRIM(C152))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C152))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C152))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C152))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G152" s="7" t="n"/>
@@ -6248,7 +6294,7 @@
       <c r="D153" s="7" t="n"/>
       <c r="E153" s="7" t="n"/>
       <c r="F153" s="8">
-        <f>IF(E153&lt;&gt;"",E153,IF(UPPER(TRIM(C153))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C153))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C153))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E153&lt;&gt;"",E153,IF(UPPER(TRIM(C153))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C153))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C153))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C153))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G153" s="7" t="n"/>
@@ -6270,7 +6316,7 @@
       <c r="D154" s="7" t="n"/>
       <c r="E154" s="7" t="n"/>
       <c r="F154" s="8">
-        <f>IF(E154&lt;&gt;"",E154,IF(UPPER(TRIM(C154))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C154))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C154))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E154&lt;&gt;"",E154,IF(UPPER(TRIM(C154))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C154))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C154))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C154))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G154" s="7" t="n"/>
@@ -6292,7 +6338,7 @@
       <c r="D155" s="7" t="n"/>
       <c r="E155" s="7" t="n"/>
       <c r="F155" s="8">
-        <f>IF(E155&lt;&gt;"",E155,IF(UPPER(TRIM(C155))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C155))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C155))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E155&lt;&gt;"",E155,IF(UPPER(TRIM(C155))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C155))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C155))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C155))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G155" s="7" t="n"/>
@@ -6314,7 +6360,7 @@
       <c r="D156" s="7" t="n"/>
       <c r="E156" s="7" t="n"/>
       <c r="F156" s="8">
-        <f>IF(E156&lt;&gt;"",E156,IF(UPPER(TRIM(C156))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C156))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C156))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E156&lt;&gt;"",E156,IF(UPPER(TRIM(C156))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C156))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C156))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C156))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G156" s="7" t="n"/>
@@ -6336,7 +6382,7 @@
       <c r="D157" s="7" t="n"/>
       <c r="E157" s="7" t="n"/>
       <c r="F157" s="8">
-        <f>IF(E157&lt;&gt;"",E157,IF(UPPER(TRIM(C157))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C157))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C157))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E157&lt;&gt;"",E157,IF(UPPER(TRIM(C157))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C157))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C157))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C157))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G157" s="7" t="n"/>
@@ -6358,7 +6404,7 @@
       <c r="D158" s="7" t="n"/>
       <c r="E158" s="7" t="n"/>
       <c r="F158" s="8">
-        <f>IF(E158&lt;&gt;"",E158,IF(UPPER(TRIM(C158))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C158))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C158))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E158&lt;&gt;"",E158,IF(UPPER(TRIM(C158))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C158))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C158))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C158))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G158" s="7" t="n"/>
@@ -6380,7 +6426,7 @@
       <c r="D159" s="7" t="n"/>
       <c r="E159" s="7" t="n"/>
       <c r="F159" s="8">
-        <f>IF(E159&lt;&gt;"",E159,IF(UPPER(TRIM(C159))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C159))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C159))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E159&lt;&gt;"",E159,IF(UPPER(TRIM(C159))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C159))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C159))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C159))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G159" s="7" t="n"/>
@@ -6402,7 +6448,7 @@
       <c r="D160" s="7" t="n"/>
       <c r="E160" s="7" t="n"/>
       <c r="F160" s="8">
-        <f>IF(E160&lt;&gt;"",E160,IF(UPPER(TRIM(C160))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C160))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C160))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E160&lt;&gt;"",E160,IF(UPPER(TRIM(C160))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C160))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C160))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C160))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G160" s="7" t="n"/>
@@ -6424,7 +6470,7 @@
       <c r="D161" s="7" t="n"/>
       <c r="E161" s="7" t="n"/>
       <c r="F161" s="8">
-        <f>IF(E161&lt;&gt;"",E161,IF(UPPER(TRIM(C161))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C161))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C161))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E161&lt;&gt;"",E161,IF(UPPER(TRIM(C161))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C161))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C161))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C161))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G161" s="7" t="n"/>
@@ -6446,7 +6492,7 @@
       <c r="D162" s="7" t="n"/>
       <c r="E162" s="7" t="n"/>
       <c r="F162" s="8">
-        <f>IF(E162&lt;&gt;"",E162,IF(UPPER(TRIM(C162))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C162))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C162))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E162&lt;&gt;"",E162,IF(UPPER(TRIM(C162))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C162))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C162))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C162))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G162" s="7" t="n"/>
@@ -6468,7 +6514,7 @@
       <c r="D163" s="7" t="n"/>
       <c r="E163" s="7" t="n"/>
       <c r="F163" s="8">
-        <f>IF(E163&lt;&gt;"",E163,IF(UPPER(TRIM(C163))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C163))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C163))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E163&lt;&gt;"",E163,IF(UPPER(TRIM(C163))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C163))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C163))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C163))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G163" s="7" t="n"/>
@@ -6490,7 +6536,7 @@
       <c r="D164" s="7" t="n"/>
       <c r="E164" s="7" t="n"/>
       <c r="F164" s="8">
-        <f>IF(E164&lt;&gt;"",E164,IF(UPPER(TRIM(C164))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C164))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C164))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E164&lt;&gt;"",E164,IF(UPPER(TRIM(C164))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C164))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C164))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C164))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G164" s="7" t="n"/>
@@ -6512,7 +6558,7 @@
       <c r="D165" s="7" t="n"/>
       <c r="E165" s="7" t="n"/>
       <c r="F165" s="8">
-        <f>IF(E165&lt;&gt;"",E165,IF(UPPER(TRIM(C165))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C165))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C165))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E165&lt;&gt;"",E165,IF(UPPER(TRIM(C165))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C165))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C165))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C165))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G165" s="7" t="n"/>
@@ -6534,7 +6580,7 @@
       <c r="D166" s="7" t="n"/>
       <c r="E166" s="7" t="n"/>
       <c r="F166" s="8">
-        <f>IF(E166&lt;&gt;"",E166,IF(UPPER(TRIM(C166))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C166))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C166))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E166&lt;&gt;"",E166,IF(UPPER(TRIM(C166))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C166))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C166))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C166))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G166" s="7" t="n"/>
@@ -6556,7 +6602,7 @@
       <c r="D167" s="7" t="n"/>
       <c r="E167" s="7" t="n"/>
       <c r="F167" s="8">
-        <f>IF(E167&lt;&gt;"",E167,IF(UPPER(TRIM(C167))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C167))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C167))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E167&lt;&gt;"",E167,IF(UPPER(TRIM(C167))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C167))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C167))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C167))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G167" s="7" t="n"/>
@@ -6578,7 +6624,7 @@
       <c r="D168" s="7" t="n"/>
       <c r="E168" s="7" t="n"/>
       <c r="F168" s="8">
-        <f>IF(E168&lt;&gt;"",E168,IF(UPPER(TRIM(C168))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C168))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C168))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E168&lt;&gt;"",E168,IF(UPPER(TRIM(C168))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C168))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C168))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C168))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G168" s="7" t="n"/>
@@ -6600,7 +6646,7 @@
       <c r="D169" s="7" t="n"/>
       <c r="E169" s="7" t="n"/>
       <c r="F169" s="8">
-        <f>IF(E169&lt;&gt;"",E169,IF(UPPER(TRIM(C169))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C169))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C169))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E169&lt;&gt;"",E169,IF(UPPER(TRIM(C169))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C169))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C169))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C169))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G169" s="7" t="n"/>
@@ -6622,7 +6668,7 @@
       <c r="D170" s="7" t="n"/>
       <c r="E170" s="7" t="n"/>
       <c r="F170" s="8">
-        <f>IF(E170&lt;&gt;"",E170,IF(UPPER(TRIM(C170))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C170))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C170))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E170&lt;&gt;"",E170,IF(UPPER(TRIM(C170))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C170))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C170))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C170))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G170" s="7" t="n"/>
@@ -6644,7 +6690,7 @@
       <c r="D171" s="7" t="n"/>
       <c r="E171" s="7" t="n"/>
       <c r="F171" s="8">
-        <f>IF(E171&lt;&gt;"",E171,IF(UPPER(TRIM(C171))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C171))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C171))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E171&lt;&gt;"",E171,IF(UPPER(TRIM(C171))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C171))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C171))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C171))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G171" s="7" t="n"/>
@@ -6666,7 +6712,7 @@
       <c r="D172" s="7" t="n"/>
       <c r="E172" s="7" t="n"/>
       <c r="F172" s="8">
-        <f>IF(E172&lt;&gt;"",E172,IF(UPPER(TRIM(C172))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C172))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C172))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E172&lt;&gt;"",E172,IF(UPPER(TRIM(C172))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C172))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C172))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C172))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G172" s="7" t="n"/>
@@ -6688,7 +6734,7 @@
       <c r="D173" s="7" t="n"/>
       <c r="E173" s="7" t="n"/>
       <c r="F173" s="8">
-        <f>IF(E173&lt;&gt;"",E173,IF(UPPER(TRIM(C173))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C173))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C173))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E173&lt;&gt;"",E173,IF(UPPER(TRIM(C173))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C173))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C173))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C173))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G173" s="7" t="n"/>
@@ -6710,7 +6756,7 @@
       <c r="D174" s="7" t="n"/>
       <c r="E174" s="7" t="n"/>
       <c r="F174" s="8">
-        <f>IF(E174&lt;&gt;"",E174,IF(UPPER(TRIM(C174))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C174))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C174))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E174&lt;&gt;"",E174,IF(UPPER(TRIM(C174))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C174))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C174))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C174))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G174" s="7" t="n"/>
@@ -6732,7 +6778,7 @@
       <c r="D175" s="7" t="n"/>
       <c r="E175" s="7" t="n"/>
       <c r="F175" s="8">
-        <f>IF(E175&lt;&gt;"",E175,IF(UPPER(TRIM(C175))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C175))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C175))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E175&lt;&gt;"",E175,IF(UPPER(TRIM(C175))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C175))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C175))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C175))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G175" s="7" t="n"/>
@@ -6754,7 +6800,7 @@
       <c r="D176" s="7" t="n"/>
       <c r="E176" s="7" t="n"/>
       <c r="F176" s="8">
-        <f>IF(E176&lt;&gt;"",E176,IF(UPPER(TRIM(C176))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C176))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C176))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E176&lt;&gt;"",E176,IF(UPPER(TRIM(C176))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C176))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C176))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C176))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G176" s="7" t="n"/>
@@ -6776,7 +6822,7 @@
       <c r="D177" s="7" t="n"/>
       <c r="E177" s="7" t="n"/>
       <c r="F177" s="8">
-        <f>IF(E177&lt;&gt;"",E177,IF(UPPER(TRIM(C177))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C177))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C177))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E177&lt;&gt;"",E177,IF(UPPER(TRIM(C177))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C177))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C177))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C177))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G177" s="7" t="n"/>
@@ -6798,7 +6844,7 @@
       <c r="D178" s="7" t="n"/>
       <c r="E178" s="7" t="n"/>
       <c r="F178" s="8">
-        <f>IF(E178&lt;&gt;"",E178,IF(UPPER(TRIM(C178))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C178))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C178))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E178&lt;&gt;"",E178,IF(UPPER(TRIM(C178))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C178))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C178))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C178))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G178" s="7" t="n"/>
@@ -6820,7 +6866,7 @@
       <c r="D179" s="7" t="n"/>
       <c r="E179" s="7" t="n"/>
       <c r="F179" s="8">
-        <f>IF(E179&lt;&gt;"",E179,IF(UPPER(TRIM(C179))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C179))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C179))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E179&lt;&gt;"",E179,IF(UPPER(TRIM(C179))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C179))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C179))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C179))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G179" s="7" t="n"/>
@@ -6842,7 +6888,7 @@
       <c r="D180" s="7" t="n"/>
       <c r="E180" s="7" t="n"/>
       <c r="F180" s="8">
-        <f>IF(E180&lt;&gt;"",E180,IF(UPPER(TRIM(C180))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C180))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C180))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E180&lt;&gt;"",E180,IF(UPPER(TRIM(C180))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C180))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C180))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C180))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G180" s="7" t="n"/>
@@ -6864,7 +6910,7 @@
       <c r="D181" s="7" t="n"/>
       <c r="E181" s="7" t="n"/>
       <c r="F181" s="8">
-        <f>IF(E181&lt;&gt;"",E181,IF(UPPER(TRIM(C181))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C181))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C181))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E181&lt;&gt;"",E181,IF(UPPER(TRIM(C181))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C181))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C181))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C181))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G181" s="7" t="n"/>
@@ -6886,7 +6932,7 @@
       <c r="D182" s="7" t="n"/>
       <c r="E182" s="7" t="n"/>
       <c r="F182" s="8">
-        <f>IF(E182&lt;&gt;"",E182,IF(UPPER(TRIM(C182))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C182))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C182))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E182&lt;&gt;"",E182,IF(UPPER(TRIM(C182))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C182))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C182))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C182))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G182" s="7" t="n"/>
@@ -6908,7 +6954,7 @@
       <c r="D183" s="7" t="n"/>
       <c r="E183" s="7" t="n"/>
       <c r="F183" s="8">
-        <f>IF(E183&lt;&gt;"",E183,IF(UPPER(TRIM(C183))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C183))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C183))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E183&lt;&gt;"",E183,IF(UPPER(TRIM(C183))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C183))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C183))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C183))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G183" s="7" t="n"/>
@@ -6930,7 +6976,7 @@
       <c r="D184" s="7" t="n"/>
       <c r="E184" s="7" t="n"/>
       <c r="F184" s="8">
-        <f>IF(E184&lt;&gt;"",E184,IF(UPPER(TRIM(C184))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C184))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C184))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E184&lt;&gt;"",E184,IF(UPPER(TRIM(C184))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C184))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C184))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C184))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G184" s="7" t="n"/>
@@ -6952,7 +6998,7 @@
       <c r="D185" s="7" t="n"/>
       <c r="E185" s="7" t="n"/>
       <c r="F185" s="8">
-        <f>IF(E185&lt;&gt;"",E185,IF(UPPER(TRIM(C185))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C185))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C185))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E185&lt;&gt;"",E185,IF(UPPER(TRIM(C185))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C185))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C185))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C185))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G185" s="7" t="n"/>
@@ -6974,7 +7020,7 @@
       <c r="D186" s="7" t="n"/>
       <c r="E186" s="7" t="n"/>
       <c r="F186" s="8">
-        <f>IF(E186&lt;&gt;"",E186,IF(UPPER(TRIM(C186))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C186))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C186))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E186&lt;&gt;"",E186,IF(UPPER(TRIM(C186))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C186))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C186))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C186))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G186" s="7" t="n"/>
@@ -6996,7 +7042,7 @@
       <c r="D187" s="7" t="n"/>
       <c r="E187" s="7" t="n"/>
       <c r="F187" s="8">
-        <f>IF(E187&lt;&gt;"",E187,IF(UPPER(TRIM(C187))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C187))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C187))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E187&lt;&gt;"",E187,IF(UPPER(TRIM(C187))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C187))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C187))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C187))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G187" s="7" t="n"/>
@@ -7018,7 +7064,7 @@
       <c r="D188" s="7" t="n"/>
       <c r="E188" s="7" t="n"/>
       <c r="F188" s="8">
-        <f>IF(E188&lt;&gt;"",E188,IF(UPPER(TRIM(C188))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C188))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C188))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E188&lt;&gt;"",E188,IF(UPPER(TRIM(C188))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C188))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C188))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C188))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G188" s="7" t="n"/>
@@ -7040,7 +7086,7 @@
       <c r="D189" s="7" t="n"/>
       <c r="E189" s="7" t="n"/>
       <c r="F189" s="8">
-        <f>IF(E189&lt;&gt;"",E189,IF(UPPER(TRIM(C189))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C189))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C189))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E189&lt;&gt;"",E189,IF(UPPER(TRIM(C189))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C189))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C189))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C189))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G189" s="7" t="n"/>
@@ -7062,7 +7108,7 @@
       <c r="D190" s="7" t="n"/>
       <c r="E190" s="7" t="n"/>
       <c r="F190" s="8">
-        <f>IF(E190&lt;&gt;"",E190,IF(UPPER(TRIM(C190))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C190))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C190))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E190&lt;&gt;"",E190,IF(UPPER(TRIM(C190))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C190))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C190))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C190))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G190" s="7" t="n"/>
@@ -7084,7 +7130,7 @@
       <c r="D191" s="7" t="n"/>
       <c r="E191" s="7" t="n"/>
       <c r="F191" s="8">
-        <f>IF(E191&lt;&gt;"",E191,IF(UPPER(TRIM(C191))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C191))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C191))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E191&lt;&gt;"",E191,IF(UPPER(TRIM(C191))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C191))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C191))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C191))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G191" s="7" t="n"/>
@@ -7106,7 +7152,7 @@
       <c r="D192" s="7" t="n"/>
       <c r="E192" s="7" t="n"/>
       <c r="F192" s="8">
-        <f>IF(E192&lt;&gt;"",E192,IF(UPPER(TRIM(C192))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C192))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C192))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E192&lt;&gt;"",E192,IF(UPPER(TRIM(C192))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C192))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C192))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C192))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G192" s="7" t="n"/>
@@ -7128,7 +7174,7 @@
       <c r="D193" s="7" t="n"/>
       <c r="E193" s="7" t="n"/>
       <c r="F193" s="8">
-        <f>IF(E193&lt;&gt;"",E193,IF(UPPER(TRIM(C193))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C193))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C193))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E193&lt;&gt;"",E193,IF(UPPER(TRIM(C193))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C193))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C193))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C193))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G193" s="7" t="n"/>
@@ -7150,7 +7196,7 @@
       <c r="D194" s="7" t="n"/>
       <c r="E194" s="7" t="n"/>
       <c r="F194" s="8">
-        <f>IF(E194&lt;&gt;"",E194,IF(UPPER(TRIM(C194))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C194))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C194))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E194&lt;&gt;"",E194,IF(UPPER(TRIM(C194))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C194))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C194))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C194))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G194" s="7" t="n"/>
@@ -7172,7 +7218,7 @@
       <c r="D195" s="7" t="n"/>
       <c r="E195" s="7" t="n"/>
       <c r="F195" s="8">
-        <f>IF(E195&lt;&gt;"",E195,IF(UPPER(TRIM(C195))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C195))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C195))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E195&lt;&gt;"",E195,IF(UPPER(TRIM(C195))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C195))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C195))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C195))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G195" s="7" t="n"/>
@@ -7194,7 +7240,7 @@
       <c r="D196" s="7" t="n"/>
       <c r="E196" s="7" t="n"/>
       <c r="F196" s="8">
-        <f>IF(E196&lt;&gt;"",E196,IF(UPPER(TRIM(C196))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C196))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C196))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E196&lt;&gt;"",E196,IF(UPPER(TRIM(C196))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C196))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C196))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C196))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G196" s="7" t="n"/>
@@ -7216,7 +7262,7 @@
       <c r="D197" s="7" t="n"/>
       <c r="E197" s="7" t="n"/>
       <c r="F197" s="8">
-        <f>IF(E197&lt;&gt;"",E197,IF(UPPER(TRIM(C197))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C197))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C197))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E197&lt;&gt;"",E197,IF(UPPER(TRIM(C197))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C197))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C197))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C197))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G197" s="7" t="n"/>
@@ -7238,7 +7284,7 @@
       <c r="D198" s="7" t="n"/>
       <c r="E198" s="7" t="n"/>
       <c r="F198" s="8">
-        <f>IF(E198&lt;&gt;"",E198,IF(UPPER(TRIM(C198))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C198))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C198))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E198&lt;&gt;"",E198,IF(UPPER(TRIM(C198))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C198))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C198))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C198))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G198" s="7" t="n"/>
@@ -7260,7 +7306,7 @@
       <c r="D199" s="7" t="n"/>
       <c r="E199" s="7" t="n"/>
       <c r="F199" s="8">
-        <f>IF(E199&lt;&gt;"",E199,IF(UPPER(TRIM(C199))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C199))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C199))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E199&lt;&gt;"",E199,IF(UPPER(TRIM(C199))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C199))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C199))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C199))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G199" s="7" t="n"/>
@@ -7282,7 +7328,7 @@
       <c r="D200" s="7" t="n"/>
       <c r="E200" s="7" t="n"/>
       <c r="F200" s="8">
-        <f>IF(E200&lt;&gt;"",E200,IF(UPPER(TRIM(C200))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C200))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C200))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E200&lt;&gt;"",E200,IF(UPPER(TRIM(C200))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C200))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C200))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C200))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G200" s="7" t="n"/>
@@ -7304,7 +7350,7 @@
       <c r="D201" s="7" t="n"/>
       <c r="E201" s="7" t="n"/>
       <c r="F201" s="8">
-        <f>IF(E201&lt;&gt;"",E201,IF(UPPER(TRIM(C201))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C201))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C201))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E201&lt;&gt;"",E201,IF(UPPER(TRIM(C201))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C201))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C201))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C201))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G201" s="7" t="n"/>
@@ -7326,7 +7372,7 @@
       <c r="D202" s="7" t="n"/>
       <c r="E202" s="7" t="n"/>
       <c r="F202" s="8">
-        <f>IF(E202&lt;&gt;"",E202,IF(UPPER(TRIM(C202))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C202))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C202))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E202&lt;&gt;"",E202,IF(UPPER(TRIM(C202))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C202))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C202))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C202))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G202" s="7" t="n"/>
@@ -7348,7 +7394,7 @@
       <c r="D203" s="7" t="n"/>
       <c r="E203" s="7" t="n"/>
       <c r="F203" s="8">
-        <f>IF(E203&lt;&gt;"",E203,IF(UPPER(TRIM(C203))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C203))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C203))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E203&lt;&gt;"",E203,IF(UPPER(TRIM(C203))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C203))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C203))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C203))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G203" s="7" t="n"/>
@@ -7370,7 +7416,7 @@
       <c r="D204" s="7" t="n"/>
       <c r="E204" s="7" t="n"/>
       <c r="F204" s="8">
-        <f>IF(E204&lt;&gt;"",E204,IF(UPPER(TRIM(C204))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C204))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C204))="GRASS",Inputs!$B$12,Inputs!$B$13))))</f>
+        <f>IF(E204&lt;&gt;"",E204,IF(UPPER(TRIM(C204))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C204))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C204))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C204))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
         <v/>
       </c>
       <c r="G204" s="7" t="n"/>
@@ -7923,7 +7969,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>20</v>
+        <v>16.1</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>0.006</v>
@@ -7996,7 +8042,7 @@
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>Collecteur est vers entree bassin.</t>
+          <t>Corrige: P-03 -&gt; J-BASSIN-IN = 16.1 m (pas 20 m).</t>
         </is>
       </c>
       <c r="AC6" s="7" t="n"/>
@@ -8034,12 +8080,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>J-SUD-EST</t>
+          <t>J-OUEST-AVAL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>J-SUD-OUEST</t>
+          <t>J-BASSIN-IN</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -8048,10 +8094,10 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>16.1</v>
+        <v>20</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="H7" s="7" t="inlineStr"/>
       <c r="I7" s="8">
@@ -8060,19 +8106,22 @@
       </c>
       <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7">
-        <f>Inputs!$B$25</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="L7" s="7">
-        <f>Inputs!$B$26</f>
-        <v/>
-      </c>
-      <c r="M7" s="7">
-        <f>Inputs!$B$20</f>
-        <v/>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>0</v>
+        <f>Inputs!$B$36</f>
+        <v/>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O7" s="8">
         <f>IF(A7="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A7))</f>
@@ -8128,7 +8177,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Noue sud principale (corridor 2 m).</t>
+          <t>Segment sud 20 m correspondant a l'emprise du bassin lineaire (pas superpose a E03).</t>
         </is>
       </c>
       <c r="AC7" s="7" t="n"/>
@@ -8688,7 +8737,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="F12" s="15">
@@ -8796,51 +8845,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>E06</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>J-OUEST-AVAL</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>J-BASSIN-IN</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>E07</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="H13" s="7" t="inlineStr"/>
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
       <c r="I13" s="8">
         <f>IF(A13="","",IF(H13&lt;&gt;"",H13,IF(UPPER(TRIM(B13))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B13))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J13" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
-      <c r="M13" s="7" t="inlineStr"/>
-      <c r="N13" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
       <c r="O13" s="8">
         <f>IF(A13="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A13))</f>
         <v/>
@@ -8893,11 +8914,7 @@
         <f>IF(A13="","",IF(OR(U13&gt;1,AND(X13&lt;&gt;"",X13&lt;Inputs!$B$16),AND(X13&lt;&gt;"",X13&gt;Inputs!$B$17),G13&lt;Inputs!$B$18,AH13="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB13" s="4" t="inlineStr">
-        <is>
-          <t>Branche ouest vers entree bassin.</t>
-        </is>
-      </c>
+      <c r="AB13" s="4" t="n"/>
       <c r="AC13" s="7" t="n"/>
       <c r="AD13" s="8">
         <f>IF(A13="","",IF(AC13&lt;&gt;"",AC13,IF(E13="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E13,$A$4:$A$204,0)),""))))</f>
@@ -8943,10 +8960,10 @@
       </c>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="8">
@@ -8954,7 +8971,7 @@
         <v/>
       </c>
       <c r="J14" s="7" t="n">
-        <v>525</v>
+        <v>450</v>
       </c>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr"/>
@@ -9016,7 +9033,7 @@
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
-          <t>Injection finale vers bassin retention.</t>
+          <t>Courte liaison d'entree/ouvrage de regulation vers noeud de stockage BASSIN-RET.</t>
         </is>
       </c>
       <c r="AC14" s="7" t="n"/>

</xml_diff>

<commit_message>
Set west basin entry to 4.7m and add dual east-west basin inlets
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -742,6 +742,34 @@
       <c r="A32" t="inlineStr">
         <is>
           <t>Bassin retention longueur mise a 20 m (Inputs!B35) selon releve plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Deux entrees bassin implementees: EST via E03-&gt;E07 et OUEST via E04-&gt;E08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>E04 corrige a 4.7 m (J-OUEST-AVAL -&gt; J-BASSIN-OUEST), sans superposition avec E03.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Traverses pave-uni ouest conservees en caniveau + conduite (E05B, E05D).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Principe invert: fond swale a l'entree doit rester au-dessus de l'invert du tuyau d'entree + chute locale (drop).</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2596,6 +2624,26 @@
       <c r="D52" s="4" t="inlineStr">
         <is>
           <t>NO recommande: empreinte bassin n'est pas contributive au bassin lui-meme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>West_swale_to_basin_inlet_m</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Distance mesuree J-OUEST-AVAL -&gt; entree ouest bassin (image utilisateur).</t>
         </is>
       </c>
     </row>
@@ -2737,12 +2785,12 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Toiture vers collecte sud</t>
+          <t>Routage provisoire vers entree EST; scinder est/ouest plus tard si detail aval disponible.</t>
         </is>
       </c>
     </row>
@@ -3147,12 +3195,12 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Vers noue sud</t>
+          <t>Routage vers entree EST (courbe cote est sur plan).</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8090,7 @@
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>Corrige: P-03 -&gt; J-BASSIN-IN = 16.1 m (pas 20 m).</t>
+          <t>Entree EST: P-03 -&gt; J-BASSIN-IN (16.1 m).</t>
         </is>
       </c>
       <c r="AC6" s="7" t="n"/>
@@ -8085,16 +8133,17 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>J-BASSIN-IN</t>
+          <t>J-BASSIN-OUEST</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>E07</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>20</v>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="F7" s="7">
+        <f>Inputs!$B$53</f>
+        <v/>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.004</v>
@@ -8105,23 +8154,17 @@
         <v/>
       </c>
       <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7">
-        <f>Inputs!$B$34</f>
-        <v/>
-      </c>
-      <c r="L7" s="7">
-        <f>Inputs!$B$36</f>
-        <v/>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K7" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="O7" s="8">
         <f>IF(A7="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A7))</f>
@@ -8177,7 +8220,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Segment sud 20 m correspondant a l'emprise du bassin lineaire (pas superpose a E03).</t>
+          <t>Corrige: liaison ouest courte vers entree ouest bassin (4.7 m mesure).</t>
         </is>
       </c>
       <c r="AC7" s="7" t="n"/>
@@ -8433,7 +8476,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Ouest pave-uni court - longueur cotee 2.3 m.</t>
+          <t>Traverse pave-uni court via caniveau/grille + conduite (DN250).</t>
         </is>
       </c>
       <c r="AC9" s="7" t="n"/>
@@ -8689,7 +8732,7 @@
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>Ouest pave-uni inferieur - longueur cotee 5.1 m.</t>
+          <t>Traverse pave-uni principal via caniveau/grille + conduite (DN300).</t>
         </is>
       </c>
       <c r="AC11" s="7" t="n"/>
@@ -9059,23 +9102,47 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>J-BASSIN-OUEST</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0.005</v>
+      </c>
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="8">
         <f>IF(A15="","",IF(H15&lt;&gt;"",H15,IF(UPPER(TRIM(B15))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B15))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
+      <c r="J15" s="7" t="n">
+        <v>375</v>
+      </c>
+      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="O15" s="8">
         <f>IF(A15="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A15))</f>
         <v/>
@@ -9128,7 +9195,11 @@
         <f>IF(A15="","",IF(OR(U15&gt;1,AND(X15&lt;&gt;"",X15&lt;Inputs!$B$16),AND(X15&lt;&gt;"",X15&gt;Inputs!$B$17),G15&lt;Inputs!$B$18,AH15="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB15" s="4" t="n"/>
+      <c r="AB15" s="4" t="inlineStr">
+        <is>
+          <t>Entree OUEST: liaison caniveau/ouvrage vers bassin (2e entree).</t>
+        </is>
+      </c>
       <c r="AC15" s="7" t="n"/>
       <c r="AD15" s="8">
         <f>IF(A15="","",IF(AC15&lt;&gt;"",AC15,IF(E15="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E15,$A$4:$A$204,0)),""))))</f>
@@ -27849,22 +27920,39 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>J-BASSIN-OUEST</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="8">
         <f>IF(OR(C17="",D17=""),"",MAX(0,C17-D17))</f>
         <v/>
       </c>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H17" s="7" t="inlineStr"/>
       <c r="I17" s="8">
         <f>IF(A17="","",IF(UPPER(TRIM(F17))="CIRC",PI()*(G17/2)^2*E17,IF(UPPER(TRIM(F17))="RECT",G17*H17*E17,"")))</f>
         <v/>
       </c>
-      <c r="J17" s="7" t="n"/>
+      <c r="J17" s="7">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
       <c r="K17" s="8">
         <f>IF(A17="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A17))</f>
         <v/>

</xml_diff>

<commit_message>
Update surface types to pavage and retune IDF plus swale-pipe drop logic
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -801,6 +801,34 @@
       <c r="A40" t="inlineStr">
         <is>
           <t>Si AL=CHECK: ajuster invert aval/amont (AC override ou pente/longueur) ou ajouter ouvrage de chute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Types de surface mis a jour: PAVAGE ajoute explicitement (Inputs!B58) et applique a Z07/Z08/Z10/Z12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Z13 supprime de la configuration active (ligne vide).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Raccord SWALE/TRENCH -&gt; PIPE: AD applique automatiquement une chute cible Inputs!B57 (si pas d'override AC).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cela represente un raccord via regard/caniveau: fond noue plus haut que l'invert de conduite aval.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1656,7 +1684,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>4156.21</v>
+        <v>7423.67</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -1676,7 +1704,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>15.1</v>
+        <v>33.5</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -1696,7 +1724,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1.026</v>
+        <v>1.148</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1876,7 +1904,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
@@ -2755,6 +2783,26 @@
       <c r="D57" s="4" t="inlineStr">
         <is>
           <t>Valeur cible pratique pour entree swale/trench vers conduite bassin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>C_pavage</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Coefficient ruissellement pour surfaces pavees (pave-uni/pavage).</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2928,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr"/>
       <c r="F4" s="8">
-        <f>IF(E4&lt;&gt;"",E4,IF(UPPER(TRIM(C4))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C4))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C4))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C4))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E4&lt;&gt;"",E4,IF(UPPER(TRIM(C4))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C4))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C4))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C4))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C4))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G4" s="7" t="n">
@@ -2926,7 +2974,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="8">
-        <f>IF(E5&lt;&gt;"",E5,IF(UPPER(TRIM(C5))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C5))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C5))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C5))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E5&lt;&gt;"",E5,IF(UPPER(TRIM(C5))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C5))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C5))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C5))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C5))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G5" s="7" t="n">
@@ -2972,7 +3020,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr"/>
       <c r="F6" s="8">
-        <f>IF(E6&lt;&gt;"",E6,IF(UPPER(TRIM(C6))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C6))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C6))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C6))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E6&lt;&gt;"",E6,IF(UPPER(TRIM(C6))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C6))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C6))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C6))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C6))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G6" s="7" t="n">
@@ -3018,7 +3066,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="8">
-        <f>IF(E7&lt;&gt;"",E7,IF(UPPER(TRIM(C7))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C7))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C7))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C7))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E7&lt;&gt;"",E7,IF(UPPER(TRIM(C7))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C7))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C7))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C7))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C7))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G7" s="7" t="n">
@@ -3056,7 +3104,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>PAVAGE</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -3064,7 +3112,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr"/>
       <c r="F8" s="8">
-        <f>IF(E8&lt;&gt;"",E8,IF(UPPER(TRIM(C8))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C8))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C8))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C8))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E8&lt;&gt;"",E8,IF(UPPER(TRIM(C8))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C8))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C8))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C8))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C8))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G8" s="7" t="n">
@@ -3085,7 +3133,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Image: petit troncon pave entre zones gazon.</t>
+          <t>Surface pavage (pas tresfond).</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3158,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="8">
-        <f>IF(E9&lt;&gt;"",E9,IF(UPPER(TRIM(C9))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C9))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C9))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C9))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E9&lt;&gt;"",E9,IF(UPPER(TRIM(C9))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C9))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C9))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C9))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C9))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G9" s="7" t="n">
@@ -3148,7 +3196,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>PAVAGE</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
@@ -3156,7 +3204,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr"/>
       <c r="F10" s="8">
-        <f>IF(E10&lt;&gt;"",E10,IF(UPPER(TRIM(C10))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C10))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C10))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C10))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E10&lt;&gt;"",E10,IF(UPPER(TRIM(C10))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C10))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C10))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C10))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C10))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G10" s="7" t="n">
@@ -3177,7 +3225,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>LOCALISATION: zone pavee entre Z05 et Z06 (pas l'entree pavee externe).</t>
+          <t>Surface pavage principal (pave-uni), entre Z05 et Z06.</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3250,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="8">
-        <f>IF(E11&lt;&gt;"",E11,IF(UPPER(TRIM(C11))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C11))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C11))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C11))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E11&lt;&gt;"",E11,IF(UPPER(TRIM(C11))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C11))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C11))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C11))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C11))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G11" s="7" t="n">
@@ -3248,7 +3296,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr"/>
       <c r="F12" s="8">
-        <f>IF(E12&lt;&gt;"",E12,IF(UPPER(TRIM(C12))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C12))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C12))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C12))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E12&lt;&gt;"",E12,IF(UPPER(TRIM(C12))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C12))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C12))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C12))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C12))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G12" s="7" t="n">
@@ -3277,12 +3325,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Sud gris local</t>
+          <t>Sud gris local (pavage)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>PAVAGE</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
@@ -3290,7 +3338,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="8">
-        <f>IF(E13&lt;&gt;"",E13,IF(UPPER(TRIM(C13))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C13))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C13))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C13))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E13&lt;&gt;"",E13,IF(UPPER(TRIM(C13))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C13))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C13))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C13))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C13))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G13" s="7" t="n">
@@ -3311,7 +3359,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Routage vers entree EST (courbe cote est sur plan).</t>
+          <t>Surface pavage locale (pas tresfond), routage vers entree EST.</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3384,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr"/>
       <c r="F14" s="8">
-        <f>IF(E14&lt;&gt;"",E14,IF(UPPER(TRIM(C14))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C14))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C14))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C14))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E14&lt;&gt;"",E14,IF(UPPER(TRIM(C14))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C14))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C14))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C14))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C14))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G14" s="7" t="n">
@@ -3369,12 +3417,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Sud est gris petit</t>
+          <t>Sud est gris petit (pavage)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TRESFOND</t>
+          <t>PAVAGE</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
@@ -3382,7 +3430,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="8">
-        <f>IF(E15&lt;&gt;"",E15,IF(UPPER(TRIM(C15))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C15))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C15))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C15))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E15&lt;&gt;"",E15,IF(UPPER(TRIM(C15))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C15))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C15))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C15))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C15))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G15" s="7" t="n">
@@ -3403,38 +3451,21 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Vers noue sud</t>
+          <t>Surface pavage petite zone sud-est (pas tresfond).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Z13</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Tresfond haut central (bande nord centrale)</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>TRESFOND</t>
-        </is>
-      </c>
-      <c r="D16" s="7">
-        <f>Inputs!$B$51</f>
-        <v/>
-      </c>
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="7" t="n"/>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="8">
-        <f>IF(E16&lt;&gt;"",E16,IF(UPPER(TRIM(C16))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C16))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C16))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C16))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
-        <v/>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>8</v>
-      </c>
+        <f>IF(E16&lt;&gt;"",E16,IF(UPPER(TRIM(C16))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C16))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C16))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C16))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C16))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="n"/>
       <c r="H16" s="8">
         <f>IF(A16="","",Inputs!$B$3/((IF(G16="",Inputs!$B$14,G16)+Inputs!$B$4)^Inputs!$B$5))</f>
         <v/>
@@ -3443,16 +3474,8 @@
         <f>IF(A16="","",2.78E-7*F16*D16*H16)</f>
         <v/>
       </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Ajoute pour inclure le tresfond central haut; saisir aire exacte Inputs!B51.</t>
-        </is>
-      </c>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -3461,7 +3484,7 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="8">
-        <f>IF(E17&lt;&gt;"",E17,IF(UPPER(TRIM(C17))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C17))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C17))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C17))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E17&lt;&gt;"",E17,IF(UPPER(TRIM(C17))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C17))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C17))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C17))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C17))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G17" s="7" t="n"/>
@@ -3483,7 +3506,7 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="8">
-        <f>IF(E18&lt;&gt;"",E18,IF(UPPER(TRIM(C18))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C18))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C18))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C18))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E18&lt;&gt;"",E18,IF(UPPER(TRIM(C18))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C18))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C18))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C18))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C18))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G18" s="7" t="n"/>
@@ -3505,7 +3528,7 @@
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="8">
-        <f>IF(E19&lt;&gt;"",E19,IF(UPPER(TRIM(C19))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C19))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C19))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C19))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E19&lt;&gt;"",E19,IF(UPPER(TRIM(C19))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C19))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C19))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C19))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C19))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G19" s="7" t="n"/>
@@ -3527,7 +3550,7 @@
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="8">
-        <f>IF(E20&lt;&gt;"",E20,IF(UPPER(TRIM(C20))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C20))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C20))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C20))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E20&lt;&gt;"",E20,IF(UPPER(TRIM(C20))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C20))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C20))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C20))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C20))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G20" s="7" t="n"/>
@@ -3549,7 +3572,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="8">
-        <f>IF(E21&lt;&gt;"",E21,IF(UPPER(TRIM(C21))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C21))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C21))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C21))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E21&lt;&gt;"",E21,IF(UPPER(TRIM(C21))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C21))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C21))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C21))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C21))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G21" s="7" t="n"/>
@@ -3571,7 +3594,7 @@
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="8">
-        <f>IF(E22&lt;&gt;"",E22,IF(UPPER(TRIM(C22))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C22))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C22))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C22))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E22&lt;&gt;"",E22,IF(UPPER(TRIM(C22))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C22))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C22))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C22))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C22))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G22" s="7" t="n"/>
@@ -3593,7 +3616,7 @@
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="8">
-        <f>IF(E23&lt;&gt;"",E23,IF(UPPER(TRIM(C23))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C23))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C23))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C23))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E23&lt;&gt;"",E23,IF(UPPER(TRIM(C23))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C23))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C23))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C23))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C23))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G23" s="7" t="n"/>
@@ -3615,7 +3638,7 @@
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="8">
-        <f>IF(E24&lt;&gt;"",E24,IF(UPPER(TRIM(C24))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C24))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C24))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C24))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E24&lt;&gt;"",E24,IF(UPPER(TRIM(C24))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C24))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C24))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C24))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C24))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G24" s="7" t="n"/>
@@ -3637,7 +3660,7 @@
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="8">
-        <f>IF(E25&lt;&gt;"",E25,IF(UPPER(TRIM(C25))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C25))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C25))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C25))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E25&lt;&gt;"",E25,IF(UPPER(TRIM(C25))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C25))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C25))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C25))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C25))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G25" s="7" t="n"/>
@@ -3659,7 +3682,7 @@
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="8">
-        <f>IF(E26&lt;&gt;"",E26,IF(UPPER(TRIM(C26))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C26))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C26))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C26))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E26&lt;&gt;"",E26,IF(UPPER(TRIM(C26))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C26))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C26))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C26))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C26))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G26" s="7" t="n"/>
@@ -3681,7 +3704,7 @@
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="8">
-        <f>IF(E27&lt;&gt;"",E27,IF(UPPER(TRIM(C27))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C27))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C27))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C27))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E27&lt;&gt;"",E27,IF(UPPER(TRIM(C27))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C27))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C27))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C27))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C27))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G27" s="7" t="n"/>
@@ -3703,7 +3726,7 @@
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="8">
-        <f>IF(E28&lt;&gt;"",E28,IF(UPPER(TRIM(C28))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C28))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C28))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C28))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E28&lt;&gt;"",E28,IF(UPPER(TRIM(C28))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C28))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C28))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C28))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C28))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G28" s="7" t="n"/>
@@ -3725,7 +3748,7 @@
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="8">
-        <f>IF(E29&lt;&gt;"",E29,IF(UPPER(TRIM(C29))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C29))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C29))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C29))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E29&lt;&gt;"",E29,IF(UPPER(TRIM(C29))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C29))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C29))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C29))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C29))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G29" s="7" t="n"/>
@@ -3747,7 +3770,7 @@
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="8">
-        <f>IF(E30&lt;&gt;"",E30,IF(UPPER(TRIM(C30))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C30))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C30))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C30))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E30&lt;&gt;"",E30,IF(UPPER(TRIM(C30))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C30))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C30))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C30))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C30))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G30" s="7" t="n"/>
@@ -3769,7 +3792,7 @@
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="8">
-        <f>IF(E31&lt;&gt;"",E31,IF(UPPER(TRIM(C31))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C31))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C31))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C31))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E31&lt;&gt;"",E31,IF(UPPER(TRIM(C31))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C31))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C31))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C31))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C31))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G31" s="7" t="n"/>
@@ -3791,7 +3814,7 @@
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="8">
-        <f>IF(E32&lt;&gt;"",E32,IF(UPPER(TRIM(C32))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C32))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C32))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C32))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E32&lt;&gt;"",E32,IF(UPPER(TRIM(C32))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C32))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C32))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C32))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C32))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G32" s="7" t="n"/>
@@ -3813,7 +3836,7 @@
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="8">
-        <f>IF(E33&lt;&gt;"",E33,IF(UPPER(TRIM(C33))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C33))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C33))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C33))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E33&lt;&gt;"",E33,IF(UPPER(TRIM(C33))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C33))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C33))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C33))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C33))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G33" s="7" t="n"/>
@@ -3835,7 +3858,7 @@
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="8">
-        <f>IF(E34&lt;&gt;"",E34,IF(UPPER(TRIM(C34))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C34))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C34))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C34))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E34&lt;&gt;"",E34,IF(UPPER(TRIM(C34))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C34))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C34))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C34))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C34))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G34" s="7" t="n"/>
@@ -3857,7 +3880,7 @@
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="8">
-        <f>IF(E35&lt;&gt;"",E35,IF(UPPER(TRIM(C35))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C35))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C35))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C35))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E35&lt;&gt;"",E35,IF(UPPER(TRIM(C35))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C35))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C35))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C35))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C35))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G35" s="7" t="n"/>
@@ -3879,7 +3902,7 @@
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="8">
-        <f>IF(E36&lt;&gt;"",E36,IF(UPPER(TRIM(C36))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C36))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C36))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C36))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E36&lt;&gt;"",E36,IF(UPPER(TRIM(C36))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C36))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C36))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C36))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C36))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G36" s="7" t="n"/>
@@ -3901,7 +3924,7 @@
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="8">
-        <f>IF(E37&lt;&gt;"",E37,IF(UPPER(TRIM(C37))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C37))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C37))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C37))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E37&lt;&gt;"",E37,IF(UPPER(TRIM(C37))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C37))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C37))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C37))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C37))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G37" s="7" t="n"/>
@@ -3923,7 +3946,7 @@
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="8">
-        <f>IF(E38&lt;&gt;"",E38,IF(UPPER(TRIM(C38))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C38))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C38))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C38))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E38&lt;&gt;"",E38,IF(UPPER(TRIM(C38))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C38))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C38))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C38))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C38))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G38" s="7" t="n"/>
@@ -3945,7 +3968,7 @@
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="8">
-        <f>IF(E39&lt;&gt;"",E39,IF(UPPER(TRIM(C39))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C39))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C39))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C39))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E39&lt;&gt;"",E39,IF(UPPER(TRIM(C39))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C39))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C39))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C39))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C39))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G39" s="7" t="n"/>
@@ -3967,7 +3990,7 @@
       <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="8">
-        <f>IF(E40&lt;&gt;"",E40,IF(UPPER(TRIM(C40))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C40))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C40))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C40))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E40&lt;&gt;"",E40,IF(UPPER(TRIM(C40))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C40))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C40))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C40))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C40))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G40" s="7" t="n"/>
@@ -3989,7 +4012,7 @@
       <c r="D41" s="7" t="n"/>
       <c r="E41" s="7" t="n"/>
       <c r="F41" s="8">
-        <f>IF(E41&lt;&gt;"",E41,IF(UPPER(TRIM(C41))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C41))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C41))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C41))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E41&lt;&gt;"",E41,IF(UPPER(TRIM(C41))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C41))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C41))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C41))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C41))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G41" s="7" t="n"/>
@@ -4011,7 +4034,7 @@
       <c r="D42" s="7" t="n"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="8">
-        <f>IF(E42&lt;&gt;"",E42,IF(UPPER(TRIM(C42))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C42))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C42))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C42))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E42&lt;&gt;"",E42,IF(UPPER(TRIM(C42))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C42))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C42))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C42))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C42))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G42" s="7" t="n"/>
@@ -4033,7 +4056,7 @@
       <c r="D43" s="7" t="n"/>
       <c r="E43" s="7" t="n"/>
       <c r="F43" s="8">
-        <f>IF(E43&lt;&gt;"",E43,IF(UPPER(TRIM(C43))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C43))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C43))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C43))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E43&lt;&gt;"",E43,IF(UPPER(TRIM(C43))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C43))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C43))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C43))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C43))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G43" s="7" t="n"/>
@@ -4055,7 +4078,7 @@
       <c r="D44" s="7" t="n"/>
       <c r="E44" s="7" t="n"/>
       <c r="F44" s="8">
-        <f>IF(E44&lt;&gt;"",E44,IF(UPPER(TRIM(C44))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C44))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C44))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C44))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E44&lt;&gt;"",E44,IF(UPPER(TRIM(C44))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C44))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C44))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C44))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C44))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G44" s="7" t="n"/>
@@ -4077,7 +4100,7 @@
       <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="8">
-        <f>IF(E45&lt;&gt;"",E45,IF(UPPER(TRIM(C45))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C45))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C45))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C45))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E45&lt;&gt;"",E45,IF(UPPER(TRIM(C45))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C45))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C45))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C45))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C45))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G45" s="7" t="n"/>
@@ -4099,7 +4122,7 @@
       <c r="D46" s="7" t="n"/>
       <c r="E46" s="7" t="n"/>
       <c r="F46" s="8">
-        <f>IF(E46&lt;&gt;"",E46,IF(UPPER(TRIM(C46))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C46))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C46))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C46))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E46&lt;&gt;"",E46,IF(UPPER(TRIM(C46))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C46))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C46))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C46))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C46))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G46" s="7" t="n"/>
@@ -4121,7 +4144,7 @@
       <c r="D47" s="7" t="n"/>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="8">
-        <f>IF(E47&lt;&gt;"",E47,IF(UPPER(TRIM(C47))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C47))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C47))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C47))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E47&lt;&gt;"",E47,IF(UPPER(TRIM(C47))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C47))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C47))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C47))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C47))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G47" s="7" t="n"/>
@@ -4143,7 +4166,7 @@
       <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="8">
-        <f>IF(E48&lt;&gt;"",E48,IF(UPPER(TRIM(C48))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C48))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C48))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C48))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E48&lt;&gt;"",E48,IF(UPPER(TRIM(C48))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C48))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C48))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C48))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C48))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G48" s="7" t="n"/>
@@ -4165,7 +4188,7 @@
       <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="8">
-        <f>IF(E49&lt;&gt;"",E49,IF(UPPER(TRIM(C49))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C49))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C49))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C49))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E49&lt;&gt;"",E49,IF(UPPER(TRIM(C49))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C49))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C49))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C49))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C49))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G49" s="7" t="n"/>
@@ -4187,7 +4210,7 @@
       <c r="D50" s="7" t="n"/>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="8">
-        <f>IF(E50&lt;&gt;"",E50,IF(UPPER(TRIM(C50))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C50))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C50))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C50))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E50&lt;&gt;"",E50,IF(UPPER(TRIM(C50))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C50))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C50))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C50))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C50))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G50" s="7" t="n"/>
@@ -4209,7 +4232,7 @@
       <c r="D51" s="7" t="n"/>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="8">
-        <f>IF(E51&lt;&gt;"",E51,IF(UPPER(TRIM(C51))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C51))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C51))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C51))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E51&lt;&gt;"",E51,IF(UPPER(TRIM(C51))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C51))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C51))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C51))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C51))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G51" s="7" t="n"/>
@@ -4231,7 +4254,7 @@
       <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="8">
-        <f>IF(E52&lt;&gt;"",E52,IF(UPPER(TRIM(C52))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C52))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C52))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C52))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E52&lt;&gt;"",E52,IF(UPPER(TRIM(C52))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C52))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C52))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C52))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C52))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G52" s="7" t="n"/>
@@ -4253,7 +4276,7 @@
       <c r="D53" s="7" t="n"/>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="8">
-        <f>IF(E53&lt;&gt;"",E53,IF(UPPER(TRIM(C53))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C53))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C53))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C53))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E53&lt;&gt;"",E53,IF(UPPER(TRIM(C53))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C53))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C53))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C53))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C53))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G53" s="7" t="n"/>
@@ -4275,7 +4298,7 @@
       <c r="D54" s="7" t="n"/>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="8">
-        <f>IF(E54&lt;&gt;"",E54,IF(UPPER(TRIM(C54))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C54))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C54))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C54))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E54&lt;&gt;"",E54,IF(UPPER(TRIM(C54))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C54))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C54))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C54))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C54))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G54" s="7" t="n"/>
@@ -4297,7 +4320,7 @@
       <c r="D55" s="7" t="n"/>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="8">
-        <f>IF(E55&lt;&gt;"",E55,IF(UPPER(TRIM(C55))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C55))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C55))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C55))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E55&lt;&gt;"",E55,IF(UPPER(TRIM(C55))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C55))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C55))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C55))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C55))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G55" s="7" t="n"/>
@@ -4319,7 +4342,7 @@
       <c r="D56" s="7" t="n"/>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="8">
-        <f>IF(E56&lt;&gt;"",E56,IF(UPPER(TRIM(C56))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C56))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C56))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C56))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E56&lt;&gt;"",E56,IF(UPPER(TRIM(C56))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C56))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C56))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C56))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C56))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G56" s="7" t="n"/>
@@ -4341,7 +4364,7 @@
       <c r="D57" s="7" t="n"/>
       <c r="E57" s="7" t="n"/>
       <c r="F57" s="8">
-        <f>IF(E57&lt;&gt;"",E57,IF(UPPER(TRIM(C57))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C57))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C57))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C57))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E57&lt;&gt;"",E57,IF(UPPER(TRIM(C57))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C57))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C57))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C57))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C57))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G57" s="7" t="n"/>
@@ -4363,7 +4386,7 @@
       <c r="D58" s="7" t="n"/>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="8">
-        <f>IF(E58&lt;&gt;"",E58,IF(UPPER(TRIM(C58))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C58))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C58))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C58))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E58&lt;&gt;"",E58,IF(UPPER(TRIM(C58))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C58))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C58))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C58))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C58))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G58" s="7" t="n"/>
@@ -4385,7 +4408,7 @@
       <c r="D59" s="7" t="n"/>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="8">
-        <f>IF(E59&lt;&gt;"",E59,IF(UPPER(TRIM(C59))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C59))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C59))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C59))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E59&lt;&gt;"",E59,IF(UPPER(TRIM(C59))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C59))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C59))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C59))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C59))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G59" s="7" t="n"/>
@@ -4407,7 +4430,7 @@
       <c r="D60" s="7" t="n"/>
       <c r="E60" s="7" t="n"/>
       <c r="F60" s="8">
-        <f>IF(E60&lt;&gt;"",E60,IF(UPPER(TRIM(C60))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C60))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C60))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C60))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E60&lt;&gt;"",E60,IF(UPPER(TRIM(C60))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C60))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C60))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C60))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C60))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G60" s="7" t="n"/>
@@ -4429,7 +4452,7 @@
       <c r="D61" s="7" t="n"/>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="8">
-        <f>IF(E61&lt;&gt;"",E61,IF(UPPER(TRIM(C61))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C61))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C61))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C61))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E61&lt;&gt;"",E61,IF(UPPER(TRIM(C61))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C61))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C61))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C61))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C61))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G61" s="7" t="n"/>
@@ -4451,7 +4474,7 @@
       <c r="D62" s="7" t="n"/>
       <c r="E62" s="7" t="n"/>
       <c r="F62" s="8">
-        <f>IF(E62&lt;&gt;"",E62,IF(UPPER(TRIM(C62))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C62))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C62))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C62))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E62&lt;&gt;"",E62,IF(UPPER(TRIM(C62))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C62))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C62))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C62))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C62))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G62" s="7" t="n"/>
@@ -4473,7 +4496,7 @@
       <c r="D63" s="7" t="n"/>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="8">
-        <f>IF(E63&lt;&gt;"",E63,IF(UPPER(TRIM(C63))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C63))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C63))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C63))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E63&lt;&gt;"",E63,IF(UPPER(TRIM(C63))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C63))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C63))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C63))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C63))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G63" s="7" t="n"/>
@@ -4495,7 +4518,7 @@
       <c r="D64" s="7" t="n"/>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="8">
-        <f>IF(E64&lt;&gt;"",E64,IF(UPPER(TRIM(C64))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C64))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C64))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C64))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E64&lt;&gt;"",E64,IF(UPPER(TRIM(C64))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C64))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C64))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C64))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C64))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G64" s="7" t="n"/>
@@ -4517,7 +4540,7 @@
       <c r="D65" s="7" t="n"/>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="8">
-        <f>IF(E65&lt;&gt;"",E65,IF(UPPER(TRIM(C65))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C65))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C65))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C65))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E65&lt;&gt;"",E65,IF(UPPER(TRIM(C65))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C65))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C65))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C65))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C65))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G65" s="7" t="n"/>
@@ -4539,7 +4562,7 @@
       <c r="D66" s="7" t="n"/>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="8">
-        <f>IF(E66&lt;&gt;"",E66,IF(UPPER(TRIM(C66))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C66))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C66))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C66))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E66&lt;&gt;"",E66,IF(UPPER(TRIM(C66))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C66))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C66))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C66))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C66))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G66" s="7" t="n"/>
@@ -4561,7 +4584,7 @@
       <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="8">
-        <f>IF(E67&lt;&gt;"",E67,IF(UPPER(TRIM(C67))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C67))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C67))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C67))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E67&lt;&gt;"",E67,IF(UPPER(TRIM(C67))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C67))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C67))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C67))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C67))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G67" s="7" t="n"/>
@@ -4583,7 +4606,7 @@
       <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="8">
-        <f>IF(E68&lt;&gt;"",E68,IF(UPPER(TRIM(C68))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C68))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C68))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C68))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E68&lt;&gt;"",E68,IF(UPPER(TRIM(C68))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C68))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C68))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C68))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C68))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G68" s="7" t="n"/>
@@ -4605,7 +4628,7 @@
       <c r="D69" s="7" t="n"/>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="8">
-        <f>IF(E69&lt;&gt;"",E69,IF(UPPER(TRIM(C69))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C69))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C69))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C69))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E69&lt;&gt;"",E69,IF(UPPER(TRIM(C69))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C69))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C69))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C69))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C69))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G69" s="7" t="n"/>
@@ -4627,7 +4650,7 @@
       <c r="D70" s="7" t="n"/>
       <c r="E70" s="7" t="n"/>
       <c r="F70" s="8">
-        <f>IF(E70&lt;&gt;"",E70,IF(UPPER(TRIM(C70))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C70))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C70))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C70))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E70&lt;&gt;"",E70,IF(UPPER(TRIM(C70))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C70))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C70))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C70))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C70))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G70" s="7" t="n"/>
@@ -4649,7 +4672,7 @@
       <c r="D71" s="7" t="n"/>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="8">
-        <f>IF(E71&lt;&gt;"",E71,IF(UPPER(TRIM(C71))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C71))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C71))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C71))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E71&lt;&gt;"",E71,IF(UPPER(TRIM(C71))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C71))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C71))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C71))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C71))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G71" s="7" t="n"/>
@@ -4671,7 +4694,7 @@
       <c r="D72" s="7" t="n"/>
       <c r="E72" s="7" t="n"/>
       <c r="F72" s="8">
-        <f>IF(E72&lt;&gt;"",E72,IF(UPPER(TRIM(C72))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C72))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C72))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C72))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E72&lt;&gt;"",E72,IF(UPPER(TRIM(C72))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C72))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C72))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C72))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C72))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G72" s="7" t="n"/>
@@ -4693,7 +4716,7 @@
       <c r="D73" s="7" t="n"/>
       <c r="E73" s="7" t="n"/>
       <c r="F73" s="8">
-        <f>IF(E73&lt;&gt;"",E73,IF(UPPER(TRIM(C73))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C73))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C73))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C73))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E73&lt;&gt;"",E73,IF(UPPER(TRIM(C73))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C73))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C73))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C73))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C73))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G73" s="7" t="n"/>
@@ -4715,7 +4738,7 @@
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="8">
-        <f>IF(E74&lt;&gt;"",E74,IF(UPPER(TRIM(C74))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C74))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C74))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C74))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E74&lt;&gt;"",E74,IF(UPPER(TRIM(C74))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C74))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C74))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C74))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C74))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G74" s="7" t="n"/>
@@ -4737,7 +4760,7 @@
       <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="8">
-        <f>IF(E75&lt;&gt;"",E75,IF(UPPER(TRIM(C75))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C75))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C75))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C75))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E75&lt;&gt;"",E75,IF(UPPER(TRIM(C75))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C75))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C75))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C75))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C75))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G75" s="7" t="n"/>
@@ -4759,7 +4782,7 @@
       <c r="D76" s="7" t="n"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="8">
-        <f>IF(E76&lt;&gt;"",E76,IF(UPPER(TRIM(C76))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C76))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C76))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C76))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E76&lt;&gt;"",E76,IF(UPPER(TRIM(C76))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C76))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C76))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C76))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C76))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G76" s="7" t="n"/>
@@ -4781,7 +4804,7 @@
       <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="8">
-        <f>IF(E77&lt;&gt;"",E77,IF(UPPER(TRIM(C77))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C77))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C77))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C77))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E77&lt;&gt;"",E77,IF(UPPER(TRIM(C77))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C77))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C77))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C77))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C77))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G77" s="7" t="n"/>
@@ -4803,7 +4826,7 @@
       <c r="D78" s="7" t="n"/>
       <c r="E78" s="7" t="n"/>
       <c r="F78" s="8">
-        <f>IF(E78&lt;&gt;"",E78,IF(UPPER(TRIM(C78))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C78))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C78))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C78))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E78&lt;&gt;"",E78,IF(UPPER(TRIM(C78))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C78))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C78))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C78))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C78))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G78" s="7" t="n"/>
@@ -4825,7 +4848,7 @@
       <c r="D79" s="7" t="n"/>
       <c r="E79" s="7" t="n"/>
       <c r="F79" s="8">
-        <f>IF(E79&lt;&gt;"",E79,IF(UPPER(TRIM(C79))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C79))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C79))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C79))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E79&lt;&gt;"",E79,IF(UPPER(TRIM(C79))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C79))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C79))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C79))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C79))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G79" s="7" t="n"/>
@@ -4847,7 +4870,7 @@
       <c r="D80" s="7" t="n"/>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="8">
-        <f>IF(E80&lt;&gt;"",E80,IF(UPPER(TRIM(C80))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C80))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C80))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C80))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E80&lt;&gt;"",E80,IF(UPPER(TRIM(C80))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C80))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C80))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C80))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C80))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G80" s="7" t="n"/>
@@ -4869,7 +4892,7 @@
       <c r="D81" s="7" t="n"/>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="8">
-        <f>IF(E81&lt;&gt;"",E81,IF(UPPER(TRIM(C81))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C81))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C81))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C81))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E81&lt;&gt;"",E81,IF(UPPER(TRIM(C81))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C81))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C81))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C81))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C81))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G81" s="7" t="n"/>
@@ -4891,7 +4914,7 @@
       <c r="D82" s="7" t="n"/>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="8">
-        <f>IF(E82&lt;&gt;"",E82,IF(UPPER(TRIM(C82))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C82))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C82))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C82))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E82&lt;&gt;"",E82,IF(UPPER(TRIM(C82))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C82))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C82))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C82))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C82))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G82" s="7" t="n"/>
@@ -4913,7 +4936,7 @@
       <c r="D83" s="7" t="n"/>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="8">
-        <f>IF(E83&lt;&gt;"",E83,IF(UPPER(TRIM(C83))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C83))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C83))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C83))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E83&lt;&gt;"",E83,IF(UPPER(TRIM(C83))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C83))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C83))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C83))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C83))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G83" s="7" t="n"/>
@@ -4935,7 +4958,7 @@
       <c r="D84" s="7" t="n"/>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="8">
-        <f>IF(E84&lt;&gt;"",E84,IF(UPPER(TRIM(C84))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C84))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C84))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C84))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E84&lt;&gt;"",E84,IF(UPPER(TRIM(C84))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C84))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C84))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C84))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C84))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G84" s="7" t="n"/>
@@ -4957,7 +4980,7 @@
       <c r="D85" s="7" t="n"/>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="8">
-        <f>IF(E85&lt;&gt;"",E85,IF(UPPER(TRIM(C85))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C85))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C85))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C85))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E85&lt;&gt;"",E85,IF(UPPER(TRIM(C85))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C85))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C85))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C85))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C85))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G85" s="7" t="n"/>
@@ -4979,7 +5002,7 @@
       <c r="D86" s="7" t="n"/>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="8">
-        <f>IF(E86&lt;&gt;"",E86,IF(UPPER(TRIM(C86))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C86))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C86))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C86))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E86&lt;&gt;"",E86,IF(UPPER(TRIM(C86))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C86))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C86))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C86))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C86))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G86" s="7" t="n"/>
@@ -5001,7 +5024,7 @@
       <c r="D87" s="7" t="n"/>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="8">
-        <f>IF(E87&lt;&gt;"",E87,IF(UPPER(TRIM(C87))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C87))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C87))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C87))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E87&lt;&gt;"",E87,IF(UPPER(TRIM(C87))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C87))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C87))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C87))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C87))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G87" s="7" t="n"/>
@@ -5023,7 +5046,7 @@
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="8">
-        <f>IF(E88&lt;&gt;"",E88,IF(UPPER(TRIM(C88))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C88))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C88))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C88))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E88&lt;&gt;"",E88,IF(UPPER(TRIM(C88))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C88))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C88))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C88))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C88))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G88" s="7" t="n"/>
@@ -5045,7 +5068,7 @@
       <c r="D89" s="7" t="n"/>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="8">
-        <f>IF(E89&lt;&gt;"",E89,IF(UPPER(TRIM(C89))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C89))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C89))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C89))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E89&lt;&gt;"",E89,IF(UPPER(TRIM(C89))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C89))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C89))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C89))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C89))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G89" s="7" t="n"/>
@@ -5067,7 +5090,7 @@
       <c r="D90" s="7" t="n"/>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="8">
-        <f>IF(E90&lt;&gt;"",E90,IF(UPPER(TRIM(C90))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C90))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C90))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C90))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E90&lt;&gt;"",E90,IF(UPPER(TRIM(C90))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C90))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C90))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C90))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C90))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G90" s="7" t="n"/>
@@ -5089,7 +5112,7 @@
       <c r="D91" s="7" t="n"/>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="8">
-        <f>IF(E91&lt;&gt;"",E91,IF(UPPER(TRIM(C91))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C91))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C91))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C91))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E91&lt;&gt;"",E91,IF(UPPER(TRIM(C91))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C91))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C91))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C91))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C91))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G91" s="7" t="n"/>
@@ -5111,7 +5134,7 @@
       <c r="D92" s="7" t="n"/>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="8">
-        <f>IF(E92&lt;&gt;"",E92,IF(UPPER(TRIM(C92))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C92))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C92))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C92))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E92&lt;&gt;"",E92,IF(UPPER(TRIM(C92))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C92))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C92))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C92))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C92))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G92" s="7" t="n"/>
@@ -5133,7 +5156,7 @@
       <c r="D93" s="7" t="n"/>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="8">
-        <f>IF(E93&lt;&gt;"",E93,IF(UPPER(TRIM(C93))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C93))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C93))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C93))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E93&lt;&gt;"",E93,IF(UPPER(TRIM(C93))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C93))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C93))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C93))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C93))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G93" s="7" t="n"/>
@@ -5155,7 +5178,7 @@
       <c r="D94" s="7" t="n"/>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="8">
-        <f>IF(E94&lt;&gt;"",E94,IF(UPPER(TRIM(C94))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C94))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C94))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C94))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E94&lt;&gt;"",E94,IF(UPPER(TRIM(C94))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C94))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C94))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C94))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C94))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G94" s="7" t="n"/>
@@ -5177,7 +5200,7 @@
       <c r="D95" s="7" t="n"/>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="8">
-        <f>IF(E95&lt;&gt;"",E95,IF(UPPER(TRIM(C95))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C95))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C95))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C95))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E95&lt;&gt;"",E95,IF(UPPER(TRIM(C95))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C95))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C95))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C95))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C95))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G95" s="7" t="n"/>
@@ -5199,7 +5222,7 @@
       <c r="D96" s="7" t="n"/>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="8">
-        <f>IF(E96&lt;&gt;"",E96,IF(UPPER(TRIM(C96))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C96))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C96))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C96))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E96&lt;&gt;"",E96,IF(UPPER(TRIM(C96))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C96))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C96))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C96))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C96))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G96" s="7" t="n"/>
@@ -5221,7 +5244,7 @@
       <c r="D97" s="7" t="n"/>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="8">
-        <f>IF(E97&lt;&gt;"",E97,IF(UPPER(TRIM(C97))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C97))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C97))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C97))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E97&lt;&gt;"",E97,IF(UPPER(TRIM(C97))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C97))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C97))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C97))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C97))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G97" s="7" t="n"/>
@@ -5243,7 +5266,7 @@
       <c r="D98" s="7" t="n"/>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="8">
-        <f>IF(E98&lt;&gt;"",E98,IF(UPPER(TRIM(C98))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C98))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C98))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C98))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E98&lt;&gt;"",E98,IF(UPPER(TRIM(C98))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C98))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C98))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C98))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C98))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G98" s="7" t="n"/>
@@ -5265,7 +5288,7 @@
       <c r="D99" s="7" t="n"/>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="8">
-        <f>IF(E99&lt;&gt;"",E99,IF(UPPER(TRIM(C99))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C99))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C99))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C99))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E99&lt;&gt;"",E99,IF(UPPER(TRIM(C99))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C99))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C99))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C99))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C99))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G99" s="7" t="n"/>
@@ -5287,7 +5310,7 @@
       <c r="D100" s="7" t="n"/>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="8">
-        <f>IF(E100&lt;&gt;"",E100,IF(UPPER(TRIM(C100))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C100))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C100))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C100))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E100&lt;&gt;"",E100,IF(UPPER(TRIM(C100))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C100))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C100))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C100))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C100))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G100" s="7" t="n"/>
@@ -5309,7 +5332,7 @@
       <c r="D101" s="7" t="n"/>
       <c r="E101" s="7" t="n"/>
       <c r="F101" s="8">
-        <f>IF(E101&lt;&gt;"",E101,IF(UPPER(TRIM(C101))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C101))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C101))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C101))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E101&lt;&gt;"",E101,IF(UPPER(TRIM(C101))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C101))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C101))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C101))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C101))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G101" s="7" t="n"/>
@@ -5331,7 +5354,7 @@
       <c r="D102" s="7" t="n"/>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="8">
-        <f>IF(E102&lt;&gt;"",E102,IF(UPPER(TRIM(C102))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C102))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C102))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C102))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E102&lt;&gt;"",E102,IF(UPPER(TRIM(C102))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C102))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C102))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C102))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C102))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G102" s="7" t="n"/>
@@ -5353,7 +5376,7 @@
       <c r="D103" s="7" t="n"/>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="8">
-        <f>IF(E103&lt;&gt;"",E103,IF(UPPER(TRIM(C103))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C103))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C103))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C103))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E103&lt;&gt;"",E103,IF(UPPER(TRIM(C103))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C103))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C103))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C103))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C103))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G103" s="7" t="n"/>
@@ -5375,7 +5398,7 @@
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="8">
-        <f>IF(E104&lt;&gt;"",E104,IF(UPPER(TRIM(C104))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C104))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C104))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C104))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E104&lt;&gt;"",E104,IF(UPPER(TRIM(C104))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C104))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C104))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C104))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C104))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G104" s="7" t="n"/>
@@ -5397,7 +5420,7 @@
       <c r="D105" s="7" t="n"/>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="8">
-        <f>IF(E105&lt;&gt;"",E105,IF(UPPER(TRIM(C105))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C105))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C105))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C105))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E105&lt;&gt;"",E105,IF(UPPER(TRIM(C105))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C105))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C105))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C105))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C105))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G105" s="7" t="n"/>
@@ -5419,7 +5442,7 @@
       <c r="D106" s="7" t="n"/>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="8">
-        <f>IF(E106&lt;&gt;"",E106,IF(UPPER(TRIM(C106))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C106))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C106))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C106))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E106&lt;&gt;"",E106,IF(UPPER(TRIM(C106))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C106))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C106))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C106))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C106))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G106" s="7" t="n"/>
@@ -5441,7 +5464,7 @@
       <c r="D107" s="7" t="n"/>
       <c r="E107" s="7" t="n"/>
       <c r="F107" s="8">
-        <f>IF(E107&lt;&gt;"",E107,IF(UPPER(TRIM(C107))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C107))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C107))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C107))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E107&lt;&gt;"",E107,IF(UPPER(TRIM(C107))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C107))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C107))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C107))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C107))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G107" s="7" t="n"/>
@@ -5463,7 +5486,7 @@
       <c r="D108" s="7" t="n"/>
       <c r="E108" s="7" t="n"/>
       <c r="F108" s="8">
-        <f>IF(E108&lt;&gt;"",E108,IF(UPPER(TRIM(C108))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C108))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C108))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C108))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E108&lt;&gt;"",E108,IF(UPPER(TRIM(C108))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C108))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C108))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C108))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C108))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G108" s="7" t="n"/>
@@ -5485,7 +5508,7 @@
       <c r="D109" s="7" t="n"/>
       <c r="E109" s="7" t="n"/>
       <c r="F109" s="8">
-        <f>IF(E109&lt;&gt;"",E109,IF(UPPER(TRIM(C109))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C109))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C109))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C109))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E109&lt;&gt;"",E109,IF(UPPER(TRIM(C109))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C109))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C109))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C109))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C109))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G109" s="7" t="n"/>
@@ -5507,7 +5530,7 @@
       <c r="D110" s="7" t="n"/>
       <c r="E110" s="7" t="n"/>
       <c r="F110" s="8">
-        <f>IF(E110&lt;&gt;"",E110,IF(UPPER(TRIM(C110))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C110))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C110))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C110))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E110&lt;&gt;"",E110,IF(UPPER(TRIM(C110))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C110))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C110))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C110))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C110))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G110" s="7" t="n"/>
@@ -5529,7 +5552,7 @@
       <c r="D111" s="7" t="n"/>
       <c r="E111" s="7" t="n"/>
       <c r="F111" s="8">
-        <f>IF(E111&lt;&gt;"",E111,IF(UPPER(TRIM(C111))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C111))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C111))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C111))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E111&lt;&gt;"",E111,IF(UPPER(TRIM(C111))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C111))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C111))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C111))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C111))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G111" s="7" t="n"/>
@@ -5551,7 +5574,7 @@
       <c r="D112" s="7" t="n"/>
       <c r="E112" s="7" t="n"/>
       <c r="F112" s="8">
-        <f>IF(E112&lt;&gt;"",E112,IF(UPPER(TRIM(C112))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C112))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C112))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C112))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E112&lt;&gt;"",E112,IF(UPPER(TRIM(C112))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C112))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C112))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C112))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C112))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G112" s="7" t="n"/>
@@ -5573,7 +5596,7 @@
       <c r="D113" s="7" t="n"/>
       <c r="E113" s="7" t="n"/>
       <c r="F113" s="8">
-        <f>IF(E113&lt;&gt;"",E113,IF(UPPER(TRIM(C113))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C113))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C113))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C113))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E113&lt;&gt;"",E113,IF(UPPER(TRIM(C113))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C113))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C113))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C113))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C113))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G113" s="7" t="n"/>
@@ -5595,7 +5618,7 @@
       <c r="D114" s="7" t="n"/>
       <c r="E114" s="7" t="n"/>
       <c r="F114" s="8">
-        <f>IF(E114&lt;&gt;"",E114,IF(UPPER(TRIM(C114))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C114))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C114))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C114))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E114&lt;&gt;"",E114,IF(UPPER(TRIM(C114))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C114))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C114))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C114))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C114))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G114" s="7" t="n"/>
@@ -5617,7 +5640,7 @@
       <c r="D115" s="7" t="n"/>
       <c r="E115" s="7" t="n"/>
       <c r="F115" s="8">
-        <f>IF(E115&lt;&gt;"",E115,IF(UPPER(TRIM(C115))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C115))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C115))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C115))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E115&lt;&gt;"",E115,IF(UPPER(TRIM(C115))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C115))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C115))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C115))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C115))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G115" s="7" t="n"/>
@@ -5639,7 +5662,7 @@
       <c r="D116" s="7" t="n"/>
       <c r="E116" s="7" t="n"/>
       <c r="F116" s="8">
-        <f>IF(E116&lt;&gt;"",E116,IF(UPPER(TRIM(C116))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C116))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C116))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C116))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E116&lt;&gt;"",E116,IF(UPPER(TRIM(C116))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C116))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C116))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C116))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C116))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G116" s="7" t="n"/>
@@ -5661,7 +5684,7 @@
       <c r="D117" s="7" t="n"/>
       <c r="E117" s="7" t="n"/>
       <c r="F117" s="8">
-        <f>IF(E117&lt;&gt;"",E117,IF(UPPER(TRIM(C117))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C117))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C117))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C117))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E117&lt;&gt;"",E117,IF(UPPER(TRIM(C117))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C117))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C117))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C117))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C117))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G117" s="7" t="n"/>
@@ -5683,7 +5706,7 @@
       <c r="D118" s="7" t="n"/>
       <c r="E118" s="7" t="n"/>
       <c r="F118" s="8">
-        <f>IF(E118&lt;&gt;"",E118,IF(UPPER(TRIM(C118))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C118))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C118))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C118))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E118&lt;&gt;"",E118,IF(UPPER(TRIM(C118))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C118))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C118))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C118))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C118))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G118" s="7" t="n"/>
@@ -5705,7 +5728,7 @@
       <c r="D119" s="7" t="n"/>
       <c r="E119" s="7" t="n"/>
       <c r="F119" s="8">
-        <f>IF(E119&lt;&gt;"",E119,IF(UPPER(TRIM(C119))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C119))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C119))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C119))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E119&lt;&gt;"",E119,IF(UPPER(TRIM(C119))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C119))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C119))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C119))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C119))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G119" s="7" t="n"/>
@@ -5727,7 +5750,7 @@
       <c r="D120" s="7" t="n"/>
       <c r="E120" s="7" t="n"/>
       <c r="F120" s="8">
-        <f>IF(E120&lt;&gt;"",E120,IF(UPPER(TRIM(C120))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C120))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C120))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C120))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E120&lt;&gt;"",E120,IF(UPPER(TRIM(C120))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C120))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C120))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C120))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C120))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G120" s="7" t="n"/>
@@ -5749,7 +5772,7 @@
       <c r="D121" s="7" t="n"/>
       <c r="E121" s="7" t="n"/>
       <c r="F121" s="8">
-        <f>IF(E121&lt;&gt;"",E121,IF(UPPER(TRIM(C121))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C121))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C121))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C121))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E121&lt;&gt;"",E121,IF(UPPER(TRIM(C121))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C121))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C121))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C121))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C121))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G121" s="7" t="n"/>
@@ -5771,7 +5794,7 @@
       <c r="D122" s="7" t="n"/>
       <c r="E122" s="7" t="n"/>
       <c r="F122" s="8">
-        <f>IF(E122&lt;&gt;"",E122,IF(UPPER(TRIM(C122))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C122))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C122))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C122))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E122&lt;&gt;"",E122,IF(UPPER(TRIM(C122))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C122))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C122))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C122))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C122))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G122" s="7" t="n"/>
@@ -5793,7 +5816,7 @@
       <c r="D123" s="7" t="n"/>
       <c r="E123" s="7" t="n"/>
       <c r="F123" s="8">
-        <f>IF(E123&lt;&gt;"",E123,IF(UPPER(TRIM(C123))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C123))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C123))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C123))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E123&lt;&gt;"",E123,IF(UPPER(TRIM(C123))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C123))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C123))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C123))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C123))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G123" s="7" t="n"/>
@@ -5815,7 +5838,7 @@
       <c r="D124" s="7" t="n"/>
       <c r="E124" s="7" t="n"/>
       <c r="F124" s="8">
-        <f>IF(E124&lt;&gt;"",E124,IF(UPPER(TRIM(C124))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C124))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C124))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C124))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E124&lt;&gt;"",E124,IF(UPPER(TRIM(C124))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C124))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C124))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C124))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C124))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G124" s="7" t="n"/>
@@ -5837,7 +5860,7 @@
       <c r="D125" s="7" t="n"/>
       <c r="E125" s="7" t="n"/>
       <c r="F125" s="8">
-        <f>IF(E125&lt;&gt;"",E125,IF(UPPER(TRIM(C125))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C125))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C125))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C125))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E125&lt;&gt;"",E125,IF(UPPER(TRIM(C125))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C125))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C125))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C125))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C125))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G125" s="7" t="n"/>
@@ -5859,7 +5882,7 @@
       <c r="D126" s="7" t="n"/>
       <c r="E126" s="7" t="n"/>
       <c r="F126" s="8">
-        <f>IF(E126&lt;&gt;"",E126,IF(UPPER(TRIM(C126))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C126))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C126))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C126))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E126&lt;&gt;"",E126,IF(UPPER(TRIM(C126))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C126))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C126))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C126))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C126))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G126" s="7" t="n"/>
@@ -5881,7 +5904,7 @@
       <c r="D127" s="7" t="n"/>
       <c r="E127" s="7" t="n"/>
       <c r="F127" s="8">
-        <f>IF(E127&lt;&gt;"",E127,IF(UPPER(TRIM(C127))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C127))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C127))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C127))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E127&lt;&gt;"",E127,IF(UPPER(TRIM(C127))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C127))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C127))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C127))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C127))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G127" s="7" t="n"/>
@@ -5903,7 +5926,7 @@
       <c r="D128" s="7" t="n"/>
       <c r="E128" s="7" t="n"/>
       <c r="F128" s="8">
-        <f>IF(E128&lt;&gt;"",E128,IF(UPPER(TRIM(C128))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C128))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C128))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C128))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E128&lt;&gt;"",E128,IF(UPPER(TRIM(C128))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C128))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C128))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C128))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C128))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G128" s="7" t="n"/>
@@ -5925,7 +5948,7 @@
       <c r="D129" s="7" t="n"/>
       <c r="E129" s="7" t="n"/>
       <c r="F129" s="8">
-        <f>IF(E129&lt;&gt;"",E129,IF(UPPER(TRIM(C129))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C129))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C129))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C129))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E129&lt;&gt;"",E129,IF(UPPER(TRIM(C129))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C129))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C129))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C129))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C129))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G129" s="7" t="n"/>
@@ -5947,7 +5970,7 @@
       <c r="D130" s="7" t="n"/>
       <c r="E130" s="7" t="n"/>
       <c r="F130" s="8">
-        <f>IF(E130&lt;&gt;"",E130,IF(UPPER(TRIM(C130))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C130))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C130))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C130))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E130&lt;&gt;"",E130,IF(UPPER(TRIM(C130))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C130))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C130))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C130))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C130))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G130" s="7" t="n"/>
@@ -5969,7 +5992,7 @@
       <c r="D131" s="7" t="n"/>
       <c r="E131" s="7" t="n"/>
       <c r="F131" s="8">
-        <f>IF(E131&lt;&gt;"",E131,IF(UPPER(TRIM(C131))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C131))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C131))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C131))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E131&lt;&gt;"",E131,IF(UPPER(TRIM(C131))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C131))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C131))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C131))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C131))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G131" s="7" t="n"/>
@@ -5991,7 +6014,7 @@
       <c r="D132" s="7" t="n"/>
       <c r="E132" s="7" t="n"/>
       <c r="F132" s="8">
-        <f>IF(E132&lt;&gt;"",E132,IF(UPPER(TRIM(C132))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C132))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C132))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C132))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E132&lt;&gt;"",E132,IF(UPPER(TRIM(C132))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C132))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C132))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C132))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C132))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G132" s="7" t="n"/>
@@ -6013,7 +6036,7 @@
       <c r="D133" s="7" t="n"/>
       <c r="E133" s="7" t="n"/>
       <c r="F133" s="8">
-        <f>IF(E133&lt;&gt;"",E133,IF(UPPER(TRIM(C133))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C133))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C133))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C133))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E133&lt;&gt;"",E133,IF(UPPER(TRIM(C133))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C133))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C133))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C133))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C133))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G133" s="7" t="n"/>
@@ -6035,7 +6058,7 @@
       <c r="D134" s="7" t="n"/>
       <c r="E134" s="7" t="n"/>
       <c r="F134" s="8">
-        <f>IF(E134&lt;&gt;"",E134,IF(UPPER(TRIM(C134))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C134))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C134))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C134))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E134&lt;&gt;"",E134,IF(UPPER(TRIM(C134))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C134))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C134))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C134))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C134))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G134" s="7" t="n"/>
@@ -6057,7 +6080,7 @@
       <c r="D135" s="7" t="n"/>
       <c r="E135" s="7" t="n"/>
       <c r="F135" s="8">
-        <f>IF(E135&lt;&gt;"",E135,IF(UPPER(TRIM(C135))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C135))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C135))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C135))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E135&lt;&gt;"",E135,IF(UPPER(TRIM(C135))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C135))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C135))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C135))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C135))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G135" s="7" t="n"/>
@@ -6079,7 +6102,7 @@
       <c r="D136" s="7" t="n"/>
       <c r="E136" s="7" t="n"/>
       <c r="F136" s="8">
-        <f>IF(E136&lt;&gt;"",E136,IF(UPPER(TRIM(C136))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C136))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C136))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C136))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E136&lt;&gt;"",E136,IF(UPPER(TRIM(C136))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C136))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C136))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C136))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C136))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G136" s="7" t="n"/>
@@ -6101,7 +6124,7 @@
       <c r="D137" s="7" t="n"/>
       <c r="E137" s="7" t="n"/>
       <c r="F137" s="8">
-        <f>IF(E137&lt;&gt;"",E137,IF(UPPER(TRIM(C137))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C137))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C137))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C137))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E137&lt;&gt;"",E137,IF(UPPER(TRIM(C137))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C137))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C137))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C137))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C137))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G137" s="7" t="n"/>
@@ -6123,7 +6146,7 @@
       <c r="D138" s="7" t="n"/>
       <c r="E138" s="7" t="n"/>
       <c r="F138" s="8">
-        <f>IF(E138&lt;&gt;"",E138,IF(UPPER(TRIM(C138))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C138))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C138))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C138))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E138&lt;&gt;"",E138,IF(UPPER(TRIM(C138))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C138))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C138))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C138))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C138))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G138" s="7" t="n"/>
@@ -6145,7 +6168,7 @@
       <c r="D139" s="7" t="n"/>
       <c r="E139" s="7" t="n"/>
       <c r="F139" s="8">
-        <f>IF(E139&lt;&gt;"",E139,IF(UPPER(TRIM(C139))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C139))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C139))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C139))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E139&lt;&gt;"",E139,IF(UPPER(TRIM(C139))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C139))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C139))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C139))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C139))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G139" s="7" t="n"/>
@@ -6167,7 +6190,7 @@
       <c r="D140" s="7" t="n"/>
       <c r="E140" s="7" t="n"/>
       <c r="F140" s="8">
-        <f>IF(E140&lt;&gt;"",E140,IF(UPPER(TRIM(C140))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C140))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C140))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C140))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E140&lt;&gt;"",E140,IF(UPPER(TRIM(C140))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C140))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C140))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C140))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C140))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G140" s="7" t="n"/>
@@ -6189,7 +6212,7 @@
       <c r="D141" s="7" t="n"/>
       <c r="E141" s="7" t="n"/>
       <c r="F141" s="8">
-        <f>IF(E141&lt;&gt;"",E141,IF(UPPER(TRIM(C141))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C141))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C141))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C141))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E141&lt;&gt;"",E141,IF(UPPER(TRIM(C141))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C141))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C141))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C141))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C141))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G141" s="7" t="n"/>
@@ -6211,7 +6234,7 @@
       <c r="D142" s="7" t="n"/>
       <c r="E142" s="7" t="n"/>
       <c r="F142" s="8">
-        <f>IF(E142&lt;&gt;"",E142,IF(UPPER(TRIM(C142))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C142))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C142))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C142))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E142&lt;&gt;"",E142,IF(UPPER(TRIM(C142))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C142))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C142))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C142))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C142))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G142" s="7" t="n"/>
@@ -6233,7 +6256,7 @@
       <c r="D143" s="7" t="n"/>
       <c r="E143" s="7" t="n"/>
       <c r="F143" s="8">
-        <f>IF(E143&lt;&gt;"",E143,IF(UPPER(TRIM(C143))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C143))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C143))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C143))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E143&lt;&gt;"",E143,IF(UPPER(TRIM(C143))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C143))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C143))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C143))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C143))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G143" s="7" t="n"/>
@@ -6255,7 +6278,7 @@
       <c r="D144" s="7" t="n"/>
       <c r="E144" s="7" t="n"/>
       <c r="F144" s="8">
-        <f>IF(E144&lt;&gt;"",E144,IF(UPPER(TRIM(C144))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C144))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C144))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C144))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E144&lt;&gt;"",E144,IF(UPPER(TRIM(C144))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C144))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C144))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C144))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C144))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G144" s="7" t="n"/>
@@ -6277,7 +6300,7 @@
       <c r="D145" s="7" t="n"/>
       <c r="E145" s="7" t="n"/>
       <c r="F145" s="8">
-        <f>IF(E145&lt;&gt;"",E145,IF(UPPER(TRIM(C145))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C145))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C145))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C145))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E145&lt;&gt;"",E145,IF(UPPER(TRIM(C145))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C145))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C145))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C145))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C145))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G145" s="7" t="n"/>
@@ -6299,7 +6322,7 @@
       <c r="D146" s="7" t="n"/>
       <c r="E146" s="7" t="n"/>
       <c r="F146" s="8">
-        <f>IF(E146&lt;&gt;"",E146,IF(UPPER(TRIM(C146))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C146))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C146))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C146))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E146&lt;&gt;"",E146,IF(UPPER(TRIM(C146))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C146))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C146))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C146))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C146))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G146" s="7" t="n"/>
@@ -6321,7 +6344,7 @@
       <c r="D147" s="7" t="n"/>
       <c r="E147" s="7" t="n"/>
       <c r="F147" s="8">
-        <f>IF(E147&lt;&gt;"",E147,IF(UPPER(TRIM(C147))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C147))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C147))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C147))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E147&lt;&gt;"",E147,IF(UPPER(TRIM(C147))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C147))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C147))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C147))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C147))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G147" s="7" t="n"/>
@@ -6343,7 +6366,7 @@
       <c r="D148" s="7" t="n"/>
       <c r="E148" s="7" t="n"/>
       <c r="F148" s="8">
-        <f>IF(E148&lt;&gt;"",E148,IF(UPPER(TRIM(C148))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C148))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C148))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C148))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E148&lt;&gt;"",E148,IF(UPPER(TRIM(C148))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C148))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C148))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C148))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C148))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G148" s="7" t="n"/>
@@ -6365,7 +6388,7 @@
       <c r="D149" s="7" t="n"/>
       <c r="E149" s="7" t="n"/>
       <c r="F149" s="8">
-        <f>IF(E149&lt;&gt;"",E149,IF(UPPER(TRIM(C149))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C149))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C149))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C149))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E149&lt;&gt;"",E149,IF(UPPER(TRIM(C149))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C149))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C149))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C149))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C149))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G149" s="7" t="n"/>
@@ -6387,7 +6410,7 @@
       <c r="D150" s="7" t="n"/>
       <c r="E150" s="7" t="n"/>
       <c r="F150" s="8">
-        <f>IF(E150&lt;&gt;"",E150,IF(UPPER(TRIM(C150))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C150))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C150))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C150))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E150&lt;&gt;"",E150,IF(UPPER(TRIM(C150))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C150))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C150))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C150))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C150))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G150" s="7" t="n"/>
@@ -6409,7 +6432,7 @@
       <c r="D151" s="7" t="n"/>
       <c r="E151" s="7" t="n"/>
       <c r="F151" s="8">
-        <f>IF(E151&lt;&gt;"",E151,IF(UPPER(TRIM(C151))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C151))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C151))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C151))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E151&lt;&gt;"",E151,IF(UPPER(TRIM(C151))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C151))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C151))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C151))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C151))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G151" s="7" t="n"/>
@@ -6431,7 +6454,7 @@
       <c r="D152" s="7" t="n"/>
       <c r="E152" s="7" t="n"/>
       <c r="F152" s="8">
-        <f>IF(E152&lt;&gt;"",E152,IF(UPPER(TRIM(C152))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C152))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C152))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C152))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E152&lt;&gt;"",E152,IF(UPPER(TRIM(C152))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C152))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C152))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C152))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C152))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G152" s="7" t="n"/>
@@ -6453,7 +6476,7 @@
       <c r="D153" s="7" t="n"/>
       <c r="E153" s="7" t="n"/>
       <c r="F153" s="8">
-        <f>IF(E153&lt;&gt;"",E153,IF(UPPER(TRIM(C153))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C153))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C153))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C153))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E153&lt;&gt;"",E153,IF(UPPER(TRIM(C153))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C153))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C153))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C153))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C153))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G153" s="7" t="n"/>
@@ -6475,7 +6498,7 @@
       <c r="D154" s="7" t="n"/>
       <c r="E154" s="7" t="n"/>
       <c r="F154" s="8">
-        <f>IF(E154&lt;&gt;"",E154,IF(UPPER(TRIM(C154))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C154))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C154))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C154))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E154&lt;&gt;"",E154,IF(UPPER(TRIM(C154))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C154))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C154))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C154))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C154))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G154" s="7" t="n"/>
@@ -6497,7 +6520,7 @@
       <c r="D155" s="7" t="n"/>
       <c r="E155" s="7" t="n"/>
       <c r="F155" s="8">
-        <f>IF(E155&lt;&gt;"",E155,IF(UPPER(TRIM(C155))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C155))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C155))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C155))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E155&lt;&gt;"",E155,IF(UPPER(TRIM(C155))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C155))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C155))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C155))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C155))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G155" s="7" t="n"/>
@@ -6519,7 +6542,7 @@
       <c r="D156" s="7" t="n"/>
       <c r="E156" s="7" t="n"/>
       <c r="F156" s="8">
-        <f>IF(E156&lt;&gt;"",E156,IF(UPPER(TRIM(C156))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C156))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C156))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C156))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E156&lt;&gt;"",E156,IF(UPPER(TRIM(C156))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C156))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C156))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C156))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C156))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G156" s="7" t="n"/>
@@ -6541,7 +6564,7 @@
       <c r="D157" s="7" t="n"/>
       <c r="E157" s="7" t="n"/>
       <c r="F157" s="8">
-        <f>IF(E157&lt;&gt;"",E157,IF(UPPER(TRIM(C157))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C157))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C157))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C157))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E157&lt;&gt;"",E157,IF(UPPER(TRIM(C157))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C157))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C157))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C157))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C157))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G157" s="7" t="n"/>
@@ -6563,7 +6586,7 @@
       <c r="D158" s="7" t="n"/>
       <c r="E158" s="7" t="n"/>
       <c r="F158" s="8">
-        <f>IF(E158&lt;&gt;"",E158,IF(UPPER(TRIM(C158))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C158))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C158))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C158))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E158&lt;&gt;"",E158,IF(UPPER(TRIM(C158))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C158))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C158))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C158))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C158))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G158" s="7" t="n"/>
@@ -6585,7 +6608,7 @@
       <c r="D159" s="7" t="n"/>
       <c r="E159" s="7" t="n"/>
       <c r="F159" s="8">
-        <f>IF(E159&lt;&gt;"",E159,IF(UPPER(TRIM(C159))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C159))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C159))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C159))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E159&lt;&gt;"",E159,IF(UPPER(TRIM(C159))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C159))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C159))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C159))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C159))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G159" s="7" t="n"/>
@@ -6607,7 +6630,7 @@
       <c r="D160" s="7" t="n"/>
       <c r="E160" s="7" t="n"/>
       <c r="F160" s="8">
-        <f>IF(E160&lt;&gt;"",E160,IF(UPPER(TRIM(C160))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C160))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C160))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C160))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E160&lt;&gt;"",E160,IF(UPPER(TRIM(C160))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C160))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C160))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C160))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C160))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G160" s="7" t="n"/>
@@ -6629,7 +6652,7 @@
       <c r="D161" s="7" t="n"/>
       <c r="E161" s="7" t="n"/>
       <c r="F161" s="8">
-        <f>IF(E161&lt;&gt;"",E161,IF(UPPER(TRIM(C161))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C161))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C161))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C161))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E161&lt;&gt;"",E161,IF(UPPER(TRIM(C161))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C161))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C161))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C161))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C161))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G161" s="7" t="n"/>
@@ -6651,7 +6674,7 @@
       <c r="D162" s="7" t="n"/>
       <c r="E162" s="7" t="n"/>
       <c r="F162" s="8">
-        <f>IF(E162&lt;&gt;"",E162,IF(UPPER(TRIM(C162))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C162))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C162))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C162))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E162&lt;&gt;"",E162,IF(UPPER(TRIM(C162))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C162))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C162))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C162))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C162))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G162" s="7" t="n"/>
@@ -6673,7 +6696,7 @@
       <c r="D163" s="7" t="n"/>
       <c r="E163" s="7" t="n"/>
       <c r="F163" s="8">
-        <f>IF(E163&lt;&gt;"",E163,IF(UPPER(TRIM(C163))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C163))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C163))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C163))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E163&lt;&gt;"",E163,IF(UPPER(TRIM(C163))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C163))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C163))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C163))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C163))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G163" s="7" t="n"/>
@@ -6695,7 +6718,7 @@
       <c r="D164" s="7" t="n"/>
       <c r="E164" s="7" t="n"/>
       <c r="F164" s="8">
-        <f>IF(E164&lt;&gt;"",E164,IF(UPPER(TRIM(C164))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C164))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C164))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C164))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E164&lt;&gt;"",E164,IF(UPPER(TRIM(C164))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C164))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C164))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C164))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C164))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G164" s="7" t="n"/>
@@ -6717,7 +6740,7 @@
       <c r="D165" s="7" t="n"/>
       <c r="E165" s="7" t="n"/>
       <c r="F165" s="8">
-        <f>IF(E165&lt;&gt;"",E165,IF(UPPER(TRIM(C165))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C165))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C165))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C165))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E165&lt;&gt;"",E165,IF(UPPER(TRIM(C165))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C165))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C165))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C165))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C165))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G165" s="7" t="n"/>
@@ -6739,7 +6762,7 @@
       <c r="D166" s="7" t="n"/>
       <c r="E166" s="7" t="n"/>
       <c r="F166" s="8">
-        <f>IF(E166&lt;&gt;"",E166,IF(UPPER(TRIM(C166))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C166))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C166))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C166))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E166&lt;&gt;"",E166,IF(UPPER(TRIM(C166))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C166))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C166))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C166))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C166))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G166" s="7" t="n"/>
@@ -6761,7 +6784,7 @@
       <c r="D167" s="7" t="n"/>
       <c r="E167" s="7" t="n"/>
       <c r="F167" s="8">
-        <f>IF(E167&lt;&gt;"",E167,IF(UPPER(TRIM(C167))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C167))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C167))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C167))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E167&lt;&gt;"",E167,IF(UPPER(TRIM(C167))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C167))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C167))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C167))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C167))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G167" s="7" t="n"/>
@@ -6783,7 +6806,7 @@
       <c r="D168" s="7" t="n"/>
       <c r="E168" s="7" t="n"/>
       <c r="F168" s="8">
-        <f>IF(E168&lt;&gt;"",E168,IF(UPPER(TRIM(C168))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C168))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C168))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C168))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E168&lt;&gt;"",E168,IF(UPPER(TRIM(C168))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C168))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C168))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C168))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C168))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G168" s="7" t="n"/>
@@ -6805,7 +6828,7 @@
       <c r="D169" s="7" t="n"/>
       <c r="E169" s="7" t="n"/>
       <c r="F169" s="8">
-        <f>IF(E169&lt;&gt;"",E169,IF(UPPER(TRIM(C169))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C169))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C169))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C169))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E169&lt;&gt;"",E169,IF(UPPER(TRIM(C169))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C169))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C169))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C169))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C169))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G169" s="7" t="n"/>
@@ -6827,7 +6850,7 @@
       <c r="D170" s="7" t="n"/>
       <c r="E170" s="7" t="n"/>
       <c r="F170" s="8">
-        <f>IF(E170&lt;&gt;"",E170,IF(UPPER(TRIM(C170))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C170))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C170))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C170))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E170&lt;&gt;"",E170,IF(UPPER(TRIM(C170))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C170))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C170))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C170))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C170))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G170" s="7" t="n"/>
@@ -6849,7 +6872,7 @@
       <c r="D171" s="7" t="n"/>
       <c r="E171" s="7" t="n"/>
       <c r="F171" s="8">
-        <f>IF(E171&lt;&gt;"",E171,IF(UPPER(TRIM(C171))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C171))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C171))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C171))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E171&lt;&gt;"",E171,IF(UPPER(TRIM(C171))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C171))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C171))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C171))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C171))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G171" s="7" t="n"/>
@@ -6871,7 +6894,7 @@
       <c r="D172" s="7" t="n"/>
       <c r="E172" s="7" t="n"/>
       <c r="F172" s="8">
-        <f>IF(E172&lt;&gt;"",E172,IF(UPPER(TRIM(C172))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C172))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C172))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C172))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E172&lt;&gt;"",E172,IF(UPPER(TRIM(C172))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C172))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C172))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C172))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C172))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G172" s="7" t="n"/>
@@ -6893,7 +6916,7 @@
       <c r="D173" s="7" t="n"/>
       <c r="E173" s="7" t="n"/>
       <c r="F173" s="8">
-        <f>IF(E173&lt;&gt;"",E173,IF(UPPER(TRIM(C173))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C173))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C173))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C173))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E173&lt;&gt;"",E173,IF(UPPER(TRIM(C173))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C173))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C173))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C173))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C173))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G173" s="7" t="n"/>
@@ -6915,7 +6938,7 @@
       <c r="D174" s="7" t="n"/>
       <c r="E174" s="7" t="n"/>
       <c r="F174" s="8">
-        <f>IF(E174&lt;&gt;"",E174,IF(UPPER(TRIM(C174))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C174))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C174))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C174))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E174&lt;&gt;"",E174,IF(UPPER(TRIM(C174))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C174))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C174))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C174))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C174))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G174" s="7" t="n"/>
@@ -6937,7 +6960,7 @@
       <c r="D175" s="7" t="n"/>
       <c r="E175" s="7" t="n"/>
       <c r="F175" s="8">
-        <f>IF(E175&lt;&gt;"",E175,IF(UPPER(TRIM(C175))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C175))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C175))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C175))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E175&lt;&gt;"",E175,IF(UPPER(TRIM(C175))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C175))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C175))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C175))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C175))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G175" s="7" t="n"/>
@@ -6959,7 +6982,7 @@
       <c r="D176" s="7" t="n"/>
       <c r="E176" s="7" t="n"/>
       <c r="F176" s="8">
-        <f>IF(E176&lt;&gt;"",E176,IF(UPPER(TRIM(C176))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C176))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C176))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C176))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E176&lt;&gt;"",E176,IF(UPPER(TRIM(C176))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C176))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C176))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C176))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C176))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G176" s="7" t="n"/>
@@ -6981,7 +7004,7 @@
       <c r="D177" s="7" t="n"/>
       <c r="E177" s="7" t="n"/>
       <c r="F177" s="8">
-        <f>IF(E177&lt;&gt;"",E177,IF(UPPER(TRIM(C177))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C177))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C177))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C177))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E177&lt;&gt;"",E177,IF(UPPER(TRIM(C177))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C177))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C177))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C177))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C177))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G177" s="7" t="n"/>
@@ -7003,7 +7026,7 @@
       <c r="D178" s="7" t="n"/>
       <c r="E178" s="7" t="n"/>
       <c r="F178" s="8">
-        <f>IF(E178&lt;&gt;"",E178,IF(UPPER(TRIM(C178))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C178))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C178))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C178))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E178&lt;&gt;"",E178,IF(UPPER(TRIM(C178))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C178))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C178))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C178))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C178))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G178" s="7" t="n"/>
@@ -7025,7 +7048,7 @@
       <c r="D179" s="7" t="n"/>
       <c r="E179" s="7" t="n"/>
       <c r="F179" s="8">
-        <f>IF(E179&lt;&gt;"",E179,IF(UPPER(TRIM(C179))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C179))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C179))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C179))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E179&lt;&gt;"",E179,IF(UPPER(TRIM(C179))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C179))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C179))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C179))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C179))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G179" s="7" t="n"/>
@@ -7047,7 +7070,7 @@
       <c r="D180" s="7" t="n"/>
       <c r="E180" s="7" t="n"/>
       <c r="F180" s="8">
-        <f>IF(E180&lt;&gt;"",E180,IF(UPPER(TRIM(C180))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C180))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C180))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C180))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E180&lt;&gt;"",E180,IF(UPPER(TRIM(C180))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C180))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C180))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C180))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C180))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G180" s="7" t="n"/>
@@ -7069,7 +7092,7 @@
       <c r="D181" s="7" t="n"/>
       <c r="E181" s="7" t="n"/>
       <c r="F181" s="8">
-        <f>IF(E181&lt;&gt;"",E181,IF(UPPER(TRIM(C181))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C181))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C181))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C181))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E181&lt;&gt;"",E181,IF(UPPER(TRIM(C181))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C181))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C181))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C181))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C181))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G181" s="7" t="n"/>
@@ -7091,7 +7114,7 @@
       <c r="D182" s="7" t="n"/>
       <c r="E182" s="7" t="n"/>
       <c r="F182" s="8">
-        <f>IF(E182&lt;&gt;"",E182,IF(UPPER(TRIM(C182))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C182))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C182))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C182))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E182&lt;&gt;"",E182,IF(UPPER(TRIM(C182))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C182))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C182))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C182))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C182))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G182" s="7" t="n"/>
@@ -7113,7 +7136,7 @@
       <c r="D183" s="7" t="n"/>
       <c r="E183" s="7" t="n"/>
       <c r="F183" s="8">
-        <f>IF(E183&lt;&gt;"",E183,IF(UPPER(TRIM(C183))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C183))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C183))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C183))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E183&lt;&gt;"",E183,IF(UPPER(TRIM(C183))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C183))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C183))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C183))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C183))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G183" s="7" t="n"/>
@@ -7135,7 +7158,7 @@
       <c r="D184" s="7" t="n"/>
       <c r="E184" s="7" t="n"/>
       <c r="F184" s="8">
-        <f>IF(E184&lt;&gt;"",E184,IF(UPPER(TRIM(C184))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C184))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C184))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C184))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E184&lt;&gt;"",E184,IF(UPPER(TRIM(C184))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C184))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C184))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C184))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C184))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G184" s="7" t="n"/>
@@ -7157,7 +7180,7 @@
       <c r="D185" s="7" t="n"/>
       <c r="E185" s="7" t="n"/>
       <c r="F185" s="8">
-        <f>IF(E185&lt;&gt;"",E185,IF(UPPER(TRIM(C185))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C185))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C185))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C185))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E185&lt;&gt;"",E185,IF(UPPER(TRIM(C185))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C185))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C185))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C185))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C185))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G185" s="7" t="n"/>
@@ -7179,7 +7202,7 @@
       <c r="D186" s="7" t="n"/>
       <c r="E186" s="7" t="n"/>
       <c r="F186" s="8">
-        <f>IF(E186&lt;&gt;"",E186,IF(UPPER(TRIM(C186))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C186))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C186))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C186))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E186&lt;&gt;"",E186,IF(UPPER(TRIM(C186))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C186))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C186))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C186))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C186))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G186" s="7" t="n"/>
@@ -7201,7 +7224,7 @@
       <c r="D187" s="7" t="n"/>
       <c r="E187" s="7" t="n"/>
       <c r="F187" s="8">
-        <f>IF(E187&lt;&gt;"",E187,IF(UPPER(TRIM(C187))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C187))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C187))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C187))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E187&lt;&gt;"",E187,IF(UPPER(TRIM(C187))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C187))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C187))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C187))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C187))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G187" s="7" t="n"/>
@@ -7223,7 +7246,7 @@
       <c r="D188" s="7" t="n"/>
       <c r="E188" s="7" t="n"/>
       <c r="F188" s="8">
-        <f>IF(E188&lt;&gt;"",E188,IF(UPPER(TRIM(C188))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C188))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C188))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C188))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E188&lt;&gt;"",E188,IF(UPPER(TRIM(C188))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C188))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C188))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C188))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C188))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G188" s="7" t="n"/>
@@ -7245,7 +7268,7 @@
       <c r="D189" s="7" t="n"/>
       <c r="E189" s="7" t="n"/>
       <c r="F189" s="8">
-        <f>IF(E189&lt;&gt;"",E189,IF(UPPER(TRIM(C189))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C189))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C189))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C189))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E189&lt;&gt;"",E189,IF(UPPER(TRIM(C189))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C189))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C189))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C189))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C189))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G189" s="7" t="n"/>
@@ -7267,7 +7290,7 @@
       <c r="D190" s="7" t="n"/>
       <c r="E190" s="7" t="n"/>
       <c r="F190" s="8">
-        <f>IF(E190&lt;&gt;"",E190,IF(UPPER(TRIM(C190))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C190))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C190))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C190))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E190&lt;&gt;"",E190,IF(UPPER(TRIM(C190))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C190))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C190))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C190))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C190))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G190" s="7" t="n"/>
@@ -7289,7 +7312,7 @@
       <c r="D191" s="7" t="n"/>
       <c r="E191" s="7" t="n"/>
       <c r="F191" s="8">
-        <f>IF(E191&lt;&gt;"",E191,IF(UPPER(TRIM(C191))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C191))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C191))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C191))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E191&lt;&gt;"",E191,IF(UPPER(TRIM(C191))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C191))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C191))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C191))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C191))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G191" s="7" t="n"/>
@@ -7311,7 +7334,7 @@
       <c r="D192" s="7" t="n"/>
       <c r="E192" s="7" t="n"/>
       <c r="F192" s="8">
-        <f>IF(E192&lt;&gt;"",E192,IF(UPPER(TRIM(C192))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C192))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C192))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C192))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E192&lt;&gt;"",E192,IF(UPPER(TRIM(C192))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C192))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C192))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C192))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C192))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G192" s="7" t="n"/>
@@ -7333,7 +7356,7 @@
       <c r="D193" s="7" t="n"/>
       <c r="E193" s="7" t="n"/>
       <c r="F193" s="8">
-        <f>IF(E193&lt;&gt;"",E193,IF(UPPER(TRIM(C193))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C193))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C193))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C193))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E193&lt;&gt;"",E193,IF(UPPER(TRIM(C193))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C193))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C193))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C193))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C193))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G193" s="7" t="n"/>
@@ -7355,7 +7378,7 @@
       <c r="D194" s="7" t="n"/>
       <c r="E194" s="7" t="n"/>
       <c r="F194" s="8">
-        <f>IF(E194&lt;&gt;"",E194,IF(UPPER(TRIM(C194))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C194))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C194))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C194))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E194&lt;&gt;"",E194,IF(UPPER(TRIM(C194))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C194))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C194))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C194))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C194))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G194" s="7" t="n"/>
@@ -7377,7 +7400,7 @@
       <c r="D195" s="7" t="n"/>
       <c r="E195" s="7" t="n"/>
       <c r="F195" s="8">
-        <f>IF(E195&lt;&gt;"",E195,IF(UPPER(TRIM(C195))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C195))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C195))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C195))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E195&lt;&gt;"",E195,IF(UPPER(TRIM(C195))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C195))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C195))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C195))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C195))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G195" s="7" t="n"/>
@@ -7399,7 +7422,7 @@
       <c r="D196" s="7" t="n"/>
       <c r="E196" s="7" t="n"/>
       <c r="F196" s="8">
-        <f>IF(E196&lt;&gt;"",E196,IF(UPPER(TRIM(C196))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C196))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C196))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C196))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E196&lt;&gt;"",E196,IF(UPPER(TRIM(C196))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C196))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C196))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C196))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C196))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G196" s="7" t="n"/>
@@ -7421,7 +7444,7 @@
       <c r="D197" s="7" t="n"/>
       <c r="E197" s="7" t="n"/>
       <c r="F197" s="8">
-        <f>IF(E197&lt;&gt;"",E197,IF(UPPER(TRIM(C197))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C197))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C197))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C197))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E197&lt;&gt;"",E197,IF(UPPER(TRIM(C197))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C197))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C197))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C197))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C197))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G197" s="7" t="n"/>
@@ -7443,7 +7466,7 @@
       <c r="D198" s="7" t="n"/>
       <c r="E198" s="7" t="n"/>
       <c r="F198" s="8">
-        <f>IF(E198&lt;&gt;"",E198,IF(UPPER(TRIM(C198))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C198))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C198))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C198))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E198&lt;&gt;"",E198,IF(UPPER(TRIM(C198))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C198))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C198))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C198))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C198))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G198" s="7" t="n"/>
@@ -7465,7 +7488,7 @@
       <c r="D199" s="7" t="n"/>
       <c r="E199" s="7" t="n"/>
       <c r="F199" s="8">
-        <f>IF(E199&lt;&gt;"",E199,IF(UPPER(TRIM(C199))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C199))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C199))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C199))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E199&lt;&gt;"",E199,IF(UPPER(TRIM(C199))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C199))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C199))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C199))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C199))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G199" s="7" t="n"/>
@@ -7487,7 +7510,7 @@
       <c r="D200" s="7" t="n"/>
       <c r="E200" s="7" t="n"/>
       <c r="F200" s="8">
-        <f>IF(E200&lt;&gt;"",E200,IF(UPPER(TRIM(C200))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C200))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C200))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C200))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E200&lt;&gt;"",E200,IF(UPPER(TRIM(C200))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C200))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C200))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C200))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C200))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G200" s="7" t="n"/>
@@ -7509,7 +7532,7 @@
       <c r="D201" s="7" t="n"/>
       <c r="E201" s="7" t="n"/>
       <c r="F201" s="8">
-        <f>IF(E201&lt;&gt;"",E201,IF(UPPER(TRIM(C201))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C201))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C201))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C201))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E201&lt;&gt;"",E201,IF(UPPER(TRIM(C201))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C201))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C201))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C201))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C201))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G201" s="7" t="n"/>
@@ -7531,7 +7554,7 @@
       <c r="D202" s="7" t="n"/>
       <c r="E202" s="7" t="n"/>
       <c r="F202" s="8">
-        <f>IF(E202&lt;&gt;"",E202,IF(UPPER(TRIM(C202))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C202))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C202))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C202))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E202&lt;&gt;"",E202,IF(UPPER(TRIM(C202))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C202))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C202))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C202))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C202))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G202" s="7" t="n"/>
@@ -7553,7 +7576,7 @@
       <c r="D203" s="7" t="n"/>
       <c r="E203" s="7" t="n"/>
       <c r="F203" s="8">
-        <f>IF(E203&lt;&gt;"",E203,IF(UPPER(TRIM(C203))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C203))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C203))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C203))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E203&lt;&gt;"",E203,IF(UPPER(TRIM(C203))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C203))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C203))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C203))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C203))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G203" s="7" t="n"/>
@@ -7575,7 +7598,7 @@
       <c r="D204" s="7" t="n"/>
       <c r="E204" s="7" t="n"/>
       <c r="F204" s="8">
-        <f>IF(E204&lt;&gt;"",E204,IF(UPPER(TRIM(C204))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C204))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C204))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C204))="GRASS",Inputs!$B$12,Inputs!$B$13)))))</f>
+        <f>IF(E204&lt;&gt;"",E204,IF(UPPER(TRIM(C204))="BASIN",IF(UPPER(TRIM(Inputs!$B$52))="YES",Inputs!$B$12,0),IF(UPPER(TRIM(C204))="ROOF",Inputs!$B$10,IF(UPPER(TRIM(C204))="PAVAGE",Inputs!$B$58,IF(UPPER(TRIM(C204))="TRESFOND",Inputs!$B$11,IF(UPPER(TRIM(C204))="GRASS",Inputs!$B$12,Inputs!$B$13))))))</f>
         <v/>
       </c>
       <c r="G204" s="7" t="n"/>
@@ -7969,7 +7992,7 @@
       </c>
       <c r="AC4" s="7" t="n"/>
       <c r="AD4" s="8">
-        <f>IF(A4="","",IF(AC4&lt;&gt;"",AC4,IF(E4="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E4,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A4="","",IF(AC4&lt;&gt;"",AC4,IF(E4="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E4,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B4))="SWALE",UPPER(TRIM(AI4))="PIPE"),AND(UPPER(TRIM(B4))="TRENCH",UPPER(TRIM(AI4))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE4" s="8">
@@ -8121,7 +8144,7 @@
       </c>
       <c r="AC5" s="7" t="n"/>
       <c r="AD5" s="8">
-        <f>IF(A5="","",IF(AC5&lt;&gt;"",AC5,IF(E5="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E5,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A5="","",IF(AC5&lt;&gt;"",AC5,IF(E5="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E5,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B5))="SWALE",UPPER(TRIM(AI5))="PIPE"),AND(UPPER(TRIM(B5))="TRENCH",UPPER(TRIM(AI5))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE5" s="8">
@@ -8262,7 +8285,7 @@
       </c>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="8">
-        <f>IF(A6="","",IF(AC6&lt;&gt;"",AC6,IF(E6="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E6,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A6="","",IF(AC6&lt;&gt;"",AC6,IF(E6="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E6,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B6))="SWALE",UPPER(TRIM(AI6))="PIPE"),AND(UPPER(TRIM(B6))="TRENCH",UPPER(TRIM(AI6))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE6" s="8">
@@ -8408,7 +8431,7 @@
       </c>
       <c r="AC7" s="7" t="n"/>
       <c r="AD7" s="8">
-        <f>IF(A7="","",IF(AC7&lt;&gt;"",AC7,IF(E7="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E7,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A7="","",IF(AC7&lt;&gt;"",AC7,IF(E7="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E7,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B7))="SWALE",UPPER(TRIM(AI7))="PIPE"),AND(UPPER(TRIM(B7))="TRENCH",UPPER(TRIM(AI7))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE7" s="8">
@@ -8554,7 +8577,7 @@
       </c>
       <c r="AC8" s="7" t="n"/>
       <c r="AD8" s="8">
-        <f>IF(A8="","",IF(AC8&lt;&gt;"",AC8,IF(E8="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E8,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A8="","",IF(AC8&lt;&gt;"",AC8,IF(E8="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E8,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B8))="SWALE",UPPER(TRIM(AI8))="PIPE"),AND(UPPER(TRIM(B8))="TRENCH",UPPER(TRIM(AI8))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE8" s="8">
@@ -8696,7 +8719,7 @@
       </c>
       <c r="AC9" s="7" t="n"/>
       <c r="AD9" s="8">
-        <f>IF(A9="","",IF(AC9&lt;&gt;"",AC9,IF(E9="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E9,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A9="","",IF(AC9&lt;&gt;"",AC9,IF(E9="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E9,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B9))="SWALE",UPPER(TRIM(AI9))="PIPE"),AND(UPPER(TRIM(B9))="TRENCH",UPPER(TRIM(AI9))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE9" s="8">
@@ -8842,7 +8865,7 @@
       </c>
       <c r="AC10" s="7" t="n"/>
       <c r="AD10" s="8">
-        <f>IF(A10="","",IF(AC10&lt;&gt;"",AC10,IF(E10="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E10,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A10="","",IF(AC10&lt;&gt;"",AC10,IF(E10="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E10,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B10))="SWALE",UPPER(TRIM(AI10))="PIPE"),AND(UPPER(TRIM(B10))="TRENCH",UPPER(TRIM(AI10))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE10" s="8">
@@ -8984,7 +9007,7 @@
       </c>
       <c r="AC11" s="7" t="n"/>
       <c r="AD11" s="8">
-        <f>IF(A11="","",IF(AC11&lt;&gt;"",AC11,IF(E11="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E11,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A11="","",IF(AC11&lt;&gt;"",AC11,IF(E11="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E11,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B11))="SWALE",UPPER(TRIM(AI11))="PIPE"),AND(UPPER(TRIM(B11))="TRENCH",UPPER(TRIM(AI11))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE11" s="8">
@@ -9130,7 +9153,7 @@
       </c>
       <c r="AC12" s="7" t="n"/>
       <c r="AD12" s="8">
-        <f>IF(A12="","",IF(AC12&lt;&gt;"",AC12,IF(E12="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E12,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A12="","",IF(AC12&lt;&gt;"",AC12,IF(E12="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E12,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B12))="SWALE",UPPER(TRIM(AI12))="PIPE"),AND(UPPER(TRIM(B12))="TRENCH",UPPER(TRIM(AI12))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE12" s="8">
@@ -9239,7 +9262,7 @@
       <c r="AB13" s="4" t="n"/>
       <c r="AC13" s="7" t="n"/>
       <c r="AD13" s="8">
-        <f>IF(A13="","",IF(AC13&lt;&gt;"",AC13,IF(E13="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E13,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A13="","",IF(AC13&lt;&gt;"",AC13,IF(E13="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E13,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B13))="SWALE",UPPER(TRIM(AI13))="PIPE"),AND(UPPER(TRIM(B13))="TRENCH",UPPER(TRIM(AI13))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE13" s="8">
@@ -9376,7 +9399,7 @@
       </c>
       <c r="AC14" s="7" t="n"/>
       <c r="AD14" s="8">
-        <f>IF(A14="","",IF(AC14&lt;&gt;"",AC14,IF(E14="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E14,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A14="","",IF(AC14&lt;&gt;"",AC14,IF(E14="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E14,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B14))="SWALE",UPPER(TRIM(AI14))="PIPE"),AND(UPPER(TRIM(B14))="TRENCH",UPPER(TRIM(AI14))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE14" s="8">
@@ -9513,7 +9536,7 @@
       </c>
       <c r="AC15" s="7" t="n"/>
       <c r="AD15" s="8">
-        <f>IF(A15="","",IF(AC15&lt;&gt;"",AC15,IF(E15="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E15,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A15="","",IF(AC15&lt;&gt;"",AC15,IF(E15="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E15,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B15))="SWALE",UPPER(TRIM(AI15))="PIPE"),AND(UPPER(TRIM(B15))="TRENCH",UPPER(TRIM(AI15))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE15" s="8">
@@ -9622,7 +9645,7 @@
       <c r="AB16" s="4" t="n"/>
       <c r="AC16" s="7" t="n"/>
       <c r="AD16" s="8">
-        <f>IF(A16="","",IF(AC16&lt;&gt;"",AC16,IF(E16="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E16,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A16="","",IF(AC16&lt;&gt;"",AC16,IF(E16="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E16,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B16))="SWALE",UPPER(TRIM(AI16))="PIPE"),AND(UPPER(TRIM(B16))="TRENCH",UPPER(TRIM(AI16))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE16" s="8">
@@ -9731,7 +9754,7 @@
       <c r="AB17" s="4" t="n"/>
       <c r="AC17" s="7" t="n"/>
       <c r="AD17" s="8">
-        <f>IF(A17="","",IF(AC17&lt;&gt;"",AC17,IF(E17="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E17,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A17="","",IF(AC17&lt;&gt;"",AC17,IF(E17="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E17,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B17))="SWALE",UPPER(TRIM(AI17))="PIPE"),AND(UPPER(TRIM(B17))="TRENCH",UPPER(TRIM(AI17))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE17" s="8">
@@ -9840,7 +9863,7 @@
       <c r="AB18" s="4" t="n"/>
       <c r="AC18" s="7" t="n"/>
       <c r="AD18" s="8">
-        <f>IF(A18="","",IF(AC18&lt;&gt;"",AC18,IF(E18="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E18,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A18="","",IF(AC18&lt;&gt;"",AC18,IF(E18="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E18,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B18))="SWALE",UPPER(TRIM(AI18))="PIPE"),AND(UPPER(TRIM(B18))="TRENCH",UPPER(TRIM(AI18))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE18" s="8">
@@ -9949,7 +9972,7 @@
       <c r="AB19" s="4" t="n"/>
       <c r="AC19" s="7" t="n"/>
       <c r="AD19" s="8">
-        <f>IF(A19="","",IF(AC19&lt;&gt;"",AC19,IF(E19="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E19,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A19="","",IF(AC19&lt;&gt;"",AC19,IF(E19="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E19,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B19))="SWALE",UPPER(TRIM(AI19))="PIPE"),AND(UPPER(TRIM(B19))="TRENCH",UPPER(TRIM(AI19))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE19" s="8">
@@ -10058,7 +10081,7 @@
       <c r="AB20" s="4" t="n"/>
       <c r="AC20" s="7" t="n"/>
       <c r="AD20" s="8">
-        <f>IF(A20="","",IF(AC20&lt;&gt;"",AC20,IF(E20="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E20,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A20="","",IF(AC20&lt;&gt;"",AC20,IF(E20="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E20,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B20))="SWALE",UPPER(TRIM(AI20))="PIPE"),AND(UPPER(TRIM(B20))="TRENCH",UPPER(TRIM(AI20))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE20" s="8">
@@ -10169,7 +10192,7 @@
       <c r="AB21" s="4" t="n"/>
       <c r="AC21" s="7" t="n"/>
       <c r="AD21" s="8">
-        <f>IF(A21="","",IF(AC21&lt;&gt;"",AC21,IF(E21="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E21,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A21="","",IF(AC21&lt;&gt;"",AC21,IF(E21="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E21,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE21" s="8">
@@ -10280,7 +10303,7 @@
       <c r="AB22" s="4" t="n"/>
       <c r="AC22" s="7" t="n"/>
       <c r="AD22" s="8">
-        <f>IF(A22="","",IF(AC22&lt;&gt;"",AC22,IF(E22="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E22,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A22="","",IF(AC22&lt;&gt;"",AC22,IF(E22="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E22,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE22" s="8">
@@ -10391,7 +10414,7 @@
       <c r="AB23" s="4" t="n"/>
       <c r="AC23" s="7" t="n"/>
       <c r="AD23" s="8">
-        <f>IF(A23="","",IF(AC23&lt;&gt;"",AC23,IF(E23="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E23,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A23="","",IF(AC23&lt;&gt;"",AC23,IF(E23="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E23,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE23" s="8">
@@ -10502,7 +10525,7 @@
       <c r="AB24" s="4" t="n"/>
       <c r="AC24" s="7" t="n"/>
       <c r="AD24" s="8">
-        <f>IF(A24="","",IF(AC24&lt;&gt;"",AC24,IF(E24="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E24,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A24="","",IF(AC24&lt;&gt;"",AC24,IF(E24="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E24,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE24" s="8">
@@ -10613,7 +10636,7 @@
       <c r="AB25" s="4" t="n"/>
       <c r="AC25" s="7" t="n"/>
       <c r="AD25" s="8">
-        <f>IF(A25="","",IF(AC25&lt;&gt;"",AC25,IF(E25="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E25,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A25="","",IF(AC25&lt;&gt;"",AC25,IF(E25="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E25,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE25" s="8">
@@ -10724,7 +10747,7 @@
       <c r="AB26" s="4" t="n"/>
       <c r="AC26" s="7" t="n"/>
       <c r="AD26" s="8">
-        <f>IF(A26="","",IF(AC26&lt;&gt;"",AC26,IF(E26="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E26,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A26="","",IF(AC26&lt;&gt;"",AC26,IF(E26="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E26,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B26))="SWALE",UPPER(TRIM(AI26))="PIPE"),AND(UPPER(TRIM(B26))="TRENCH",UPPER(TRIM(AI26))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE26" s="8">
@@ -10835,7 +10858,7 @@
       <c r="AB27" s="4" t="n"/>
       <c r="AC27" s="7" t="n"/>
       <c r="AD27" s="8">
-        <f>IF(A27="","",IF(AC27&lt;&gt;"",AC27,IF(E27="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E27,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A27="","",IF(AC27&lt;&gt;"",AC27,IF(E27="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E27,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B27))="SWALE",UPPER(TRIM(AI27))="PIPE"),AND(UPPER(TRIM(B27))="TRENCH",UPPER(TRIM(AI27))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE27" s="8">
@@ -10946,7 +10969,7 @@
       <c r="AB28" s="4" t="n"/>
       <c r="AC28" s="7" t="n"/>
       <c r="AD28" s="8">
-        <f>IF(A28="","",IF(AC28&lt;&gt;"",AC28,IF(E28="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E28,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A28="","",IF(AC28&lt;&gt;"",AC28,IF(E28="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E28,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B28))="SWALE",UPPER(TRIM(AI28))="PIPE"),AND(UPPER(TRIM(B28))="TRENCH",UPPER(TRIM(AI28))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE28" s="8">
@@ -11057,7 +11080,7 @@
       <c r="AB29" s="4" t="n"/>
       <c r="AC29" s="7" t="n"/>
       <c r="AD29" s="8">
-        <f>IF(A29="","",IF(AC29&lt;&gt;"",AC29,IF(E29="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E29,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A29="","",IF(AC29&lt;&gt;"",AC29,IF(E29="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E29,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B29))="SWALE",UPPER(TRIM(AI29))="PIPE"),AND(UPPER(TRIM(B29))="TRENCH",UPPER(TRIM(AI29))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE29" s="8">
@@ -11168,7 +11191,7 @@
       <c r="AB30" s="4" t="n"/>
       <c r="AC30" s="7" t="n"/>
       <c r="AD30" s="8">
-        <f>IF(A30="","",IF(AC30&lt;&gt;"",AC30,IF(E30="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E30,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A30="","",IF(AC30&lt;&gt;"",AC30,IF(E30="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E30,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B30))="SWALE",UPPER(TRIM(AI30))="PIPE"),AND(UPPER(TRIM(B30))="TRENCH",UPPER(TRIM(AI30))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE30" s="8">
@@ -11279,7 +11302,7 @@
       <c r="AB31" s="4" t="n"/>
       <c r="AC31" s="7" t="n"/>
       <c r="AD31" s="8">
-        <f>IF(A31="","",IF(AC31&lt;&gt;"",AC31,IF(E31="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E31,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A31="","",IF(AC31&lt;&gt;"",AC31,IF(E31="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E31,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B31))="SWALE",UPPER(TRIM(AI31))="PIPE"),AND(UPPER(TRIM(B31))="TRENCH",UPPER(TRIM(AI31))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE31" s="8">
@@ -11390,7 +11413,7 @@
       <c r="AB32" s="4" t="n"/>
       <c r="AC32" s="7" t="n"/>
       <c r="AD32" s="8">
-        <f>IF(A32="","",IF(AC32&lt;&gt;"",AC32,IF(E32="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E32,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A32="","",IF(AC32&lt;&gt;"",AC32,IF(E32="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E32,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B32))="SWALE",UPPER(TRIM(AI32))="PIPE"),AND(UPPER(TRIM(B32))="TRENCH",UPPER(TRIM(AI32))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE32" s="8">
@@ -11501,7 +11524,7 @@
       <c r="AB33" s="4" t="n"/>
       <c r="AC33" s="7" t="n"/>
       <c r="AD33" s="8">
-        <f>IF(A33="","",IF(AC33&lt;&gt;"",AC33,IF(E33="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E33,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A33="","",IF(AC33&lt;&gt;"",AC33,IF(E33="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E33,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B33))="SWALE",UPPER(TRIM(AI33))="PIPE"),AND(UPPER(TRIM(B33))="TRENCH",UPPER(TRIM(AI33))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE33" s="8">
@@ -11612,7 +11635,7 @@
       <c r="AB34" s="4" t="n"/>
       <c r="AC34" s="7" t="n"/>
       <c r="AD34" s="8">
-        <f>IF(A34="","",IF(AC34&lt;&gt;"",AC34,IF(E34="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E34,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A34="","",IF(AC34&lt;&gt;"",AC34,IF(E34="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E34,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B34))="SWALE",UPPER(TRIM(AI34))="PIPE"),AND(UPPER(TRIM(B34))="TRENCH",UPPER(TRIM(AI34))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE34" s="8">
@@ -11723,7 +11746,7 @@
       <c r="AB35" s="4" t="n"/>
       <c r="AC35" s="7" t="n"/>
       <c r="AD35" s="8">
-        <f>IF(A35="","",IF(AC35&lt;&gt;"",AC35,IF(E35="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E35,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A35="","",IF(AC35&lt;&gt;"",AC35,IF(E35="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E35,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B35))="SWALE",UPPER(TRIM(AI35))="PIPE"),AND(UPPER(TRIM(B35))="TRENCH",UPPER(TRIM(AI35))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE35" s="8">
@@ -11834,7 +11857,7 @@
       <c r="AB36" s="4" t="n"/>
       <c r="AC36" s="7" t="n"/>
       <c r="AD36" s="8">
-        <f>IF(A36="","",IF(AC36&lt;&gt;"",AC36,IF(E36="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E36,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A36="","",IF(AC36&lt;&gt;"",AC36,IF(E36="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E36,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B36))="SWALE",UPPER(TRIM(AI36))="PIPE"),AND(UPPER(TRIM(B36))="TRENCH",UPPER(TRIM(AI36))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE36" s="8">
@@ -11945,7 +11968,7 @@
       <c r="AB37" s="4" t="n"/>
       <c r="AC37" s="7" t="n"/>
       <c r="AD37" s="8">
-        <f>IF(A37="","",IF(AC37&lt;&gt;"",AC37,IF(E37="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E37,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A37="","",IF(AC37&lt;&gt;"",AC37,IF(E37="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E37,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B37))="SWALE",UPPER(TRIM(AI37))="PIPE"),AND(UPPER(TRIM(B37))="TRENCH",UPPER(TRIM(AI37))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE37" s="8">
@@ -12056,7 +12079,7 @@
       <c r="AB38" s="4" t="n"/>
       <c r="AC38" s="7" t="n"/>
       <c r="AD38" s="8">
-        <f>IF(A38="","",IF(AC38&lt;&gt;"",AC38,IF(E38="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E38,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A38="","",IF(AC38&lt;&gt;"",AC38,IF(E38="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E38,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B38))="SWALE",UPPER(TRIM(AI38))="PIPE"),AND(UPPER(TRIM(B38))="TRENCH",UPPER(TRIM(AI38))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE38" s="8">
@@ -12167,7 +12190,7 @@
       <c r="AB39" s="4" t="n"/>
       <c r="AC39" s="7" t="n"/>
       <c r="AD39" s="8">
-        <f>IF(A39="","",IF(AC39&lt;&gt;"",AC39,IF(E39="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E39,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A39="","",IF(AC39&lt;&gt;"",AC39,IF(E39="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E39,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B39))="SWALE",UPPER(TRIM(AI39))="PIPE"),AND(UPPER(TRIM(B39))="TRENCH",UPPER(TRIM(AI39))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE39" s="8">
@@ -12278,7 +12301,7 @@
       <c r="AB40" s="4" t="n"/>
       <c r="AC40" s="7" t="n"/>
       <c r="AD40" s="8">
-        <f>IF(A40="","",IF(AC40&lt;&gt;"",AC40,IF(E40="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E40,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A40="","",IF(AC40&lt;&gt;"",AC40,IF(E40="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E40,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B40))="SWALE",UPPER(TRIM(AI40))="PIPE"),AND(UPPER(TRIM(B40))="TRENCH",UPPER(TRIM(AI40))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE40" s="8">
@@ -12389,7 +12412,7 @@
       <c r="AB41" s="4" t="n"/>
       <c r="AC41" s="7" t="n"/>
       <c r="AD41" s="8">
-        <f>IF(A41="","",IF(AC41&lt;&gt;"",AC41,IF(E41="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E41,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A41="","",IF(AC41&lt;&gt;"",AC41,IF(E41="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E41,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B41))="SWALE",UPPER(TRIM(AI41))="PIPE"),AND(UPPER(TRIM(B41))="TRENCH",UPPER(TRIM(AI41))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE41" s="8">
@@ -12500,7 +12523,7 @@
       <c r="AB42" s="4" t="n"/>
       <c r="AC42" s="7" t="n"/>
       <c r="AD42" s="8">
-        <f>IF(A42="","",IF(AC42&lt;&gt;"",AC42,IF(E42="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E42,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A42="","",IF(AC42&lt;&gt;"",AC42,IF(E42="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E42,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B42))="SWALE",UPPER(TRIM(AI42))="PIPE"),AND(UPPER(TRIM(B42))="TRENCH",UPPER(TRIM(AI42))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE42" s="8">
@@ -12611,7 +12634,7 @@
       <c r="AB43" s="4" t="n"/>
       <c r="AC43" s="7" t="n"/>
       <c r="AD43" s="8">
-        <f>IF(A43="","",IF(AC43&lt;&gt;"",AC43,IF(E43="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E43,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A43="","",IF(AC43&lt;&gt;"",AC43,IF(E43="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E43,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B43))="SWALE",UPPER(TRIM(AI43))="PIPE"),AND(UPPER(TRIM(B43))="TRENCH",UPPER(TRIM(AI43))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE43" s="8">
@@ -12722,7 +12745,7 @@
       <c r="AB44" s="4" t="n"/>
       <c r="AC44" s="7" t="n"/>
       <c r="AD44" s="8">
-        <f>IF(A44="","",IF(AC44&lt;&gt;"",AC44,IF(E44="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E44,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A44="","",IF(AC44&lt;&gt;"",AC44,IF(E44="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E44,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B44))="SWALE",UPPER(TRIM(AI44))="PIPE"),AND(UPPER(TRIM(B44))="TRENCH",UPPER(TRIM(AI44))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE44" s="8">
@@ -12833,7 +12856,7 @@
       <c r="AB45" s="4" t="n"/>
       <c r="AC45" s="7" t="n"/>
       <c r="AD45" s="8">
-        <f>IF(A45="","",IF(AC45&lt;&gt;"",AC45,IF(E45="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E45,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A45="","",IF(AC45&lt;&gt;"",AC45,IF(E45="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E45,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B45))="SWALE",UPPER(TRIM(AI45))="PIPE"),AND(UPPER(TRIM(B45))="TRENCH",UPPER(TRIM(AI45))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE45" s="8">
@@ -12944,7 +12967,7 @@
       <c r="AB46" s="4" t="n"/>
       <c r="AC46" s="7" t="n"/>
       <c r="AD46" s="8">
-        <f>IF(A46="","",IF(AC46&lt;&gt;"",AC46,IF(E46="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E46,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A46="","",IF(AC46&lt;&gt;"",AC46,IF(E46="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E46,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B46))="SWALE",UPPER(TRIM(AI46))="PIPE"),AND(UPPER(TRIM(B46))="TRENCH",UPPER(TRIM(AI46))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE46" s="8">
@@ -13055,7 +13078,7 @@
       <c r="AB47" s="4" t="n"/>
       <c r="AC47" s="7" t="n"/>
       <c r="AD47" s="8">
-        <f>IF(A47="","",IF(AC47&lt;&gt;"",AC47,IF(E47="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E47,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A47="","",IF(AC47&lt;&gt;"",AC47,IF(E47="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E47,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B47))="SWALE",UPPER(TRIM(AI47))="PIPE"),AND(UPPER(TRIM(B47))="TRENCH",UPPER(TRIM(AI47))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE47" s="8">
@@ -13166,7 +13189,7 @@
       <c r="AB48" s="4" t="n"/>
       <c r="AC48" s="7" t="n"/>
       <c r="AD48" s="8">
-        <f>IF(A48="","",IF(AC48&lt;&gt;"",AC48,IF(E48="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E48,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A48="","",IF(AC48&lt;&gt;"",AC48,IF(E48="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E48,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B48))="SWALE",UPPER(TRIM(AI48))="PIPE"),AND(UPPER(TRIM(B48))="TRENCH",UPPER(TRIM(AI48))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE48" s="8">
@@ -13277,7 +13300,7 @@
       <c r="AB49" s="4" t="n"/>
       <c r="AC49" s="7" t="n"/>
       <c r="AD49" s="8">
-        <f>IF(A49="","",IF(AC49&lt;&gt;"",AC49,IF(E49="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E49,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A49="","",IF(AC49&lt;&gt;"",AC49,IF(E49="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E49,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B49))="SWALE",UPPER(TRIM(AI49))="PIPE"),AND(UPPER(TRIM(B49))="TRENCH",UPPER(TRIM(AI49))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE49" s="8">
@@ -13388,7 +13411,7 @@
       <c r="AB50" s="4" t="n"/>
       <c r="AC50" s="7" t="n"/>
       <c r="AD50" s="8">
-        <f>IF(A50="","",IF(AC50&lt;&gt;"",AC50,IF(E50="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E50,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A50="","",IF(AC50&lt;&gt;"",AC50,IF(E50="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E50,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B50))="SWALE",UPPER(TRIM(AI50))="PIPE"),AND(UPPER(TRIM(B50))="TRENCH",UPPER(TRIM(AI50))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE50" s="8">
@@ -13499,7 +13522,7 @@
       <c r="AB51" s="4" t="n"/>
       <c r="AC51" s="7" t="n"/>
       <c r="AD51" s="8">
-        <f>IF(A51="","",IF(AC51&lt;&gt;"",AC51,IF(E51="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E51,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A51="","",IF(AC51&lt;&gt;"",AC51,IF(E51="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E51,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B51))="SWALE",UPPER(TRIM(AI51))="PIPE"),AND(UPPER(TRIM(B51))="TRENCH",UPPER(TRIM(AI51))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE51" s="8">
@@ -13610,7 +13633,7 @@
       <c r="AB52" s="4" t="n"/>
       <c r="AC52" s="7" t="n"/>
       <c r="AD52" s="8">
-        <f>IF(A52="","",IF(AC52&lt;&gt;"",AC52,IF(E52="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E52,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A52="","",IF(AC52&lt;&gt;"",AC52,IF(E52="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E52,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B52))="SWALE",UPPER(TRIM(AI52))="PIPE"),AND(UPPER(TRIM(B52))="TRENCH",UPPER(TRIM(AI52))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE52" s="8">
@@ -13721,7 +13744,7 @@
       <c r="AB53" s="4" t="n"/>
       <c r="AC53" s="7" t="n"/>
       <c r="AD53" s="8">
-        <f>IF(A53="","",IF(AC53&lt;&gt;"",AC53,IF(E53="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E53,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A53="","",IF(AC53&lt;&gt;"",AC53,IF(E53="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E53,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B53))="SWALE",UPPER(TRIM(AI53))="PIPE"),AND(UPPER(TRIM(B53))="TRENCH",UPPER(TRIM(AI53))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE53" s="8">
@@ -13832,7 +13855,7 @@
       <c r="AB54" s="4" t="n"/>
       <c r="AC54" s="7" t="n"/>
       <c r="AD54" s="8">
-        <f>IF(A54="","",IF(AC54&lt;&gt;"",AC54,IF(E54="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E54,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A54="","",IF(AC54&lt;&gt;"",AC54,IF(E54="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E54,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B54))="SWALE",UPPER(TRIM(AI54))="PIPE"),AND(UPPER(TRIM(B54))="TRENCH",UPPER(TRIM(AI54))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE54" s="8">
@@ -13943,7 +13966,7 @@
       <c r="AB55" s="4" t="n"/>
       <c r="AC55" s="7" t="n"/>
       <c r="AD55" s="8">
-        <f>IF(A55="","",IF(AC55&lt;&gt;"",AC55,IF(E55="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E55,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A55="","",IF(AC55&lt;&gt;"",AC55,IF(E55="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E55,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B55))="SWALE",UPPER(TRIM(AI55))="PIPE"),AND(UPPER(TRIM(B55))="TRENCH",UPPER(TRIM(AI55))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE55" s="8">
@@ -14054,7 +14077,7 @@
       <c r="AB56" s="4" t="n"/>
       <c r="AC56" s="7" t="n"/>
       <c r="AD56" s="8">
-        <f>IF(A56="","",IF(AC56&lt;&gt;"",AC56,IF(E56="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E56,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A56="","",IF(AC56&lt;&gt;"",AC56,IF(E56="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E56,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B56))="SWALE",UPPER(TRIM(AI56))="PIPE"),AND(UPPER(TRIM(B56))="TRENCH",UPPER(TRIM(AI56))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE56" s="8">
@@ -14165,7 +14188,7 @@
       <c r="AB57" s="4" t="n"/>
       <c r="AC57" s="7" t="n"/>
       <c r="AD57" s="8">
-        <f>IF(A57="","",IF(AC57&lt;&gt;"",AC57,IF(E57="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E57,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A57="","",IF(AC57&lt;&gt;"",AC57,IF(E57="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E57,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B57))="SWALE",UPPER(TRIM(AI57))="PIPE"),AND(UPPER(TRIM(B57))="TRENCH",UPPER(TRIM(AI57))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE57" s="8">
@@ -14276,7 +14299,7 @@
       <c r="AB58" s="4" t="n"/>
       <c r="AC58" s="7" t="n"/>
       <c r="AD58" s="8">
-        <f>IF(A58="","",IF(AC58&lt;&gt;"",AC58,IF(E58="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E58,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A58="","",IF(AC58&lt;&gt;"",AC58,IF(E58="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E58,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B58))="SWALE",UPPER(TRIM(AI58))="PIPE"),AND(UPPER(TRIM(B58))="TRENCH",UPPER(TRIM(AI58))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE58" s="8">
@@ -14387,7 +14410,7 @@
       <c r="AB59" s="4" t="n"/>
       <c r="AC59" s="7" t="n"/>
       <c r="AD59" s="8">
-        <f>IF(A59="","",IF(AC59&lt;&gt;"",AC59,IF(E59="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E59,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A59="","",IF(AC59&lt;&gt;"",AC59,IF(E59="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E59,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B59))="SWALE",UPPER(TRIM(AI59))="PIPE"),AND(UPPER(TRIM(B59))="TRENCH",UPPER(TRIM(AI59))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE59" s="8">
@@ -14498,7 +14521,7 @@
       <c r="AB60" s="4" t="n"/>
       <c r="AC60" s="7" t="n"/>
       <c r="AD60" s="8">
-        <f>IF(A60="","",IF(AC60&lt;&gt;"",AC60,IF(E60="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E60,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A60="","",IF(AC60&lt;&gt;"",AC60,IF(E60="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E60,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B60))="SWALE",UPPER(TRIM(AI60))="PIPE"),AND(UPPER(TRIM(B60))="TRENCH",UPPER(TRIM(AI60))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE60" s="8">
@@ -14609,7 +14632,7 @@
       <c r="AB61" s="4" t="n"/>
       <c r="AC61" s="7" t="n"/>
       <c r="AD61" s="8">
-        <f>IF(A61="","",IF(AC61&lt;&gt;"",AC61,IF(E61="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E61,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A61="","",IF(AC61&lt;&gt;"",AC61,IF(E61="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E61,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B61))="SWALE",UPPER(TRIM(AI61))="PIPE"),AND(UPPER(TRIM(B61))="TRENCH",UPPER(TRIM(AI61))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE61" s="8">
@@ -14720,7 +14743,7 @@
       <c r="AB62" s="4" t="n"/>
       <c r="AC62" s="7" t="n"/>
       <c r="AD62" s="8">
-        <f>IF(A62="","",IF(AC62&lt;&gt;"",AC62,IF(E62="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E62,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A62="","",IF(AC62&lt;&gt;"",AC62,IF(E62="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E62,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B62))="SWALE",UPPER(TRIM(AI62))="PIPE"),AND(UPPER(TRIM(B62))="TRENCH",UPPER(TRIM(AI62))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE62" s="8">
@@ -14831,7 +14854,7 @@
       <c r="AB63" s="4" t="n"/>
       <c r="AC63" s="7" t="n"/>
       <c r="AD63" s="8">
-        <f>IF(A63="","",IF(AC63&lt;&gt;"",AC63,IF(E63="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E63,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A63="","",IF(AC63&lt;&gt;"",AC63,IF(E63="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E63,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B63))="SWALE",UPPER(TRIM(AI63))="PIPE"),AND(UPPER(TRIM(B63))="TRENCH",UPPER(TRIM(AI63))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE63" s="8">
@@ -14942,7 +14965,7 @@
       <c r="AB64" s="4" t="n"/>
       <c r="AC64" s="7" t="n"/>
       <c r="AD64" s="8">
-        <f>IF(A64="","",IF(AC64&lt;&gt;"",AC64,IF(E64="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E64,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A64="","",IF(AC64&lt;&gt;"",AC64,IF(E64="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E64,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B64))="SWALE",UPPER(TRIM(AI64))="PIPE"),AND(UPPER(TRIM(B64))="TRENCH",UPPER(TRIM(AI64))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE64" s="8">
@@ -15053,7 +15076,7 @@
       <c r="AB65" s="4" t="n"/>
       <c r="AC65" s="7" t="n"/>
       <c r="AD65" s="8">
-        <f>IF(A65="","",IF(AC65&lt;&gt;"",AC65,IF(E65="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E65,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A65="","",IF(AC65&lt;&gt;"",AC65,IF(E65="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E65,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B65))="SWALE",UPPER(TRIM(AI65))="PIPE"),AND(UPPER(TRIM(B65))="TRENCH",UPPER(TRIM(AI65))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE65" s="8">
@@ -15164,7 +15187,7 @@
       <c r="AB66" s="4" t="n"/>
       <c r="AC66" s="7" t="n"/>
       <c r="AD66" s="8">
-        <f>IF(A66="","",IF(AC66&lt;&gt;"",AC66,IF(E66="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E66,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A66="","",IF(AC66&lt;&gt;"",AC66,IF(E66="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E66,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B66))="SWALE",UPPER(TRIM(AI66))="PIPE"),AND(UPPER(TRIM(B66))="TRENCH",UPPER(TRIM(AI66))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE66" s="8">
@@ -15275,7 +15298,7 @@
       <c r="AB67" s="4" t="n"/>
       <c r="AC67" s="7" t="n"/>
       <c r="AD67" s="8">
-        <f>IF(A67="","",IF(AC67&lt;&gt;"",AC67,IF(E67="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E67,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A67="","",IF(AC67&lt;&gt;"",AC67,IF(E67="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E67,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B67))="SWALE",UPPER(TRIM(AI67))="PIPE"),AND(UPPER(TRIM(B67))="TRENCH",UPPER(TRIM(AI67))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE67" s="8">
@@ -15386,7 +15409,7 @@
       <c r="AB68" s="4" t="n"/>
       <c r="AC68" s="7" t="n"/>
       <c r="AD68" s="8">
-        <f>IF(A68="","",IF(AC68&lt;&gt;"",AC68,IF(E68="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E68,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A68="","",IF(AC68&lt;&gt;"",AC68,IF(E68="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E68,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B68))="SWALE",UPPER(TRIM(AI68))="PIPE"),AND(UPPER(TRIM(B68))="TRENCH",UPPER(TRIM(AI68))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE68" s="8">
@@ -15497,7 +15520,7 @@
       <c r="AB69" s="4" t="n"/>
       <c r="AC69" s="7" t="n"/>
       <c r="AD69" s="8">
-        <f>IF(A69="","",IF(AC69&lt;&gt;"",AC69,IF(E69="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E69,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A69="","",IF(AC69&lt;&gt;"",AC69,IF(E69="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E69,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B69))="SWALE",UPPER(TRIM(AI69))="PIPE"),AND(UPPER(TRIM(B69))="TRENCH",UPPER(TRIM(AI69))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE69" s="8">
@@ -15608,7 +15631,7 @@
       <c r="AB70" s="4" t="n"/>
       <c r="AC70" s="7" t="n"/>
       <c r="AD70" s="8">
-        <f>IF(A70="","",IF(AC70&lt;&gt;"",AC70,IF(E70="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E70,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A70="","",IF(AC70&lt;&gt;"",AC70,IF(E70="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E70,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B70))="SWALE",UPPER(TRIM(AI70))="PIPE"),AND(UPPER(TRIM(B70))="TRENCH",UPPER(TRIM(AI70))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE70" s="8">
@@ -15719,7 +15742,7 @@
       <c r="AB71" s="4" t="n"/>
       <c r="AC71" s="7" t="n"/>
       <c r="AD71" s="8">
-        <f>IF(A71="","",IF(AC71&lt;&gt;"",AC71,IF(E71="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E71,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A71="","",IF(AC71&lt;&gt;"",AC71,IF(E71="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E71,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B71))="SWALE",UPPER(TRIM(AI71))="PIPE"),AND(UPPER(TRIM(B71))="TRENCH",UPPER(TRIM(AI71))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE71" s="8">
@@ -15830,7 +15853,7 @@
       <c r="AB72" s="4" t="n"/>
       <c r="AC72" s="7" t="n"/>
       <c r="AD72" s="8">
-        <f>IF(A72="","",IF(AC72&lt;&gt;"",AC72,IF(E72="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E72,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A72="","",IF(AC72&lt;&gt;"",AC72,IF(E72="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E72,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B72))="SWALE",UPPER(TRIM(AI72))="PIPE"),AND(UPPER(TRIM(B72))="TRENCH",UPPER(TRIM(AI72))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE72" s="8">
@@ -15941,7 +15964,7 @@
       <c r="AB73" s="4" t="n"/>
       <c r="AC73" s="7" t="n"/>
       <c r="AD73" s="8">
-        <f>IF(A73="","",IF(AC73&lt;&gt;"",AC73,IF(E73="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E73,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A73="","",IF(AC73&lt;&gt;"",AC73,IF(E73="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E73,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B73))="SWALE",UPPER(TRIM(AI73))="PIPE"),AND(UPPER(TRIM(B73))="TRENCH",UPPER(TRIM(AI73))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE73" s="8">
@@ -16052,7 +16075,7 @@
       <c r="AB74" s="4" t="n"/>
       <c r="AC74" s="7" t="n"/>
       <c r="AD74" s="8">
-        <f>IF(A74="","",IF(AC74&lt;&gt;"",AC74,IF(E74="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E74,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A74="","",IF(AC74&lt;&gt;"",AC74,IF(E74="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E74,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B74))="SWALE",UPPER(TRIM(AI74))="PIPE"),AND(UPPER(TRIM(B74))="TRENCH",UPPER(TRIM(AI74))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE74" s="8">
@@ -16163,7 +16186,7 @@
       <c r="AB75" s="4" t="n"/>
       <c r="AC75" s="7" t="n"/>
       <c r="AD75" s="8">
-        <f>IF(A75="","",IF(AC75&lt;&gt;"",AC75,IF(E75="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E75,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A75="","",IF(AC75&lt;&gt;"",AC75,IF(E75="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E75,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B75))="SWALE",UPPER(TRIM(AI75))="PIPE"),AND(UPPER(TRIM(B75))="TRENCH",UPPER(TRIM(AI75))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE75" s="8">
@@ -16274,7 +16297,7 @@
       <c r="AB76" s="4" t="n"/>
       <c r="AC76" s="7" t="n"/>
       <c r="AD76" s="8">
-        <f>IF(A76="","",IF(AC76&lt;&gt;"",AC76,IF(E76="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E76,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A76="","",IF(AC76&lt;&gt;"",AC76,IF(E76="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E76,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B76))="SWALE",UPPER(TRIM(AI76))="PIPE"),AND(UPPER(TRIM(B76))="TRENCH",UPPER(TRIM(AI76))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE76" s="8">
@@ -16385,7 +16408,7 @@
       <c r="AB77" s="4" t="n"/>
       <c r="AC77" s="7" t="n"/>
       <c r="AD77" s="8">
-        <f>IF(A77="","",IF(AC77&lt;&gt;"",AC77,IF(E77="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E77,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A77="","",IF(AC77&lt;&gt;"",AC77,IF(E77="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E77,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B77))="SWALE",UPPER(TRIM(AI77))="PIPE"),AND(UPPER(TRIM(B77))="TRENCH",UPPER(TRIM(AI77))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE77" s="8">
@@ -16496,7 +16519,7 @@
       <c r="AB78" s="4" t="n"/>
       <c r="AC78" s="7" t="n"/>
       <c r="AD78" s="8">
-        <f>IF(A78="","",IF(AC78&lt;&gt;"",AC78,IF(E78="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E78,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A78="","",IF(AC78&lt;&gt;"",AC78,IF(E78="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E78,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B78))="SWALE",UPPER(TRIM(AI78))="PIPE"),AND(UPPER(TRIM(B78))="TRENCH",UPPER(TRIM(AI78))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE78" s="8">
@@ -16607,7 +16630,7 @@
       <c r="AB79" s="4" t="n"/>
       <c r="AC79" s="7" t="n"/>
       <c r="AD79" s="8">
-        <f>IF(A79="","",IF(AC79&lt;&gt;"",AC79,IF(E79="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E79,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A79="","",IF(AC79&lt;&gt;"",AC79,IF(E79="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E79,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B79))="SWALE",UPPER(TRIM(AI79))="PIPE"),AND(UPPER(TRIM(B79))="TRENCH",UPPER(TRIM(AI79))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE79" s="8">
@@ -16718,7 +16741,7 @@
       <c r="AB80" s="4" t="n"/>
       <c r="AC80" s="7" t="n"/>
       <c r="AD80" s="8">
-        <f>IF(A80="","",IF(AC80&lt;&gt;"",AC80,IF(E80="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E80,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A80="","",IF(AC80&lt;&gt;"",AC80,IF(E80="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E80,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B80))="SWALE",UPPER(TRIM(AI80))="PIPE"),AND(UPPER(TRIM(B80))="TRENCH",UPPER(TRIM(AI80))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE80" s="8">
@@ -16829,7 +16852,7 @@
       <c r="AB81" s="4" t="n"/>
       <c r="AC81" s="7" t="n"/>
       <c r="AD81" s="8">
-        <f>IF(A81="","",IF(AC81&lt;&gt;"",AC81,IF(E81="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E81,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A81="","",IF(AC81&lt;&gt;"",AC81,IF(E81="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E81,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B81))="SWALE",UPPER(TRIM(AI81))="PIPE"),AND(UPPER(TRIM(B81))="TRENCH",UPPER(TRIM(AI81))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE81" s="8">
@@ -16940,7 +16963,7 @@
       <c r="AB82" s="4" t="n"/>
       <c r="AC82" s="7" t="n"/>
       <c r="AD82" s="8">
-        <f>IF(A82="","",IF(AC82&lt;&gt;"",AC82,IF(E82="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E82,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A82="","",IF(AC82&lt;&gt;"",AC82,IF(E82="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E82,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B82))="SWALE",UPPER(TRIM(AI82))="PIPE"),AND(UPPER(TRIM(B82))="TRENCH",UPPER(TRIM(AI82))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE82" s="8">
@@ -17051,7 +17074,7 @@
       <c r="AB83" s="4" t="n"/>
       <c r="AC83" s="7" t="n"/>
       <c r="AD83" s="8">
-        <f>IF(A83="","",IF(AC83&lt;&gt;"",AC83,IF(E83="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E83,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A83="","",IF(AC83&lt;&gt;"",AC83,IF(E83="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E83,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B83))="SWALE",UPPER(TRIM(AI83))="PIPE"),AND(UPPER(TRIM(B83))="TRENCH",UPPER(TRIM(AI83))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE83" s="8">
@@ -17162,7 +17185,7 @@
       <c r="AB84" s="4" t="n"/>
       <c r="AC84" s="7" t="n"/>
       <c r="AD84" s="8">
-        <f>IF(A84="","",IF(AC84&lt;&gt;"",AC84,IF(E84="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E84,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A84="","",IF(AC84&lt;&gt;"",AC84,IF(E84="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E84,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B84))="SWALE",UPPER(TRIM(AI84))="PIPE"),AND(UPPER(TRIM(B84))="TRENCH",UPPER(TRIM(AI84))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE84" s="8">
@@ -17273,7 +17296,7 @@
       <c r="AB85" s="4" t="n"/>
       <c r="AC85" s="7" t="n"/>
       <c r="AD85" s="8">
-        <f>IF(A85="","",IF(AC85&lt;&gt;"",AC85,IF(E85="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E85,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A85="","",IF(AC85&lt;&gt;"",AC85,IF(E85="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E85,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B85))="SWALE",UPPER(TRIM(AI85))="PIPE"),AND(UPPER(TRIM(B85))="TRENCH",UPPER(TRIM(AI85))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE85" s="8">
@@ -17384,7 +17407,7 @@
       <c r="AB86" s="4" t="n"/>
       <c r="AC86" s="7" t="n"/>
       <c r="AD86" s="8">
-        <f>IF(A86="","",IF(AC86&lt;&gt;"",AC86,IF(E86="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E86,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A86="","",IF(AC86&lt;&gt;"",AC86,IF(E86="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E86,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B86))="SWALE",UPPER(TRIM(AI86))="PIPE"),AND(UPPER(TRIM(B86))="TRENCH",UPPER(TRIM(AI86))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE86" s="8">
@@ -17495,7 +17518,7 @@
       <c r="AB87" s="4" t="n"/>
       <c r="AC87" s="7" t="n"/>
       <c r="AD87" s="8">
-        <f>IF(A87="","",IF(AC87&lt;&gt;"",AC87,IF(E87="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E87,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A87="","",IF(AC87&lt;&gt;"",AC87,IF(E87="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E87,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B87))="SWALE",UPPER(TRIM(AI87))="PIPE"),AND(UPPER(TRIM(B87))="TRENCH",UPPER(TRIM(AI87))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE87" s="8">
@@ -17606,7 +17629,7 @@
       <c r="AB88" s="4" t="n"/>
       <c r="AC88" s="7" t="n"/>
       <c r="AD88" s="8">
-        <f>IF(A88="","",IF(AC88&lt;&gt;"",AC88,IF(E88="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E88,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A88="","",IF(AC88&lt;&gt;"",AC88,IF(E88="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E88,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B88))="SWALE",UPPER(TRIM(AI88))="PIPE"),AND(UPPER(TRIM(B88))="TRENCH",UPPER(TRIM(AI88))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE88" s="8">
@@ -17717,7 +17740,7 @@
       <c r="AB89" s="4" t="n"/>
       <c r="AC89" s="7" t="n"/>
       <c r="AD89" s="8">
-        <f>IF(A89="","",IF(AC89&lt;&gt;"",AC89,IF(E89="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E89,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A89="","",IF(AC89&lt;&gt;"",AC89,IF(E89="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E89,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B89))="SWALE",UPPER(TRIM(AI89))="PIPE"),AND(UPPER(TRIM(B89))="TRENCH",UPPER(TRIM(AI89))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE89" s="8">
@@ -17828,7 +17851,7 @@
       <c r="AB90" s="4" t="n"/>
       <c r="AC90" s="7" t="n"/>
       <c r="AD90" s="8">
-        <f>IF(A90="","",IF(AC90&lt;&gt;"",AC90,IF(E90="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E90,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A90="","",IF(AC90&lt;&gt;"",AC90,IF(E90="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E90,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B90))="SWALE",UPPER(TRIM(AI90))="PIPE"),AND(UPPER(TRIM(B90))="TRENCH",UPPER(TRIM(AI90))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE90" s="8">
@@ -17939,7 +17962,7 @@
       <c r="AB91" s="4" t="n"/>
       <c r="AC91" s="7" t="n"/>
       <c r="AD91" s="8">
-        <f>IF(A91="","",IF(AC91&lt;&gt;"",AC91,IF(E91="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E91,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A91="","",IF(AC91&lt;&gt;"",AC91,IF(E91="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E91,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B91))="SWALE",UPPER(TRIM(AI91))="PIPE"),AND(UPPER(TRIM(B91))="TRENCH",UPPER(TRIM(AI91))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE91" s="8">
@@ -18050,7 +18073,7 @@
       <c r="AB92" s="4" t="n"/>
       <c r="AC92" s="7" t="n"/>
       <c r="AD92" s="8">
-        <f>IF(A92="","",IF(AC92&lt;&gt;"",AC92,IF(E92="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E92,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A92="","",IF(AC92&lt;&gt;"",AC92,IF(E92="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E92,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B92))="SWALE",UPPER(TRIM(AI92))="PIPE"),AND(UPPER(TRIM(B92))="TRENCH",UPPER(TRIM(AI92))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE92" s="8">
@@ -18161,7 +18184,7 @@
       <c r="AB93" s="4" t="n"/>
       <c r="AC93" s="7" t="n"/>
       <c r="AD93" s="8">
-        <f>IF(A93="","",IF(AC93&lt;&gt;"",AC93,IF(E93="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E93,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A93="","",IF(AC93&lt;&gt;"",AC93,IF(E93="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E93,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B93))="SWALE",UPPER(TRIM(AI93))="PIPE"),AND(UPPER(TRIM(B93))="TRENCH",UPPER(TRIM(AI93))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE93" s="8">
@@ -18272,7 +18295,7 @@
       <c r="AB94" s="4" t="n"/>
       <c r="AC94" s="7" t="n"/>
       <c r="AD94" s="8">
-        <f>IF(A94="","",IF(AC94&lt;&gt;"",AC94,IF(E94="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E94,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A94="","",IF(AC94&lt;&gt;"",AC94,IF(E94="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E94,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B94))="SWALE",UPPER(TRIM(AI94))="PIPE"),AND(UPPER(TRIM(B94))="TRENCH",UPPER(TRIM(AI94))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE94" s="8">
@@ -18383,7 +18406,7 @@
       <c r="AB95" s="4" t="n"/>
       <c r="AC95" s="7" t="n"/>
       <c r="AD95" s="8">
-        <f>IF(A95="","",IF(AC95&lt;&gt;"",AC95,IF(E95="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E95,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A95="","",IF(AC95&lt;&gt;"",AC95,IF(E95="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E95,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B95))="SWALE",UPPER(TRIM(AI95))="PIPE"),AND(UPPER(TRIM(B95))="TRENCH",UPPER(TRIM(AI95))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE95" s="8">
@@ -18494,7 +18517,7 @@
       <c r="AB96" s="4" t="n"/>
       <c r="AC96" s="7" t="n"/>
       <c r="AD96" s="8">
-        <f>IF(A96="","",IF(AC96&lt;&gt;"",AC96,IF(E96="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E96,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A96="","",IF(AC96&lt;&gt;"",AC96,IF(E96="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E96,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B96))="SWALE",UPPER(TRIM(AI96))="PIPE"),AND(UPPER(TRIM(B96))="TRENCH",UPPER(TRIM(AI96))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE96" s="8">
@@ -18605,7 +18628,7 @@
       <c r="AB97" s="4" t="n"/>
       <c r="AC97" s="7" t="n"/>
       <c r="AD97" s="8">
-        <f>IF(A97="","",IF(AC97&lt;&gt;"",AC97,IF(E97="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E97,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A97="","",IF(AC97&lt;&gt;"",AC97,IF(E97="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E97,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B97))="SWALE",UPPER(TRIM(AI97))="PIPE"),AND(UPPER(TRIM(B97))="TRENCH",UPPER(TRIM(AI97))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE97" s="8">
@@ -18716,7 +18739,7 @@
       <c r="AB98" s="4" t="n"/>
       <c r="AC98" s="7" t="n"/>
       <c r="AD98" s="8">
-        <f>IF(A98="","",IF(AC98&lt;&gt;"",AC98,IF(E98="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E98,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A98="","",IF(AC98&lt;&gt;"",AC98,IF(E98="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E98,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B98))="SWALE",UPPER(TRIM(AI98))="PIPE"),AND(UPPER(TRIM(B98))="TRENCH",UPPER(TRIM(AI98))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE98" s="8">
@@ -18827,7 +18850,7 @@
       <c r="AB99" s="4" t="n"/>
       <c r="AC99" s="7" t="n"/>
       <c r="AD99" s="8">
-        <f>IF(A99="","",IF(AC99&lt;&gt;"",AC99,IF(E99="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E99,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A99="","",IF(AC99&lt;&gt;"",AC99,IF(E99="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E99,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B99))="SWALE",UPPER(TRIM(AI99))="PIPE"),AND(UPPER(TRIM(B99))="TRENCH",UPPER(TRIM(AI99))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE99" s="8">
@@ -18938,7 +18961,7 @@
       <c r="AB100" s="4" t="n"/>
       <c r="AC100" s="7" t="n"/>
       <c r="AD100" s="8">
-        <f>IF(A100="","",IF(AC100&lt;&gt;"",AC100,IF(E100="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E100,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A100="","",IF(AC100&lt;&gt;"",AC100,IF(E100="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E100,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B100))="SWALE",UPPER(TRIM(AI100))="PIPE"),AND(UPPER(TRIM(B100))="TRENCH",UPPER(TRIM(AI100))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE100" s="8">
@@ -19049,7 +19072,7 @@
       <c r="AB101" s="4" t="n"/>
       <c r="AC101" s="7" t="n"/>
       <c r="AD101" s="8">
-        <f>IF(A101="","",IF(AC101&lt;&gt;"",AC101,IF(E101="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E101,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A101="","",IF(AC101&lt;&gt;"",AC101,IF(E101="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E101,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B101))="SWALE",UPPER(TRIM(AI101))="PIPE"),AND(UPPER(TRIM(B101))="TRENCH",UPPER(TRIM(AI101))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE101" s="8">
@@ -19160,7 +19183,7 @@
       <c r="AB102" s="4" t="n"/>
       <c r="AC102" s="7" t="n"/>
       <c r="AD102" s="8">
-        <f>IF(A102="","",IF(AC102&lt;&gt;"",AC102,IF(E102="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E102,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A102="","",IF(AC102&lt;&gt;"",AC102,IF(E102="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E102,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B102))="SWALE",UPPER(TRIM(AI102))="PIPE"),AND(UPPER(TRIM(B102))="TRENCH",UPPER(TRIM(AI102))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE102" s="8">
@@ -19271,7 +19294,7 @@
       <c r="AB103" s="4" t="n"/>
       <c r="AC103" s="7" t="n"/>
       <c r="AD103" s="8">
-        <f>IF(A103="","",IF(AC103&lt;&gt;"",AC103,IF(E103="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E103,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A103="","",IF(AC103&lt;&gt;"",AC103,IF(E103="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E103,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B103))="SWALE",UPPER(TRIM(AI103))="PIPE"),AND(UPPER(TRIM(B103))="TRENCH",UPPER(TRIM(AI103))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE103" s="8">
@@ -19382,7 +19405,7 @@
       <c r="AB104" s="4" t="n"/>
       <c r="AC104" s="7" t="n"/>
       <c r="AD104" s="8">
-        <f>IF(A104="","",IF(AC104&lt;&gt;"",AC104,IF(E104="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E104,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A104="","",IF(AC104&lt;&gt;"",AC104,IF(E104="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E104,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B104))="SWALE",UPPER(TRIM(AI104))="PIPE"),AND(UPPER(TRIM(B104))="TRENCH",UPPER(TRIM(AI104))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE104" s="8">
@@ -19493,7 +19516,7 @@
       <c r="AB105" s="4" t="n"/>
       <c r="AC105" s="7" t="n"/>
       <c r="AD105" s="8">
-        <f>IF(A105="","",IF(AC105&lt;&gt;"",AC105,IF(E105="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E105,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A105="","",IF(AC105&lt;&gt;"",AC105,IF(E105="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E105,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B105))="SWALE",UPPER(TRIM(AI105))="PIPE"),AND(UPPER(TRIM(B105))="TRENCH",UPPER(TRIM(AI105))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE105" s="8">
@@ -19604,7 +19627,7 @@
       <c r="AB106" s="4" t="n"/>
       <c r="AC106" s="7" t="n"/>
       <c r="AD106" s="8">
-        <f>IF(A106="","",IF(AC106&lt;&gt;"",AC106,IF(E106="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E106,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A106="","",IF(AC106&lt;&gt;"",AC106,IF(E106="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E106,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B106))="SWALE",UPPER(TRIM(AI106))="PIPE"),AND(UPPER(TRIM(B106))="TRENCH",UPPER(TRIM(AI106))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE106" s="8">
@@ -19715,7 +19738,7 @@
       <c r="AB107" s="4" t="n"/>
       <c r="AC107" s="7" t="n"/>
       <c r="AD107" s="8">
-        <f>IF(A107="","",IF(AC107&lt;&gt;"",AC107,IF(E107="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E107,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A107="","",IF(AC107&lt;&gt;"",AC107,IF(E107="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E107,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B107))="SWALE",UPPER(TRIM(AI107))="PIPE"),AND(UPPER(TRIM(B107))="TRENCH",UPPER(TRIM(AI107))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE107" s="8">
@@ -19826,7 +19849,7 @@
       <c r="AB108" s="4" t="n"/>
       <c r="AC108" s="7" t="n"/>
       <c r="AD108" s="8">
-        <f>IF(A108="","",IF(AC108&lt;&gt;"",AC108,IF(E108="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E108,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A108="","",IF(AC108&lt;&gt;"",AC108,IF(E108="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E108,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B108))="SWALE",UPPER(TRIM(AI108))="PIPE"),AND(UPPER(TRIM(B108))="TRENCH",UPPER(TRIM(AI108))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE108" s="8">
@@ -19937,7 +19960,7 @@
       <c r="AB109" s="4" t="n"/>
       <c r="AC109" s="7" t="n"/>
       <c r="AD109" s="8">
-        <f>IF(A109="","",IF(AC109&lt;&gt;"",AC109,IF(E109="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E109,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A109="","",IF(AC109&lt;&gt;"",AC109,IF(E109="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E109,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B109))="SWALE",UPPER(TRIM(AI109))="PIPE"),AND(UPPER(TRIM(B109))="TRENCH",UPPER(TRIM(AI109))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE109" s="8">
@@ -20048,7 +20071,7 @@
       <c r="AB110" s="4" t="n"/>
       <c r="AC110" s="7" t="n"/>
       <c r="AD110" s="8">
-        <f>IF(A110="","",IF(AC110&lt;&gt;"",AC110,IF(E110="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E110,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A110="","",IF(AC110&lt;&gt;"",AC110,IF(E110="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E110,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B110))="SWALE",UPPER(TRIM(AI110))="PIPE"),AND(UPPER(TRIM(B110))="TRENCH",UPPER(TRIM(AI110))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE110" s="8">
@@ -20159,7 +20182,7 @@
       <c r="AB111" s="4" t="n"/>
       <c r="AC111" s="7" t="n"/>
       <c r="AD111" s="8">
-        <f>IF(A111="","",IF(AC111&lt;&gt;"",AC111,IF(E111="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E111,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A111="","",IF(AC111&lt;&gt;"",AC111,IF(E111="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E111,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B111))="SWALE",UPPER(TRIM(AI111))="PIPE"),AND(UPPER(TRIM(B111))="TRENCH",UPPER(TRIM(AI111))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE111" s="8">
@@ -20270,7 +20293,7 @@
       <c r="AB112" s="4" t="n"/>
       <c r="AC112" s="7" t="n"/>
       <c r="AD112" s="8">
-        <f>IF(A112="","",IF(AC112&lt;&gt;"",AC112,IF(E112="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E112,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A112="","",IF(AC112&lt;&gt;"",AC112,IF(E112="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E112,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B112))="SWALE",UPPER(TRIM(AI112))="PIPE"),AND(UPPER(TRIM(B112))="TRENCH",UPPER(TRIM(AI112))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE112" s="8">
@@ -20381,7 +20404,7 @@
       <c r="AB113" s="4" t="n"/>
       <c r="AC113" s="7" t="n"/>
       <c r="AD113" s="8">
-        <f>IF(A113="","",IF(AC113&lt;&gt;"",AC113,IF(E113="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E113,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A113="","",IF(AC113&lt;&gt;"",AC113,IF(E113="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E113,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B113))="SWALE",UPPER(TRIM(AI113))="PIPE"),AND(UPPER(TRIM(B113))="TRENCH",UPPER(TRIM(AI113))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE113" s="8">
@@ -20492,7 +20515,7 @@
       <c r="AB114" s="4" t="n"/>
       <c r="AC114" s="7" t="n"/>
       <c r="AD114" s="8">
-        <f>IF(A114="","",IF(AC114&lt;&gt;"",AC114,IF(E114="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E114,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A114="","",IF(AC114&lt;&gt;"",AC114,IF(E114="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E114,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B114))="SWALE",UPPER(TRIM(AI114))="PIPE"),AND(UPPER(TRIM(B114))="TRENCH",UPPER(TRIM(AI114))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE114" s="8">
@@ -20603,7 +20626,7 @@
       <c r="AB115" s="4" t="n"/>
       <c r="AC115" s="7" t="n"/>
       <c r="AD115" s="8">
-        <f>IF(A115="","",IF(AC115&lt;&gt;"",AC115,IF(E115="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E115,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A115="","",IF(AC115&lt;&gt;"",AC115,IF(E115="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E115,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B115))="SWALE",UPPER(TRIM(AI115))="PIPE"),AND(UPPER(TRIM(B115))="TRENCH",UPPER(TRIM(AI115))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE115" s="8">
@@ -20714,7 +20737,7 @@
       <c r="AB116" s="4" t="n"/>
       <c r="AC116" s="7" t="n"/>
       <c r="AD116" s="8">
-        <f>IF(A116="","",IF(AC116&lt;&gt;"",AC116,IF(E116="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E116,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A116="","",IF(AC116&lt;&gt;"",AC116,IF(E116="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E116,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B116))="SWALE",UPPER(TRIM(AI116))="PIPE"),AND(UPPER(TRIM(B116))="TRENCH",UPPER(TRIM(AI116))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE116" s="8">
@@ -20825,7 +20848,7 @@
       <c r="AB117" s="4" t="n"/>
       <c r="AC117" s="7" t="n"/>
       <c r="AD117" s="8">
-        <f>IF(A117="","",IF(AC117&lt;&gt;"",AC117,IF(E117="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E117,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A117="","",IF(AC117&lt;&gt;"",AC117,IF(E117="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E117,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B117))="SWALE",UPPER(TRIM(AI117))="PIPE"),AND(UPPER(TRIM(B117))="TRENCH",UPPER(TRIM(AI117))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE117" s="8">
@@ -20936,7 +20959,7 @@
       <c r="AB118" s="4" t="n"/>
       <c r="AC118" s="7" t="n"/>
       <c r="AD118" s="8">
-        <f>IF(A118="","",IF(AC118&lt;&gt;"",AC118,IF(E118="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E118,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A118="","",IF(AC118&lt;&gt;"",AC118,IF(E118="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E118,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B118))="SWALE",UPPER(TRIM(AI118))="PIPE"),AND(UPPER(TRIM(B118))="TRENCH",UPPER(TRIM(AI118))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE118" s="8">
@@ -21047,7 +21070,7 @@
       <c r="AB119" s="4" t="n"/>
       <c r="AC119" s="7" t="n"/>
       <c r="AD119" s="8">
-        <f>IF(A119="","",IF(AC119&lt;&gt;"",AC119,IF(E119="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E119,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A119="","",IF(AC119&lt;&gt;"",AC119,IF(E119="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E119,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B119))="SWALE",UPPER(TRIM(AI119))="PIPE"),AND(UPPER(TRIM(B119))="TRENCH",UPPER(TRIM(AI119))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE119" s="8">
@@ -21158,7 +21181,7 @@
       <c r="AB120" s="4" t="n"/>
       <c r="AC120" s="7" t="n"/>
       <c r="AD120" s="8">
-        <f>IF(A120="","",IF(AC120&lt;&gt;"",AC120,IF(E120="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E120,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A120="","",IF(AC120&lt;&gt;"",AC120,IF(E120="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E120,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B120))="SWALE",UPPER(TRIM(AI120))="PIPE"),AND(UPPER(TRIM(B120))="TRENCH",UPPER(TRIM(AI120))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE120" s="8">
@@ -21269,7 +21292,7 @@
       <c r="AB121" s="4" t="n"/>
       <c r="AC121" s="7" t="n"/>
       <c r="AD121" s="8">
-        <f>IF(A121="","",IF(AC121&lt;&gt;"",AC121,IF(E121="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E121,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A121="","",IF(AC121&lt;&gt;"",AC121,IF(E121="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E121,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B121))="SWALE",UPPER(TRIM(AI121))="PIPE"),AND(UPPER(TRIM(B121))="TRENCH",UPPER(TRIM(AI121))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE121" s="8">
@@ -21380,7 +21403,7 @@
       <c r="AB122" s="4" t="n"/>
       <c r="AC122" s="7" t="n"/>
       <c r="AD122" s="8">
-        <f>IF(A122="","",IF(AC122&lt;&gt;"",AC122,IF(E122="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E122,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A122="","",IF(AC122&lt;&gt;"",AC122,IF(E122="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E122,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B122))="SWALE",UPPER(TRIM(AI122))="PIPE"),AND(UPPER(TRIM(B122))="TRENCH",UPPER(TRIM(AI122))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE122" s="8">
@@ -21491,7 +21514,7 @@
       <c r="AB123" s="4" t="n"/>
       <c r="AC123" s="7" t="n"/>
       <c r="AD123" s="8">
-        <f>IF(A123="","",IF(AC123&lt;&gt;"",AC123,IF(E123="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E123,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A123="","",IF(AC123&lt;&gt;"",AC123,IF(E123="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E123,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B123))="SWALE",UPPER(TRIM(AI123))="PIPE"),AND(UPPER(TRIM(B123))="TRENCH",UPPER(TRIM(AI123))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE123" s="8">
@@ -21602,7 +21625,7 @@
       <c r="AB124" s="4" t="n"/>
       <c r="AC124" s="7" t="n"/>
       <c r="AD124" s="8">
-        <f>IF(A124="","",IF(AC124&lt;&gt;"",AC124,IF(E124="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E124,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A124="","",IF(AC124&lt;&gt;"",AC124,IF(E124="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E124,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B124))="SWALE",UPPER(TRIM(AI124))="PIPE"),AND(UPPER(TRIM(B124))="TRENCH",UPPER(TRIM(AI124))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE124" s="8">
@@ -21713,7 +21736,7 @@
       <c r="AB125" s="4" t="n"/>
       <c r="AC125" s="7" t="n"/>
       <c r="AD125" s="8">
-        <f>IF(A125="","",IF(AC125&lt;&gt;"",AC125,IF(E125="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E125,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A125="","",IF(AC125&lt;&gt;"",AC125,IF(E125="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E125,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B125))="SWALE",UPPER(TRIM(AI125))="PIPE"),AND(UPPER(TRIM(B125))="TRENCH",UPPER(TRIM(AI125))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE125" s="8">
@@ -21824,7 +21847,7 @@
       <c r="AB126" s="4" t="n"/>
       <c r="AC126" s="7" t="n"/>
       <c r="AD126" s="8">
-        <f>IF(A126="","",IF(AC126&lt;&gt;"",AC126,IF(E126="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E126,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A126="","",IF(AC126&lt;&gt;"",AC126,IF(E126="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E126,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B126))="SWALE",UPPER(TRIM(AI126))="PIPE"),AND(UPPER(TRIM(B126))="TRENCH",UPPER(TRIM(AI126))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE126" s="8">
@@ -21935,7 +21958,7 @@
       <c r="AB127" s="4" t="n"/>
       <c r="AC127" s="7" t="n"/>
       <c r="AD127" s="8">
-        <f>IF(A127="","",IF(AC127&lt;&gt;"",AC127,IF(E127="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E127,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A127="","",IF(AC127&lt;&gt;"",AC127,IF(E127="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E127,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B127))="SWALE",UPPER(TRIM(AI127))="PIPE"),AND(UPPER(TRIM(B127))="TRENCH",UPPER(TRIM(AI127))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE127" s="8">
@@ -22046,7 +22069,7 @@
       <c r="AB128" s="4" t="n"/>
       <c r="AC128" s="7" t="n"/>
       <c r="AD128" s="8">
-        <f>IF(A128="","",IF(AC128&lt;&gt;"",AC128,IF(E128="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E128,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A128="","",IF(AC128&lt;&gt;"",AC128,IF(E128="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E128,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B128))="SWALE",UPPER(TRIM(AI128))="PIPE"),AND(UPPER(TRIM(B128))="TRENCH",UPPER(TRIM(AI128))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE128" s="8">
@@ -22157,7 +22180,7 @@
       <c r="AB129" s="4" t="n"/>
       <c r="AC129" s="7" t="n"/>
       <c r="AD129" s="8">
-        <f>IF(A129="","",IF(AC129&lt;&gt;"",AC129,IF(E129="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E129,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A129="","",IF(AC129&lt;&gt;"",AC129,IF(E129="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E129,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B129))="SWALE",UPPER(TRIM(AI129))="PIPE"),AND(UPPER(TRIM(B129))="TRENCH",UPPER(TRIM(AI129))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE129" s="8">
@@ -22268,7 +22291,7 @@
       <c r="AB130" s="4" t="n"/>
       <c r="AC130" s="7" t="n"/>
       <c r="AD130" s="8">
-        <f>IF(A130="","",IF(AC130&lt;&gt;"",AC130,IF(E130="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E130,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A130="","",IF(AC130&lt;&gt;"",AC130,IF(E130="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E130,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B130))="SWALE",UPPER(TRIM(AI130))="PIPE"),AND(UPPER(TRIM(B130))="TRENCH",UPPER(TRIM(AI130))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE130" s="8">
@@ -22379,7 +22402,7 @@
       <c r="AB131" s="4" t="n"/>
       <c r="AC131" s="7" t="n"/>
       <c r="AD131" s="8">
-        <f>IF(A131="","",IF(AC131&lt;&gt;"",AC131,IF(E131="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E131,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A131="","",IF(AC131&lt;&gt;"",AC131,IF(E131="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E131,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B131))="SWALE",UPPER(TRIM(AI131))="PIPE"),AND(UPPER(TRIM(B131))="TRENCH",UPPER(TRIM(AI131))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE131" s="8">
@@ -22490,7 +22513,7 @@
       <c r="AB132" s="4" t="n"/>
       <c r="AC132" s="7" t="n"/>
       <c r="AD132" s="8">
-        <f>IF(A132="","",IF(AC132&lt;&gt;"",AC132,IF(E132="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E132,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A132="","",IF(AC132&lt;&gt;"",AC132,IF(E132="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E132,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B132))="SWALE",UPPER(TRIM(AI132))="PIPE"),AND(UPPER(TRIM(B132))="TRENCH",UPPER(TRIM(AI132))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE132" s="8">
@@ -22601,7 +22624,7 @@
       <c r="AB133" s="4" t="n"/>
       <c r="AC133" s="7" t="n"/>
       <c r="AD133" s="8">
-        <f>IF(A133="","",IF(AC133&lt;&gt;"",AC133,IF(E133="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E133,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A133="","",IF(AC133&lt;&gt;"",AC133,IF(E133="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E133,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B133))="SWALE",UPPER(TRIM(AI133))="PIPE"),AND(UPPER(TRIM(B133))="TRENCH",UPPER(TRIM(AI133))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE133" s="8">
@@ -22712,7 +22735,7 @@
       <c r="AB134" s="4" t="n"/>
       <c r="AC134" s="7" t="n"/>
       <c r="AD134" s="8">
-        <f>IF(A134="","",IF(AC134&lt;&gt;"",AC134,IF(E134="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E134,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A134="","",IF(AC134&lt;&gt;"",AC134,IF(E134="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E134,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B134))="SWALE",UPPER(TRIM(AI134))="PIPE"),AND(UPPER(TRIM(B134))="TRENCH",UPPER(TRIM(AI134))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE134" s="8">
@@ -22823,7 +22846,7 @@
       <c r="AB135" s="4" t="n"/>
       <c r="AC135" s="7" t="n"/>
       <c r="AD135" s="8">
-        <f>IF(A135="","",IF(AC135&lt;&gt;"",AC135,IF(E135="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E135,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A135="","",IF(AC135&lt;&gt;"",AC135,IF(E135="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E135,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B135))="SWALE",UPPER(TRIM(AI135))="PIPE"),AND(UPPER(TRIM(B135))="TRENCH",UPPER(TRIM(AI135))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE135" s="8">
@@ -22934,7 +22957,7 @@
       <c r="AB136" s="4" t="n"/>
       <c r="AC136" s="7" t="n"/>
       <c r="AD136" s="8">
-        <f>IF(A136="","",IF(AC136&lt;&gt;"",AC136,IF(E136="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E136,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A136="","",IF(AC136&lt;&gt;"",AC136,IF(E136="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E136,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B136))="SWALE",UPPER(TRIM(AI136))="PIPE"),AND(UPPER(TRIM(B136))="TRENCH",UPPER(TRIM(AI136))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE136" s="8">
@@ -23045,7 +23068,7 @@
       <c r="AB137" s="4" t="n"/>
       <c r="AC137" s="7" t="n"/>
       <c r="AD137" s="8">
-        <f>IF(A137="","",IF(AC137&lt;&gt;"",AC137,IF(E137="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E137,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A137="","",IF(AC137&lt;&gt;"",AC137,IF(E137="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E137,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B137))="SWALE",UPPER(TRIM(AI137))="PIPE"),AND(UPPER(TRIM(B137))="TRENCH",UPPER(TRIM(AI137))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE137" s="8">
@@ -23156,7 +23179,7 @@
       <c r="AB138" s="4" t="n"/>
       <c r="AC138" s="7" t="n"/>
       <c r="AD138" s="8">
-        <f>IF(A138="","",IF(AC138&lt;&gt;"",AC138,IF(E138="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E138,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A138="","",IF(AC138&lt;&gt;"",AC138,IF(E138="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E138,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B138))="SWALE",UPPER(TRIM(AI138))="PIPE"),AND(UPPER(TRIM(B138))="TRENCH",UPPER(TRIM(AI138))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE138" s="8">
@@ -23267,7 +23290,7 @@
       <c r="AB139" s="4" t="n"/>
       <c r="AC139" s="7" t="n"/>
       <c r="AD139" s="8">
-        <f>IF(A139="","",IF(AC139&lt;&gt;"",AC139,IF(E139="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E139,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A139="","",IF(AC139&lt;&gt;"",AC139,IF(E139="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E139,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B139))="SWALE",UPPER(TRIM(AI139))="PIPE"),AND(UPPER(TRIM(B139))="TRENCH",UPPER(TRIM(AI139))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE139" s="8">
@@ -23378,7 +23401,7 @@
       <c r="AB140" s="4" t="n"/>
       <c r="AC140" s="7" t="n"/>
       <c r="AD140" s="8">
-        <f>IF(A140="","",IF(AC140&lt;&gt;"",AC140,IF(E140="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E140,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A140="","",IF(AC140&lt;&gt;"",AC140,IF(E140="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E140,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B140))="SWALE",UPPER(TRIM(AI140))="PIPE"),AND(UPPER(TRIM(B140))="TRENCH",UPPER(TRIM(AI140))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE140" s="8">
@@ -23489,7 +23512,7 @@
       <c r="AB141" s="4" t="n"/>
       <c r="AC141" s="7" t="n"/>
       <c r="AD141" s="8">
-        <f>IF(A141="","",IF(AC141&lt;&gt;"",AC141,IF(E141="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E141,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A141="","",IF(AC141&lt;&gt;"",AC141,IF(E141="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E141,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B141))="SWALE",UPPER(TRIM(AI141))="PIPE"),AND(UPPER(TRIM(B141))="TRENCH",UPPER(TRIM(AI141))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE141" s="8">
@@ -23600,7 +23623,7 @@
       <c r="AB142" s="4" t="n"/>
       <c r="AC142" s="7" t="n"/>
       <c r="AD142" s="8">
-        <f>IF(A142="","",IF(AC142&lt;&gt;"",AC142,IF(E142="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E142,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A142="","",IF(AC142&lt;&gt;"",AC142,IF(E142="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E142,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B142))="SWALE",UPPER(TRIM(AI142))="PIPE"),AND(UPPER(TRIM(B142))="TRENCH",UPPER(TRIM(AI142))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE142" s="8">
@@ -23711,7 +23734,7 @@
       <c r="AB143" s="4" t="n"/>
       <c r="AC143" s="7" t="n"/>
       <c r="AD143" s="8">
-        <f>IF(A143="","",IF(AC143&lt;&gt;"",AC143,IF(E143="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E143,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A143="","",IF(AC143&lt;&gt;"",AC143,IF(E143="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E143,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B143))="SWALE",UPPER(TRIM(AI143))="PIPE"),AND(UPPER(TRIM(B143))="TRENCH",UPPER(TRIM(AI143))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE143" s="8">
@@ -23822,7 +23845,7 @@
       <c r="AB144" s="4" t="n"/>
       <c r="AC144" s="7" t="n"/>
       <c r="AD144" s="8">
-        <f>IF(A144="","",IF(AC144&lt;&gt;"",AC144,IF(E144="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E144,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A144="","",IF(AC144&lt;&gt;"",AC144,IF(E144="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E144,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B144))="SWALE",UPPER(TRIM(AI144))="PIPE"),AND(UPPER(TRIM(B144))="TRENCH",UPPER(TRIM(AI144))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE144" s="8">
@@ -23933,7 +23956,7 @@
       <c r="AB145" s="4" t="n"/>
       <c r="AC145" s="7" t="n"/>
       <c r="AD145" s="8">
-        <f>IF(A145="","",IF(AC145&lt;&gt;"",AC145,IF(E145="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E145,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A145="","",IF(AC145&lt;&gt;"",AC145,IF(E145="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E145,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B145))="SWALE",UPPER(TRIM(AI145))="PIPE"),AND(UPPER(TRIM(B145))="TRENCH",UPPER(TRIM(AI145))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE145" s="8">
@@ -24044,7 +24067,7 @@
       <c r="AB146" s="4" t="n"/>
       <c r="AC146" s="7" t="n"/>
       <c r="AD146" s="8">
-        <f>IF(A146="","",IF(AC146&lt;&gt;"",AC146,IF(E146="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E146,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A146="","",IF(AC146&lt;&gt;"",AC146,IF(E146="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E146,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B146))="SWALE",UPPER(TRIM(AI146))="PIPE"),AND(UPPER(TRIM(B146))="TRENCH",UPPER(TRIM(AI146))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE146" s="8">
@@ -24155,7 +24178,7 @@
       <c r="AB147" s="4" t="n"/>
       <c r="AC147" s="7" t="n"/>
       <c r="AD147" s="8">
-        <f>IF(A147="","",IF(AC147&lt;&gt;"",AC147,IF(E147="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E147,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A147="","",IF(AC147&lt;&gt;"",AC147,IF(E147="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E147,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B147))="SWALE",UPPER(TRIM(AI147))="PIPE"),AND(UPPER(TRIM(B147))="TRENCH",UPPER(TRIM(AI147))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE147" s="8">
@@ -24266,7 +24289,7 @@
       <c r="AB148" s="4" t="n"/>
       <c r="AC148" s="7" t="n"/>
       <c r="AD148" s="8">
-        <f>IF(A148="","",IF(AC148&lt;&gt;"",AC148,IF(E148="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E148,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A148="","",IF(AC148&lt;&gt;"",AC148,IF(E148="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E148,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B148))="SWALE",UPPER(TRIM(AI148))="PIPE"),AND(UPPER(TRIM(B148))="TRENCH",UPPER(TRIM(AI148))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE148" s="8">
@@ -24377,7 +24400,7 @@
       <c r="AB149" s="4" t="n"/>
       <c r="AC149" s="7" t="n"/>
       <c r="AD149" s="8">
-        <f>IF(A149="","",IF(AC149&lt;&gt;"",AC149,IF(E149="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E149,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A149="","",IF(AC149&lt;&gt;"",AC149,IF(E149="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E149,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B149))="SWALE",UPPER(TRIM(AI149))="PIPE"),AND(UPPER(TRIM(B149))="TRENCH",UPPER(TRIM(AI149))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE149" s="8">
@@ -24488,7 +24511,7 @@
       <c r="AB150" s="4" t="n"/>
       <c r="AC150" s="7" t="n"/>
       <c r="AD150" s="8">
-        <f>IF(A150="","",IF(AC150&lt;&gt;"",AC150,IF(E150="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E150,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A150="","",IF(AC150&lt;&gt;"",AC150,IF(E150="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E150,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B150))="SWALE",UPPER(TRIM(AI150))="PIPE"),AND(UPPER(TRIM(B150))="TRENCH",UPPER(TRIM(AI150))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE150" s="8">
@@ -24599,7 +24622,7 @@
       <c r="AB151" s="4" t="n"/>
       <c r="AC151" s="7" t="n"/>
       <c r="AD151" s="8">
-        <f>IF(A151="","",IF(AC151&lt;&gt;"",AC151,IF(E151="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E151,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A151="","",IF(AC151&lt;&gt;"",AC151,IF(E151="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E151,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B151))="SWALE",UPPER(TRIM(AI151))="PIPE"),AND(UPPER(TRIM(B151))="TRENCH",UPPER(TRIM(AI151))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE151" s="8">
@@ -24710,7 +24733,7 @@
       <c r="AB152" s="4" t="n"/>
       <c r="AC152" s="7" t="n"/>
       <c r="AD152" s="8">
-        <f>IF(A152="","",IF(AC152&lt;&gt;"",AC152,IF(E152="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E152,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A152="","",IF(AC152&lt;&gt;"",AC152,IF(E152="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E152,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B152))="SWALE",UPPER(TRIM(AI152))="PIPE"),AND(UPPER(TRIM(B152))="TRENCH",UPPER(TRIM(AI152))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE152" s="8">
@@ -24821,7 +24844,7 @@
       <c r="AB153" s="4" t="n"/>
       <c r="AC153" s="7" t="n"/>
       <c r="AD153" s="8">
-        <f>IF(A153="","",IF(AC153&lt;&gt;"",AC153,IF(E153="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E153,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A153="","",IF(AC153&lt;&gt;"",AC153,IF(E153="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E153,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B153))="SWALE",UPPER(TRIM(AI153))="PIPE"),AND(UPPER(TRIM(B153))="TRENCH",UPPER(TRIM(AI153))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE153" s="8">
@@ -24932,7 +24955,7 @@
       <c r="AB154" s="4" t="n"/>
       <c r="AC154" s="7" t="n"/>
       <c r="AD154" s="8">
-        <f>IF(A154="","",IF(AC154&lt;&gt;"",AC154,IF(E154="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E154,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A154="","",IF(AC154&lt;&gt;"",AC154,IF(E154="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E154,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B154))="SWALE",UPPER(TRIM(AI154))="PIPE"),AND(UPPER(TRIM(B154))="TRENCH",UPPER(TRIM(AI154))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE154" s="8">
@@ -25043,7 +25066,7 @@
       <c r="AB155" s="4" t="n"/>
       <c r="AC155" s="7" t="n"/>
       <c r="AD155" s="8">
-        <f>IF(A155="","",IF(AC155&lt;&gt;"",AC155,IF(E155="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E155,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A155="","",IF(AC155&lt;&gt;"",AC155,IF(E155="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E155,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B155))="SWALE",UPPER(TRIM(AI155))="PIPE"),AND(UPPER(TRIM(B155))="TRENCH",UPPER(TRIM(AI155))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE155" s="8">
@@ -25154,7 +25177,7 @@
       <c r="AB156" s="4" t="n"/>
       <c r="AC156" s="7" t="n"/>
       <c r="AD156" s="8">
-        <f>IF(A156="","",IF(AC156&lt;&gt;"",AC156,IF(E156="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E156,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A156="","",IF(AC156&lt;&gt;"",AC156,IF(E156="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E156,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B156))="SWALE",UPPER(TRIM(AI156))="PIPE"),AND(UPPER(TRIM(B156))="TRENCH",UPPER(TRIM(AI156))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE156" s="8">
@@ -25265,7 +25288,7 @@
       <c r="AB157" s="4" t="n"/>
       <c r="AC157" s="7" t="n"/>
       <c r="AD157" s="8">
-        <f>IF(A157="","",IF(AC157&lt;&gt;"",AC157,IF(E157="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E157,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A157="","",IF(AC157&lt;&gt;"",AC157,IF(E157="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E157,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B157))="SWALE",UPPER(TRIM(AI157))="PIPE"),AND(UPPER(TRIM(B157))="TRENCH",UPPER(TRIM(AI157))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE157" s="8">
@@ -25376,7 +25399,7 @@
       <c r="AB158" s="4" t="n"/>
       <c r="AC158" s="7" t="n"/>
       <c r="AD158" s="8">
-        <f>IF(A158="","",IF(AC158&lt;&gt;"",AC158,IF(E158="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E158,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A158="","",IF(AC158&lt;&gt;"",AC158,IF(E158="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E158,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B158))="SWALE",UPPER(TRIM(AI158))="PIPE"),AND(UPPER(TRIM(B158))="TRENCH",UPPER(TRIM(AI158))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE158" s="8">
@@ -25487,7 +25510,7 @@
       <c r="AB159" s="4" t="n"/>
       <c r="AC159" s="7" t="n"/>
       <c r="AD159" s="8">
-        <f>IF(A159="","",IF(AC159&lt;&gt;"",AC159,IF(E159="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E159,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A159="","",IF(AC159&lt;&gt;"",AC159,IF(E159="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E159,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B159))="SWALE",UPPER(TRIM(AI159))="PIPE"),AND(UPPER(TRIM(B159))="TRENCH",UPPER(TRIM(AI159))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE159" s="8">
@@ -25598,7 +25621,7 @@
       <c r="AB160" s="4" t="n"/>
       <c r="AC160" s="7" t="n"/>
       <c r="AD160" s="8">
-        <f>IF(A160="","",IF(AC160&lt;&gt;"",AC160,IF(E160="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E160,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A160="","",IF(AC160&lt;&gt;"",AC160,IF(E160="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E160,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B160))="SWALE",UPPER(TRIM(AI160))="PIPE"),AND(UPPER(TRIM(B160))="TRENCH",UPPER(TRIM(AI160))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE160" s="8">
@@ -25709,7 +25732,7 @@
       <c r="AB161" s="4" t="n"/>
       <c r="AC161" s="7" t="n"/>
       <c r="AD161" s="8">
-        <f>IF(A161="","",IF(AC161&lt;&gt;"",AC161,IF(E161="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E161,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A161="","",IF(AC161&lt;&gt;"",AC161,IF(E161="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E161,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B161))="SWALE",UPPER(TRIM(AI161))="PIPE"),AND(UPPER(TRIM(B161))="TRENCH",UPPER(TRIM(AI161))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE161" s="8">
@@ -25820,7 +25843,7 @@
       <c r="AB162" s="4" t="n"/>
       <c r="AC162" s="7" t="n"/>
       <c r="AD162" s="8">
-        <f>IF(A162="","",IF(AC162&lt;&gt;"",AC162,IF(E162="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E162,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A162="","",IF(AC162&lt;&gt;"",AC162,IF(E162="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E162,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B162))="SWALE",UPPER(TRIM(AI162))="PIPE"),AND(UPPER(TRIM(B162))="TRENCH",UPPER(TRIM(AI162))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE162" s="8">
@@ -25931,7 +25954,7 @@
       <c r="AB163" s="4" t="n"/>
       <c r="AC163" s="7" t="n"/>
       <c r="AD163" s="8">
-        <f>IF(A163="","",IF(AC163&lt;&gt;"",AC163,IF(E163="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E163,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A163="","",IF(AC163&lt;&gt;"",AC163,IF(E163="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E163,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B163))="SWALE",UPPER(TRIM(AI163))="PIPE"),AND(UPPER(TRIM(B163))="TRENCH",UPPER(TRIM(AI163))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE163" s="8">
@@ -26042,7 +26065,7 @@
       <c r="AB164" s="4" t="n"/>
       <c r="AC164" s="7" t="n"/>
       <c r="AD164" s="8">
-        <f>IF(A164="","",IF(AC164&lt;&gt;"",AC164,IF(E164="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E164,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A164="","",IF(AC164&lt;&gt;"",AC164,IF(E164="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E164,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B164))="SWALE",UPPER(TRIM(AI164))="PIPE"),AND(UPPER(TRIM(B164))="TRENCH",UPPER(TRIM(AI164))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE164" s="8">
@@ -26153,7 +26176,7 @@
       <c r="AB165" s="4" t="n"/>
       <c r="AC165" s="7" t="n"/>
       <c r="AD165" s="8">
-        <f>IF(A165="","",IF(AC165&lt;&gt;"",AC165,IF(E165="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E165,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A165="","",IF(AC165&lt;&gt;"",AC165,IF(E165="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E165,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B165))="SWALE",UPPER(TRIM(AI165))="PIPE"),AND(UPPER(TRIM(B165))="TRENCH",UPPER(TRIM(AI165))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE165" s="8">
@@ -26264,7 +26287,7 @@
       <c r="AB166" s="4" t="n"/>
       <c r="AC166" s="7" t="n"/>
       <c r="AD166" s="8">
-        <f>IF(A166="","",IF(AC166&lt;&gt;"",AC166,IF(E166="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E166,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A166="","",IF(AC166&lt;&gt;"",AC166,IF(E166="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E166,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B166))="SWALE",UPPER(TRIM(AI166))="PIPE"),AND(UPPER(TRIM(B166))="TRENCH",UPPER(TRIM(AI166))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE166" s="8">
@@ -26375,7 +26398,7 @@
       <c r="AB167" s="4" t="n"/>
       <c r="AC167" s="7" t="n"/>
       <c r="AD167" s="8">
-        <f>IF(A167="","",IF(AC167&lt;&gt;"",AC167,IF(E167="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E167,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A167="","",IF(AC167&lt;&gt;"",AC167,IF(E167="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E167,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B167))="SWALE",UPPER(TRIM(AI167))="PIPE"),AND(UPPER(TRIM(B167))="TRENCH",UPPER(TRIM(AI167))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE167" s="8">
@@ -26486,7 +26509,7 @@
       <c r="AB168" s="4" t="n"/>
       <c r="AC168" s="7" t="n"/>
       <c r="AD168" s="8">
-        <f>IF(A168="","",IF(AC168&lt;&gt;"",AC168,IF(E168="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E168,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A168="","",IF(AC168&lt;&gt;"",AC168,IF(E168="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E168,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B168))="SWALE",UPPER(TRIM(AI168))="PIPE"),AND(UPPER(TRIM(B168))="TRENCH",UPPER(TRIM(AI168))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE168" s="8">
@@ -26597,7 +26620,7 @@
       <c r="AB169" s="4" t="n"/>
       <c r="AC169" s="7" t="n"/>
       <c r="AD169" s="8">
-        <f>IF(A169="","",IF(AC169&lt;&gt;"",AC169,IF(E169="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E169,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A169="","",IF(AC169&lt;&gt;"",AC169,IF(E169="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E169,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B169))="SWALE",UPPER(TRIM(AI169))="PIPE"),AND(UPPER(TRIM(B169))="TRENCH",UPPER(TRIM(AI169))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE169" s="8">
@@ -26708,7 +26731,7 @@
       <c r="AB170" s="4" t="n"/>
       <c r="AC170" s="7" t="n"/>
       <c r="AD170" s="8">
-        <f>IF(A170="","",IF(AC170&lt;&gt;"",AC170,IF(E170="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E170,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A170="","",IF(AC170&lt;&gt;"",AC170,IF(E170="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E170,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B170))="SWALE",UPPER(TRIM(AI170))="PIPE"),AND(UPPER(TRIM(B170))="TRENCH",UPPER(TRIM(AI170))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE170" s="8">
@@ -26819,7 +26842,7 @@
       <c r="AB171" s="4" t="n"/>
       <c r="AC171" s="7" t="n"/>
       <c r="AD171" s="8">
-        <f>IF(A171="","",IF(AC171&lt;&gt;"",AC171,IF(E171="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E171,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A171="","",IF(AC171&lt;&gt;"",AC171,IF(E171="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E171,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B171))="SWALE",UPPER(TRIM(AI171))="PIPE"),AND(UPPER(TRIM(B171))="TRENCH",UPPER(TRIM(AI171))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE171" s="8">
@@ -26930,7 +26953,7 @@
       <c r="AB172" s="4" t="n"/>
       <c r="AC172" s="7" t="n"/>
       <c r="AD172" s="8">
-        <f>IF(A172="","",IF(AC172&lt;&gt;"",AC172,IF(E172="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E172,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A172="","",IF(AC172&lt;&gt;"",AC172,IF(E172="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E172,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B172))="SWALE",UPPER(TRIM(AI172))="PIPE"),AND(UPPER(TRIM(B172))="TRENCH",UPPER(TRIM(AI172))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE172" s="8">
@@ -27041,7 +27064,7 @@
       <c r="AB173" s="4" t="n"/>
       <c r="AC173" s="7" t="n"/>
       <c r="AD173" s="8">
-        <f>IF(A173="","",IF(AC173&lt;&gt;"",AC173,IF(E173="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E173,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A173="","",IF(AC173&lt;&gt;"",AC173,IF(E173="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E173,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B173))="SWALE",UPPER(TRIM(AI173))="PIPE"),AND(UPPER(TRIM(B173))="TRENCH",UPPER(TRIM(AI173))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE173" s="8">
@@ -27152,7 +27175,7 @@
       <c r="AB174" s="4" t="n"/>
       <c r="AC174" s="7" t="n"/>
       <c r="AD174" s="8">
-        <f>IF(A174="","",IF(AC174&lt;&gt;"",AC174,IF(E174="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E174,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A174="","",IF(AC174&lt;&gt;"",AC174,IF(E174="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E174,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B174))="SWALE",UPPER(TRIM(AI174))="PIPE"),AND(UPPER(TRIM(B174))="TRENCH",UPPER(TRIM(AI174))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE174" s="8">
@@ -27263,7 +27286,7 @@
       <c r="AB175" s="4" t="n"/>
       <c r="AC175" s="7" t="n"/>
       <c r="AD175" s="8">
-        <f>IF(A175="","",IF(AC175&lt;&gt;"",AC175,IF(E175="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E175,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A175="","",IF(AC175&lt;&gt;"",AC175,IF(E175="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E175,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B175))="SWALE",UPPER(TRIM(AI175))="PIPE"),AND(UPPER(TRIM(B175))="TRENCH",UPPER(TRIM(AI175))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE175" s="8">
@@ -27374,7 +27397,7 @@
       <c r="AB176" s="4" t="n"/>
       <c r="AC176" s="7" t="n"/>
       <c r="AD176" s="8">
-        <f>IF(A176="","",IF(AC176&lt;&gt;"",AC176,IF(E176="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E176,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A176="","",IF(AC176&lt;&gt;"",AC176,IF(E176="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E176,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B176))="SWALE",UPPER(TRIM(AI176))="PIPE"),AND(UPPER(TRIM(B176))="TRENCH",UPPER(TRIM(AI176))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE176" s="8">
@@ -27485,7 +27508,7 @@
       <c r="AB177" s="4" t="n"/>
       <c r="AC177" s="7" t="n"/>
       <c r="AD177" s="8">
-        <f>IF(A177="","",IF(AC177&lt;&gt;"",AC177,IF(E177="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E177,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A177="","",IF(AC177&lt;&gt;"",AC177,IF(E177="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E177,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B177))="SWALE",UPPER(TRIM(AI177))="PIPE"),AND(UPPER(TRIM(B177))="TRENCH",UPPER(TRIM(AI177))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE177" s="8">
@@ -27596,7 +27619,7 @@
       <c r="AB178" s="4" t="n"/>
       <c r="AC178" s="7" t="n"/>
       <c r="AD178" s="8">
-        <f>IF(A178="","",IF(AC178&lt;&gt;"",AC178,IF(E178="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E178,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A178="","",IF(AC178&lt;&gt;"",AC178,IF(E178="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E178,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B178))="SWALE",UPPER(TRIM(AI178))="PIPE"),AND(UPPER(TRIM(B178))="TRENCH",UPPER(TRIM(AI178))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE178" s="8">
@@ -27707,7 +27730,7 @@
       <c r="AB179" s="4" t="n"/>
       <c r="AC179" s="7" t="n"/>
       <c r="AD179" s="8">
-        <f>IF(A179="","",IF(AC179&lt;&gt;"",AC179,IF(E179="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E179,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A179="","",IF(AC179&lt;&gt;"",AC179,IF(E179="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E179,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B179))="SWALE",UPPER(TRIM(AI179))="PIPE"),AND(UPPER(TRIM(B179))="TRENCH",UPPER(TRIM(AI179))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE179" s="8">
@@ -27818,7 +27841,7 @@
       <c r="AB180" s="4" t="n"/>
       <c r="AC180" s="7" t="n"/>
       <c r="AD180" s="8">
-        <f>IF(A180="","",IF(AC180&lt;&gt;"",AC180,IF(E180="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E180,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A180="","",IF(AC180&lt;&gt;"",AC180,IF(E180="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E180,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B180))="SWALE",UPPER(TRIM(AI180))="PIPE"),AND(UPPER(TRIM(B180))="TRENCH",UPPER(TRIM(AI180))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE180" s="8">
@@ -27929,7 +27952,7 @@
       <c r="AB181" s="4" t="n"/>
       <c r="AC181" s="7" t="n"/>
       <c r="AD181" s="8">
-        <f>IF(A181="","",IF(AC181&lt;&gt;"",AC181,IF(E181="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E181,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A181="","",IF(AC181&lt;&gt;"",AC181,IF(E181="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E181,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B181))="SWALE",UPPER(TRIM(AI181))="PIPE"),AND(UPPER(TRIM(B181))="TRENCH",UPPER(TRIM(AI181))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE181" s="8">
@@ -28040,7 +28063,7 @@
       <c r="AB182" s="4" t="n"/>
       <c r="AC182" s="7" t="n"/>
       <c r="AD182" s="8">
-        <f>IF(A182="","",IF(AC182&lt;&gt;"",AC182,IF(E182="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E182,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A182="","",IF(AC182&lt;&gt;"",AC182,IF(E182="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E182,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B182))="SWALE",UPPER(TRIM(AI182))="PIPE"),AND(UPPER(TRIM(B182))="TRENCH",UPPER(TRIM(AI182))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE182" s="8">
@@ -28151,7 +28174,7 @@
       <c r="AB183" s="4" t="n"/>
       <c r="AC183" s="7" t="n"/>
       <c r="AD183" s="8">
-        <f>IF(A183="","",IF(AC183&lt;&gt;"",AC183,IF(E183="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E183,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A183="","",IF(AC183&lt;&gt;"",AC183,IF(E183="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E183,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B183))="SWALE",UPPER(TRIM(AI183))="PIPE"),AND(UPPER(TRIM(B183))="TRENCH",UPPER(TRIM(AI183))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE183" s="8">
@@ -28262,7 +28285,7 @@
       <c r="AB184" s="4" t="n"/>
       <c r="AC184" s="7" t="n"/>
       <c r="AD184" s="8">
-        <f>IF(A184="","",IF(AC184&lt;&gt;"",AC184,IF(E184="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E184,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A184="","",IF(AC184&lt;&gt;"",AC184,IF(E184="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E184,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B184))="SWALE",UPPER(TRIM(AI184))="PIPE"),AND(UPPER(TRIM(B184))="TRENCH",UPPER(TRIM(AI184))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE184" s="8">
@@ -28373,7 +28396,7 @@
       <c r="AB185" s="4" t="n"/>
       <c r="AC185" s="7" t="n"/>
       <c r="AD185" s="8">
-        <f>IF(A185="","",IF(AC185&lt;&gt;"",AC185,IF(E185="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E185,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A185="","",IF(AC185&lt;&gt;"",AC185,IF(E185="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E185,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B185))="SWALE",UPPER(TRIM(AI185))="PIPE"),AND(UPPER(TRIM(B185))="TRENCH",UPPER(TRIM(AI185))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE185" s="8">
@@ -28484,7 +28507,7 @@
       <c r="AB186" s="4" t="n"/>
       <c r="AC186" s="7" t="n"/>
       <c r="AD186" s="8">
-        <f>IF(A186="","",IF(AC186&lt;&gt;"",AC186,IF(E186="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E186,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A186="","",IF(AC186&lt;&gt;"",AC186,IF(E186="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E186,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B186))="SWALE",UPPER(TRIM(AI186))="PIPE"),AND(UPPER(TRIM(B186))="TRENCH",UPPER(TRIM(AI186))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE186" s="8">
@@ -28595,7 +28618,7 @@
       <c r="AB187" s="4" t="n"/>
       <c r="AC187" s="7" t="n"/>
       <c r="AD187" s="8">
-        <f>IF(A187="","",IF(AC187&lt;&gt;"",AC187,IF(E187="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E187,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A187="","",IF(AC187&lt;&gt;"",AC187,IF(E187="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E187,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B187))="SWALE",UPPER(TRIM(AI187))="PIPE"),AND(UPPER(TRIM(B187))="TRENCH",UPPER(TRIM(AI187))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE187" s="8">
@@ -28706,7 +28729,7 @@
       <c r="AB188" s="4" t="n"/>
       <c r="AC188" s="7" t="n"/>
       <c r="AD188" s="8">
-        <f>IF(A188="","",IF(AC188&lt;&gt;"",AC188,IF(E188="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E188,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A188="","",IF(AC188&lt;&gt;"",AC188,IF(E188="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E188,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B188))="SWALE",UPPER(TRIM(AI188))="PIPE"),AND(UPPER(TRIM(B188))="TRENCH",UPPER(TRIM(AI188))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE188" s="8">
@@ -28817,7 +28840,7 @@
       <c r="AB189" s="4" t="n"/>
       <c r="AC189" s="7" t="n"/>
       <c r="AD189" s="8">
-        <f>IF(A189="","",IF(AC189&lt;&gt;"",AC189,IF(E189="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E189,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A189="","",IF(AC189&lt;&gt;"",AC189,IF(E189="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E189,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B189))="SWALE",UPPER(TRIM(AI189))="PIPE"),AND(UPPER(TRIM(B189))="TRENCH",UPPER(TRIM(AI189))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE189" s="8">
@@ -28928,7 +28951,7 @@
       <c r="AB190" s="4" t="n"/>
       <c r="AC190" s="7" t="n"/>
       <c r="AD190" s="8">
-        <f>IF(A190="","",IF(AC190&lt;&gt;"",AC190,IF(E190="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E190,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A190="","",IF(AC190&lt;&gt;"",AC190,IF(E190="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E190,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B190))="SWALE",UPPER(TRIM(AI190))="PIPE"),AND(UPPER(TRIM(B190))="TRENCH",UPPER(TRIM(AI190))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE190" s="8">
@@ -29039,7 +29062,7 @@
       <c r="AB191" s="4" t="n"/>
       <c r="AC191" s="7" t="n"/>
       <c r="AD191" s="8">
-        <f>IF(A191="","",IF(AC191&lt;&gt;"",AC191,IF(E191="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E191,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A191="","",IF(AC191&lt;&gt;"",AC191,IF(E191="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E191,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B191))="SWALE",UPPER(TRIM(AI191))="PIPE"),AND(UPPER(TRIM(B191))="TRENCH",UPPER(TRIM(AI191))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE191" s="8">
@@ -29150,7 +29173,7 @@
       <c r="AB192" s="4" t="n"/>
       <c r="AC192" s="7" t="n"/>
       <c r="AD192" s="8">
-        <f>IF(A192="","",IF(AC192&lt;&gt;"",AC192,IF(E192="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E192,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A192="","",IF(AC192&lt;&gt;"",AC192,IF(E192="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E192,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B192))="SWALE",UPPER(TRIM(AI192))="PIPE"),AND(UPPER(TRIM(B192))="TRENCH",UPPER(TRIM(AI192))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE192" s="8">
@@ -29261,7 +29284,7 @@
       <c r="AB193" s="4" t="n"/>
       <c r="AC193" s="7" t="n"/>
       <c r="AD193" s="8">
-        <f>IF(A193="","",IF(AC193&lt;&gt;"",AC193,IF(E193="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E193,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A193="","",IF(AC193&lt;&gt;"",AC193,IF(E193="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E193,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B193))="SWALE",UPPER(TRIM(AI193))="PIPE"),AND(UPPER(TRIM(B193))="TRENCH",UPPER(TRIM(AI193))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE193" s="8">
@@ -29372,7 +29395,7 @@
       <c r="AB194" s="4" t="n"/>
       <c r="AC194" s="7" t="n"/>
       <c r="AD194" s="8">
-        <f>IF(A194="","",IF(AC194&lt;&gt;"",AC194,IF(E194="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E194,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A194="","",IF(AC194&lt;&gt;"",AC194,IF(E194="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E194,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B194))="SWALE",UPPER(TRIM(AI194))="PIPE"),AND(UPPER(TRIM(B194))="TRENCH",UPPER(TRIM(AI194))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE194" s="8">
@@ -29483,7 +29506,7 @@
       <c r="AB195" s="4" t="n"/>
       <c r="AC195" s="7" t="n"/>
       <c r="AD195" s="8">
-        <f>IF(A195="","",IF(AC195&lt;&gt;"",AC195,IF(E195="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E195,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A195="","",IF(AC195&lt;&gt;"",AC195,IF(E195="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E195,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B195))="SWALE",UPPER(TRIM(AI195))="PIPE"),AND(UPPER(TRIM(B195))="TRENCH",UPPER(TRIM(AI195))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE195" s="8">
@@ -29594,7 +29617,7 @@
       <c r="AB196" s="4" t="n"/>
       <c r="AC196" s="7" t="n"/>
       <c r="AD196" s="8">
-        <f>IF(A196="","",IF(AC196&lt;&gt;"",AC196,IF(E196="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E196,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A196="","",IF(AC196&lt;&gt;"",AC196,IF(E196="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E196,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B196))="SWALE",UPPER(TRIM(AI196))="PIPE"),AND(UPPER(TRIM(B196))="TRENCH",UPPER(TRIM(AI196))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE196" s="8">
@@ -29705,7 +29728,7 @@
       <c r="AB197" s="4" t="n"/>
       <c r="AC197" s="7" t="n"/>
       <c r="AD197" s="8">
-        <f>IF(A197="","",IF(AC197&lt;&gt;"",AC197,IF(E197="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E197,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A197="","",IF(AC197&lt;&gt;"",AC197,IF(E197="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E197,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B197))="SWALE",UPPER(TRIM(AI197))="PIPE"),AND(UPPER(TRIM(B197))="TRENCH",UPPER(TRIM(AI197))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE197" s="8">
@@ -29816,7 +29839,7 @@
       <c r="AB198" s="4" t="n"/>
       <c r="AC198" s="7" t="n"/>
       <c r="AD198" s="8">
-        <f>IF(A198="","",IF(AC198&lt;&gt;"",AC198,IF(E198="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E198,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A198="","",IF(AC198&lt;&gt;"",AC198,IF(E198="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E198,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B198))="SWALE",UPPER(TRIM(AI198))="PIPE"),AND(UPPER(TRIM(B198))="TRENCH",UPPER(TRIM(AI198))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE198" s="8">
@@ -29927,7 +29950,7 @@
       <c r="AB199" s="4" t="n"/>
       <c r="AC199" s="7" t="n"/>
       <c r="AD199" s="8">
-        <f>IF(A199="","",IF(AC199&lt;&gt;"",AC199,IF(E199="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E199,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A199="","",IF(AC199&lt;&gt;"",AC199,IF(E199="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E199,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B199))="SWALE",UPPER(TRIM(AI199))="PIPE"),AND(UPPER(TRIM(B199))="TRENCH",UPPER(TRIM(AI199))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE199" s="8">
@@ -30038,7 +30061,7 @@
       <c r="AB200" s="4" t="n"/>
       <c r="AC200" s="7" t="n"/>
       <c r="AD200" s="8">
-        <f>IF(A200="","",IF(AC200&lt;&gt;"",AC200,IF(E200="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E200,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A200="","",IF(AC200&lt;&gt;"",AC200,IF(E200="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E200,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B200))="SWALE",UPPER(TRIM(AI200))="PIPE"),AND(UPPER(TRIM(B200))="TRENCH",UPPER(TRIM(AI200))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE200" s="8">
@@ -30149,7 +30172,7 @@
       <c r="AB201" s="4" t="n"/>
       <c r="AC201" s="7" t="n"/>
       <c r="AD201" s="8">
-        <f>IF(A201="","",IF(AC201&lt;&gt;"",AC201,IF(E201="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E201,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A201="","",IF(AC201&lt;&gt;"",AC201,IF(E201="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E201,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B201))="SWALE",UPPER(TRIM(AI201))="PIPE"),AND(UPPER(TRIM(B201))="TRENCH",UPPER(TRIM(AI201))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE201" s="8">
@@ -30260,7 +30283,7 @@
       <c r="AB202" s="4" t="n"/>
       <c r="AC202" s="7" t="n"/>
       <c r="AD202" s="8">
-        <f>IF(A202="","",IF(AC202&lt;&gt;"",AC202,IF(E202="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E202,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A202="","",IF(AC202&lt;&gt;"",AC202,IF(E202="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E202,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B202))="SWALE",UPPER(TRIM(AI202))="PIPE"),AND(UPPER(TRIM(B202))="TRENCH",UPPER(TRIM(AI202))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE202" s="8">
@@ -30371,7 +30394,7 @@
       <c r="AB203" s="4" t="n"/>
       <c r="AC203" s="7" t="n"/>
       <c r="AD203" s="8">
-        <f>IF(A203="","",IF(AC203&lt;&gt;"",AC203,IF(E203="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E203,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A203="","",IF(AC203&lt;&gt;"",AC203,IF(E203="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E203,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B203))="SWALE",UPPER(TRIM(AI203))="PIPE"),AND(UPPER(TRIM(B203))="TRENCH",UPPER(TRIM(AI203))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE203" s="8">
@@ -30482,7 +30505,7 @@
       <c r="AB204" s="4" t="n"/>
       <c r="AC204" s="7" t="n"/>
       <c r="AD204" s="8">
-        <f>IF(A204="","",IF(AC204&lt;&gt;"",AC204,IF(E204="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E204,$A$4:$A$204,0)),""))))</f>
+        <f>IF(A204="","",IF(AC204&lt;&gt;"",AC204,IF(E204="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E204,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B204))="SWALE",UPPER(TRIM(AI204))="PIPE"),AND(UPPER(TRIM(B204))="TRENCH",UPPER(TRIM(AI204))="PIPE")),Inputs!$B$57,0),""))))</f>
         <v/>
       </c>
       <c r="AE204" s="8">

</xml_diff>

<commit_message>
Clarify decision summary: E04 corner link and basin-node geometry
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="164" formatCode="[&lt;1]0.000;0.00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -110,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -133,6 +136,7 @@
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1216,7 +1220,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4) Exutoire final au bassin de retention via J-BASSIN-IN -&gt; BASSIN-RET.</t>
+          <t>4) Deux entrees au bassin: EST (J-BASSIN-IN) et OUEST (J-BASSIN-OUEST) vers BASSIN-RET.</t>
         </is>
       </c>
     </row>
@@ -1366,18 +1370,19 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>South basin corridor width x length (m)</t>
+          <t>West connector to basin inlet (m)</t>
         </is>
       </c>
       <c r="B14" s="9">
-        <f>Inputs!B34&amp;" x "&amp;Inputs!B35</f>
+        <f>Inputs!B53</f>
         <v/>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Between building and pedestrian road</t>
-        </is>
-      </c>
+          <t>Measured corner link J-OUEST-AVAL -&gt; J-BASSIN-OUEST</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>E04</t>
@@ -1399,54 +1404,51 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Basin target depth (m)</t>
+          <t>Retention basin corridor width x length (m)</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <f>Inputs!B36</f>
+        <f>Inputs!B34&amp;" x "&amp;Inputs!B35</f>
         <v/>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Adjust with topo survey</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>E05</t>
-        </is>
-      </c>
-      <c r="F15" s="4">
-        <f>IFERROR(INDEX(Elements_hybrides!$B$4:$B$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="13">
-        <f>IFERROR(INDEX(Elements_hybrides!$Q$4:$Q$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="4">
-        <f>IFERROR(INDEX(Elements_hybrides!$AA$4:$AA$204,MATCH(E15,Elements_hybrides!$A$4:$A$204,0)),"")</f>
-        <v/>
+          <t>Storage geometry at node BASSIN-RET (not an E04 reach).</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>BASSIN-RET (node)</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Max cover near west utilities (m)</t>
+          <t>East inlet pipe length to basin (m)</t>
         </is>
       </c>
       <c r="B16" s="9">
-        <f>Inputs!B39</f>
+        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E07",Elements_hybrides!$A$4:$A$204,0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Conservative limit</t>
-        </is>
-      </c>
+          <t>J-BASSIN-IN -&gt; BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="F16" s="4">
@@ -1463,9 +1465,24 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>West inlet pipe length to basin (m)</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E08",Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>J-BASSIN-OUEST -&gt; BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="F17" s="4">

</xml_diff>

<commit_message>
Correct east segment lengths and clarify paved crossing/outlet notes
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -854,6 +854,27 @@
       <c r="A47" t="inlineStr">
         <is>
           <t>Inputs!B59 est une vitesse adoptee (pas la vitesse calculee hydraulique) pour eviter references circulaires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Important: un ecoulement gravitaire ne peut pas remonter de la conduite vers une noue plus haute sans pompage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Condition pratique PIPE-&gt;SWALE: radier sortie conduite &gt;= fond noue aval (ou tres legerement au-dessus), sinon CHECK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Le regard/ouvrage de sortie sert a dissiper/organiser la transition, pas a "lever" l eau par gravite.</t>
         </is>
       </c>
     </row>
@@ -10391,7 +10412,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>21.6</v>
+        <v>9.6</v>
       </c>
       <c r="G4" s="7">
         <f>Inputs!$B$33</f>
@@ -10475,7 +10496,7 @@
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>Bande est amont (arbres) - underdrain segment 1.</t>
+          <t>Longueur corrigee selon plan: P-01 -&gt; P-02 = 9.6 m.</t>
         </is>
       </c>
       <c r="AC4" s="7" t="n"/>
@@ -10543,7 +10564,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>21.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G5" s="7">
         <f>Inputs!$B$33</f>
@@ -10627,7 +10648,7 @@
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>Bande est aval (arbres) - underdrain segment 2.</t>
+          <t>Longueur corrigee selon plan: P-02 -&gt; P-03 = 8.7 m.</t>
         </is>
       </c>
       <c r="AC5" s="7" t="n"/>
@@ -11202,7 +11223,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni court via caniveau/grille + conduite (DN250).</t>
+          <t>Traverse pave-uni: capture ponctuelle (caniveau/avaloir grille) + conduite courte de traversee DN250.</t>
         </is>
       </c>
       <c r="AC9" s="7" t="n"/>
@@ -11490,7 +11511,7 @@
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni principal via caniveau/grille + conduite (DN300).</t>
+          <t>Traverse pave-uni: capture ponctuelle (grille) + conduite courte de traversee DN300 vers noue aval.</t>
         </is>
       </c>
       <c r="AC11" s="7" t="n"/>

</xml_diff>

<commit_message>
Revise west paved crossings to surface caniveaux for gravity continuity
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -875,6 +875,20 @@
       <c r="A50" t="inlineStr">
         <is>
           <t>Le regard/ouvrage de sortie sert a dissiper/organiser la transition, pas a "lever" l eau par gravite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Strategie ouest revisee: traverses pave-uni traitees en caniveaux de surface (E05B, E05D), pas en conduites enterrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Objectif: eviter cas pipe profond -&gt; noue aval plus haute, et garder un profil gravitaire lisible.</t>
         </is>
       </c>
     </row>
@@ -11130,7 +11144,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>SWALE</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -11155,17 +11169,23 @@
       <c r="G9" s="7" t="n">
         <v>0.01</v>
       </c>
-      <c r="H9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="n">
+        <v>0.015</v>
+      </c>
       <c r="I9" s="8">
         <f>IF(A9="","",IF(H9&lt;&gt;"",H9,IF(UPPER(TRIM(B9))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B9))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J9" s="7" t="n">
-        <v>250</v>
-      </c>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="N9" s="7" t="n">
         <v>0</v>
       </c>
@@ -11223,7 +11243,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni: capture ponctuelle (caniveau/avaloir grille) + conduite courte de traversee DN250.</t>
+          <t>Traverse pave-uni par caniveau a grille de surface (pas de conduite enterree sur ce troncon).</t>
         </is>
       </c>
       <c r="AC9" s="7" t="n"/>
@@ -11418,7 +11438,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>SWALE</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -11443,17 +11463,23 @@
       <c r="G11" s="7" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="H11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="n">
+        <v>0.015</v>
+      </c>
       <c r="I11" s="8">
         <f>IF(A11="","",IF(H11&lt;&gt;"",H11,IF(UPPER(TRIM(B11))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B11))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="K11" s="7" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
-      <c r="M11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr"/>
+      <c r="K11" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="N11" s="7" t="n">
         <v>0</v>
       </c>
@@ -11511,7 +11537,7 @@
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni: capture ponctuelle (grille) + conduite courte de traversee DN300 vers noue aval.</t>
+          <t>Traverse pave-uni principal par caniveau a grille de surface (pas de conduite enterree sur ce troncon).</t>
         </is>
       </c>
       <c r="AC11" s="7" t="n"/>
@@ -40285,22 +40311,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Caniveau grille + pipe DN250</t>
+          <t>Caniveau grille de surface</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>E05B (PIPE)</t>
+          <t>E05B (CANIVEAU SURFACE)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>slope ~1.0%</t>
+          <t>section ~0.25 x 0.08 m</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Raccorder aux noeuds MH.</t>
+          <t>Aucune remontee hydraulique requise; ecoulement de surface continu.</t>
         </is>
       </c>
     </row>
@@ -40349,22 +40375,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Caniveau grille + pipe DN300</t>
+          <t>Caniveau grille de surface</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>E05D (PIPE)</t>
+          <t>E05D (CANIVEAU SURFACE)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>slope ~0.9%</t>
+          <t>section ~0.30 x 0.10 m</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Verifier degagement lateraux.</t>
+          <t>Aucune conduite profonde de traversee sur ce troncon.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Route east tresfond via mechanical outlet and switch west branch back to pipes
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention.xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -137,6 +137,7 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -573,14 +574,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cote droite avec arbres: prioriser noue de surface peu profonde + protections racinaires; eviter conduite profonde en zone racinaire.</t>
+          <t>2) Bande sud (2.0 m): conduite/collecte vers volume de retention dans le corridor contraint.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Exutoire: bassin de retention en bas a gauche (node BASIN_RET).</t>
+          <t>3) Ouest: strategie revisee en conduites (pas de noues) vers E04 puis E08 et bassin.</t>
         </is>
       </c>
     </row>
@@ -889,6 +890,20 @@
       <c r="A52" t="inlineStr">
         <is>
           <t>Objectif: eviter cas pipe profond -&gt; noue aval plus haute, et garder un profil gravitaire lisible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Changement concept: zone grise est (tresfond) drainee vers puisards et reseau interne mecanique jusqu'a sortie sud pres bassin (E09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Resume surfaces disponibles dans Decision_Summary (A34:B37) et Resume_checks (B10:B12).</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1269,14 +1284,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3) Ouest (utilities): collecte de surface peu profonde priorisee, traverses ponctuelles controlees.</t>
+          <t>3) Ouest: drainage en conduites (DN250/DN300) vers E04 puis entree ouest bassin.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4) Deux entrees au bassin: EST (J-BASSIN-IN) et OUEST (J-BASSIN-OUEST) vers BASSIN-RET.</t>
+          <t>4) Zone grise est (tresfond): puisards + reseau interne mecanique vers sortie sud et bassin.</t>
         </is>
       </c>
     </row>
@@ -1673,6 +1688,67 @@
           <t>- Verifier protection racinaire et details constructifs (barriere racinaire + cleanouts + acces entretien).</t>
         </is>
       </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Surface summary (readable quantities)</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Impervious area total (m2)</t>
+        </is>
+      </c>
+      <c r="B35" s="4">
+        <f>Resume_checks!B10</f>
+        <v/>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>ROOF + PAVAGE + TRESFOND</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Grass area total (m2)</t>
+        </is>
+      </c>
+      <c r="B36" s="4">
+        <f>Resume_checks!B11</f>
+        <v/>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>GRASS only</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Impervious fraction</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>Resume_checks!B12</f>
+        <v/>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Impervious/(Impervious+Grass)</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1710,7 +1786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2896,6 +2972,46 @@
       <c r="D59" s="4" t="inlineStr">
         <is>
           <t>Vitesse adoptee pour calcul temps de transit dans element route (evite references circulaires).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Mech_internal_outlet_length_m</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Longueur approximative conduite interne mecanique (puisards est -&gt; sortie sud pres bassin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Mech_internal_outlet_diameter_mm</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Diametre indicatif conduite mecanique interne (a confirmer par equipe mecanique).</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3230,12 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Pente vers bande est</t>
+          <t>Puisards zone grise est -&gt; reseau interne mecanique -&gt; sortie sud pres bassin (pas vers bande est).</t>
         </is>
       </c>
       <c r="L5" s="5" t="n">
@@ -10852,7 +10968,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -10882,16 +10998,12 @@
         <f>IF(A7="","",IF(H7&lt;&gt;"",H7,IF(UPPER(TRIM(B7))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B7))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L7" s="7" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="M7" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="J7" s="7" t="n">
+        <v>375</v>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="n">
         <v>0</v>
       </c>
@@ -10949,7 +11061,7 @@
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>Corrige: liaison ouest courte vers entree ouest bassin (4.7 m mesure).</t>
+          <t>Collecteur ouest final en conduite (4.7 m) vers entree ouest bassin.</t>
         </is>
       </c>
       <c r="AC7" s="7" t="n"/>
@@ -10998,7 +11110,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -11028,16 +11140,12 @@
         <f>IF(A8="","",IF(H8&lt;&gt;"",H8,IF(UPPER(TRIM(B8))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B8))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J8" s="7" t="inlineStr"/>
-      <c r="K8" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L8" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M8" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="J8" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr"/>
       <c r="N8" s="7" t="n">
         <v>0</v>
       </c>
@@ -11095,7 +11203,7 @@
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>Ouest gazon amont - longueur issue cotes plan (chaine 11.1 m repartie par aires).</t>
+          <t>Ouest segment amont en conduite DN250 vers E05B.</t>
         </is>
       </c>
       <c r="AC8" s="7" t="n"/>
@@ -11144,7 +11252,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -11169,23 +11277,17 @@
       <c r="G9" s="7" t="n">
         <v>0.01</v>
       </c>
-      <c r="H9" s="7" t="n">
-        <v>0.015</v>
-      </c>
+      <c r="H9" s="7" t="inlineStr"/>
       <c r="I9" s="8">
         <f>IF(A9="","",IF(H9&lt;&gt;"",H9,IF(UPPER(TRIM(B9))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B9))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="M9" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="J9" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
       <c r="N9" s="7" t="n">
         <v>0</v>
       </c>
@@ -11243,7 +11345,7 @@
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni par caniveau a grille de surface (pas de conduite enterree sur ce troncon).</t>
+          <t>Traverse pave-uni court en conduite DN250 (strategy ouest tout-pipe).</t>
         </is>
       </c>
       <c r="AC9" s="7" t="n"/>
@@ -11292,7 +11394,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -11322,16 +11424,12 @@
         <f>IF(A10="","",IF(H10&lt;&gt;"",H10,IF(UPPER(TRIM(B10))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B10))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J10" s="7" t="inlineStr"/>
-      <c r="K10" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L10" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M10" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="J10" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
+      <c r="M10" s="7" t="inlineStr"/>
       <c r="N10" s="7" t="n">
         <v>0</v>
       </c>
@@ -11389,7 +11487,7 @@
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>Ouest gazon milieu - longueur issue cotes plan (chaine 11.1 m repartie par aires).</t>
+          <t>Ouest segment milieu en conduite DN300 vers E05D.</t>
         </is>
       </c>
       <c r="AC10" s="7" t="n"/>
@@ -11438,7 +11536,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -11463,23 +11561,17 @@
       <c r="G11" s="7" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="H11" s="7" t="n">
-        <v>0.015</v>
-      </c>
+      <c r="H11" s="7" t="inlineStr"/>
       <c r="I11" s="8">
         <f>IF(A11="","",IF(H11&lt;&gt;"",H11,IF(UPPER(TRIM(B11))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B11))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J11" s="7" t="inlineStr"/>
-      <c r="K11" s="7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L11" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M11" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="J11" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
       <c r="N11" s="7" t="n">
         <v>0</v>
       </c>
@@ -11537,7 +11629,7 @@
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>Traverse pave-uni principal par caniveau a grille de surface (pas de conduite enterree sur ce troncon).</t>
+          <t>Traverse pave-uni principal en conduite DN300.</t>
         </is>
       </c>
       <c r="AC11" s="7" t="n"/>
@@ -11586,7 +11678,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SWALE</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -11616,16 +11708,12 @@
         <f>IF(A12="","",IF(H12&lt;&gt;"",H12,IF(UPPER(TRIM(B12))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B12))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J12" s="7" t="inlineStr"/>
-      <c r="K12" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L12" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M12" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="J12" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr"/>
       <c r="N12" s="7" t="n">
         <v>0</v>
       </c>
@@ -11683,7 +11771,7 @@
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
-          <t>Ouest gazon aval - longueur solde sur chaine totale 23.58 m.</t>
+          <t>Ouest segment aval en conduite DN300 vers E04.</t>
         </is>
       </c>
       <c r="AC12" s="7" t="n"/>
@@ -12108,23 +12196,49 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>J-MECH-OUT</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="7">
+        <f>Inputs!$B$60</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
       <c r="I16" s="8">
         <f>IF(A16="","",IF(H16&lt;&gt;"",H16,IF(UPPER(TRIM(B16))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B16))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
+      <c r="J16" s="7">
+        <f>Inputs!$B$61</f>
+        <v/>
+      </c>
+      <c r="K16" s="7" t="inlineStr"/>
+      <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr"/>
+      <c r="N16" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="O16" s="8">
         <f>IF(A16="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A16))</f>
         <v/>
@@ -12177,7 +12291,11 @@
         <f>IF(A16="","",IF(OR(U16&gt;1,AND(X16&lt;&gt;"",X16&lt;Inputs!$B$16),AND(X16&lt;&gt;"",X16&gt;Inputs!$B$17),G16&lt;Inputs!$B$18,AH16="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB16" s="4" t="n"/>
+      <c r="AB16" s="4" t="inlineStr">
+        <is>
+          <t>Apport puisards zone grise est via reseau interne mecanique (traversant batiment) vers bassin sud.</t>
+        </is>
+      </c>
       <c r="AC16" s="7" t="n"/>
       <c r="AD16" s="8">
         <f>IF(A16="","",IF(AC16&lt;&gt;"",AC16,IF(E16="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E16,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B16))="SWALE",UPPER(TRIM(AI16))="PIPE"),AND(UPPER(TRIM(B16))="TRENCH",UPPER(TRIM(AI16))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -33881,22 +33999,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>J-MECH-OUT</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="8">
         <f>IF(OR(C18="",D18=""),"",MAX(0,C18-D18))</f>
         <v/>
       </c>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H18" s="7" t="inlineStr"/>
       <c r="I18" s="8">
         <f>IF(A18="","",IF(UPPER(TRIM(F18))="CIRC",PI()*(G18/2)^2*E18,IF(UPPER(TRIM(F18))="RECT",G18*H18*E18,"")))</f>
         <v/>
       </c>
-      <c r="J18" s="7" t="n"/>
+      <c r="J18" s="7">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
       <c r="K18" s="8">
         <f>IF(A18="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A18))</f>
         <v/>
@@ -39504,7 +39639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -39581,6 +39716,39 @@
       </c>
       <c r="B9" s="8">
         <f>IFERROR(INDEX(Noeuds_stockage!$I$4:$I$204,MATCH("BASIN_RET",Noeuds_stockage!$A$4:$A$204,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Impervious_area_total_m2 (ROOF+PAVAGE+TRESFOND)</t>
+        </is>
+      </c>
+      <c r="B10" s="4">
+        <f>SUMIFS(Zones_tributaires!$D$4:$D$204,Zones_tributaires!$C$4:$C$204,"ROOF")+SUMIFS(Zones_tributaires!$D$4:$D$204,Zones_tributaires!$C$4:$C$204,"PAVAGE")+SUMIFS(Zones_tributaires!$D$4:$D$204,Zones_tributaires!$C$4:$C$204,"TRESFOND")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Grass_area_total_m2</t>
+        </is>
+      </c>
+      <c r="B11" s="4">
+        <f>SUMIFS(Zones_tributaires!$D$4:$D$204,Zones_tributaires!$C$4:$C$204,"GRASS")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Impervious_fraction_of_(impervious+grass)</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>IF((B10+B11)=0,"",B10/(B10+B11))</f>
         <v/>
       </c>
     </row>
@@ -40279,22 +40447,22 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Ecoulement de surface peu profond</t>
+          <t>Conduite enterree peu profonde</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>E05A (SWALE)</t>
+          <t>E05A (PIPE)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>depth ~0.15-0.20 m</t>
+          <t>DN250, pente ~1.0%</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Eviter fouille profonde.</t>
+          <t>Strategie client: ouest privilegie en conduites.</t>
         </is>
       </c>
     </row>
@@ -40311,22 +40479,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Caniveau grille de surface</t>
+          <t>Conduite traversee pave-uni</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>E05B (CANIVEAU SURFACE)</t>
+          <t>E05B (PIPE)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>section ~0.25 x 0.08 m</t>
+          <t>DN250, pente ~1.0%</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Aucune remontee hydraulique requise; ecoulement de surface continu.</t>
+          <t>Raccord vers regard intermediaire.</t>
         </is>
       </c>
     </row>
@@ -40343,22 +40511,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Noue de surface</t>
+          <t>Conduite enterree</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>E05C (SWALE)</t>
+          <t>E05C (PIPE)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>depth ~0.15-0.20 m</t>
+          <t>DN300, pente ~0.9%</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Conduire vers traverse 2.</t>
+          <t>Segment principal vers aval.</t>
         </is>
       </c>
     </row>
@@ -40375,22 +40543,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Caniveau grille de surface</t>
+          <t>Conduite traversee pave-uni</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>E05D (CANIVEAU SURFACE)</t>
+          <t>E05D (PIPE)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>section ~0.30 x 0.10 m</t>
+          <t>DN300, pente ~0.9%</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Aucune conduite profonde de traversee sur ce troncon.</t>
+          <t>Traverse mineralisee en conduite.</t>
         </is>
       </c>
     </row>
@@ -40407,22 +40575,22 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Noue de surface</t>
+          <t>Conduite enterree</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>E05E (SWALE)</t>
+          <t>E05E (PIPE)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>vers J-OUEST-AVAL</t>
+          <t>DN300, pente ~0.8%</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Transition vers E06.</t>
+          <t>Vers E04 puis E08 et bassin.</t>
         </is>
       </c>
     </row>

</xml_diff>